<commit_message>
Lint and slight improvements
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\src\vivarium_gates_lsff_by_wealth_quintile\5000_analyze_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C0CDCC-1A52-4C62-9BB3-4C9059A32434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6F5217-5CA2-4BB3-8F76-2981076F8963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>Ethiopia -- Salt-- 100% NRV per average intake</t>
+  </si>
+  <si>
+    <t>*based on correlation between serum folate and hemoglobin</t>
   </si>
 </sst>
 </file>
@@ -154,7 +157,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%;\-0.0%;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,13 +182,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -197,10 +212,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -209,8 +225,12 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -513,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB45"/>
+  <dimension ref="A1:AB46"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.7265625" customWidth="1"/>
@@ -2310,11 +2330,11 @@
         <f>G32+G33+G34+G35+G36</f>
         <v>814.53034621778045</v>
       </c>
-      <c r="H30" s="3">
+      <c r="H30" s="6">
         <f>H32+H33+H34+H35+H36</f>
         <v>7.8485630910071178</v>
       </c>
-      <c r="I30" s="4">
+      <c r="I30" s="7">
         <f>IF(G30=0,0,H30/G30)</f>
         <v>9.6356914477789789E-3</v>
       </c>
@@ -2395,6 +2415,8 @@
       <c r="A31" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
@@ -2417,10 +2439,10 @@
       <c r="G32" s="3">
         <v>289.90090139463632</v>
       </c>
-      <c r="H32" s="3">
+      <c r="H32" s="6">
         <v>2.7005214785137208</v>
       </c>
-      <c r="I32" s="4">
+      <c r="I32" s="7">
         <f>IF(G32=0,0,H32/G32)</f>
         <v>9.3153262563939205E-3</v>
       </c>
@@ -2506,10 +2528,10 @@
       <c r="G33" s="3">
         <v>172.51020331953049</v>
       </c>
-      <c r="H33" s="3">
+      <c r="H33" s="6">
         <v>1.83290904215732</v>
       </c>
-      <c r="I33" s="4">
+      <c r="I33" s="7">
         <f>IF(G33=0,0,H33/G33)</f>
         <v>1.0624931203416012E-2</v>
       </c>
@@ -2595,10 +2617,10 @@
       <c r="G34" s="3">
         <v>135.45605543604131</v>
       </c>
-      <c r="H34" s="3">
+      <c r="H34" s="6">
         <v>1.933696004176745</v>
       </c>
-      <c r="I34" s="4">
+      <c r="I34" s="7">
         <f>IF(G34=0,0,H34/G34)</f>
         <v>1.4275448948753598E-2</v>
       </c>
@@ -2684,10 +2706,10 @@
       <c r="G35" s="3">
         <v>131.31388542968341</v>
       </c>
-      <c r="H35" s="3">
+      <c r="H35" s="6">
         <v>0.76651603757956766</v>
       </c>
-      <c r="I35" s="4">
+      <c r="I35" s="7">
         <f>IF(G35=0,0,H35/G35)</f>
         <v>5.8372809171808818E-3</v>
       </c>
@@ -2773,10 +2795,10 @@
       <c r="G36" s="3">
         <v>85.349300637888987</v>
       </c>
-      <c r="H36" s="3">
+      <c r="H36" s="6">
         <v>0.6149205285797652</v>
       </c>
-      <c r="I36" s="4">
+      <c r="I36" s="7">
         <f>IF(G36=0,0,H36/G36)</f>
         <v>7.2047518138278034E-3</v>
       </c>
@@ -2841,10 +2863,16 @@
         <v>0</v>
       </c>
     </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+    </row>
     <row r="38" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
     </row>
     <row r="39" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
@@ -2870,11 +2898,11 @@
         <f>G41+G42+G43+G44+G45</f>
         <v>814.53034621778045</v>
       </c>
-      <c r="H39" s="3">
+      <c r="H39" s="6">
         <f>H41+H42+H43+H44+H45</f>
         <v>29.040910758803861</v>
       </c>
-      <c r="I39" s="4">
+      <c r="I39" s="7">
         <f>IF(G39=0,0,H39/G39)</f>
         <v>3.5653565141745142E-2</v>
       </c>
@@ -2955,6 +2983,8 @@
       <c r="A40" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
     </row>
     <row r="41" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
@@ -2977,10 +3007,10 @@
       <c r="G41" s="3">
         <v>289.90090139463632</v>
       </c>
-      <c r="H41" s="3">
+      <c r="H41" s="6">
         <v>10.024387991053461</v>
       </c>
-      <c r="I41" s="4">
+      <c r="I41" s="7">
         <f>IF(G41=0,0,H41/G41)</f>
         <v>3.4578671341926812E-2</v>
       </c>
@@ -3066,10 +3096,10 @@
       <c r="G42" s="3">
         <v>172.51020331953049</v>
       </c>
-      <c r="H42" s="3">
+      <c r="H42" s="6">
         <v>6.7234499855660248</v>
       </c>
-      <c r="I42" s="4">
+      <c r="I42" s="7">
         <f>IF(G42=0,0,H42/G42)</f>
         <v>3.8974216343091166E-2</v>
       </c>
@@ -3155,10 +3185,10 @@
       <c r="G43" s="3">
         <v>135.45605543604131</v>
       </c>
-      <c r="H43" s="3">
+      <c r="H43" s="6">
         <v>6.9944547501377379</v>
       </c>
-      <c r="I43" s="4">
+      <c r="I43" s="7">
         <f>IF(G43=0,0,H43/G43)</f>
         <v>5.1636338645933262E-2</v>
       </c>
@@ -3244,10 +3274,10 @@
       <c r="G44" s="3">
         <v>131.31388542968341</v>
       </c>
-      <c r="H44" s="3">
+      <c r="H44" s="6">
         <v>2.9323600028994838</v>
       </c>
-      <c r="I44" s="4">
+      <c r="I44" s="7">
         <f>IF(G44=0,0,H44/G44)</f>
         <v>2.2330921008880802E-2</v>
       </c>
@@ -3333,10 +3363,10 @@
       <c r="G45" s="3">
         <v>85.349300637888987</v>
       </c>
-      <c r="H45" s="3">
+      <c r="H45" s="6">
         <v>2.3662580291471529</v>
       </c>
-      <c r="I45" s="4">
+      <c r="I45" s="7">
         <f>IF(G45=0,0,H45/G45)</f>
         <v>2.7724398576931087E-2</v>
       </c>
@@ -3399,6 +3429,11 @@
       <c r="AB45" s="4">
         <f>IF(Z45=0,0,AA45/Z45)</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="H46" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add rice in Nigeria, fix some bugs around vehicle consumption
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
@@ -1,44 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\src\vivarium_gates_lsff_by_wealth_quintile\5000_analyze_results\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7FDA3F-F4FB-47EA-AF6D-CA9FA4EA1BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Model Results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="J30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="J39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -51,7 +32,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="K39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -64,7 +45,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="W39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -77,7 +58,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="X39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -90,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="J48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -103,7 +84,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="K48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -116,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="W48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -129,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="X48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -147,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="40">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -260,6 +241,9 @@
     <t>Nigeria -- Bouillon</t>
   </si>
   <si>
+    <t>Nigeria -- Rice</t>
+  </si>
+  <si>
     <t>Ethiopia -- Salt-- 25% NRV per average intake</t>
   </si>
   <si>
@@ -269,12 +253,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0%;\-0.0%;&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0%;-0.0%;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,21 +340,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -408,7 +384,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -442,7 +418,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -477,10 +452,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -653,9 +627,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AD54"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
@@ -664,7 +638,7 @@
     <col min="19" max="30" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30">
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
@@ -748,1846 +722,1846 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30">
       <c r="B3" t="s">
         <v>28</v>
       </c>
       <c r="C3" s="3">
         <f>C5+C6+C7+C8+C9</f>
-        <v>1555.2611894681488</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3">
         <f>D5+D6+D7+D8+D9</f>
-        <v>83.943882240574695</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3">
         <f>E5+E6+E7+E8+E9</f>
-        <v>1471.3173072275742</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3">
         <f>F5+F6+F7+F8+F9</f>
-        <v>1581.6305477704739</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3">
         <f>G5+G6+G7+G8+G9</f>
-        <v>83.943882240574695</v>
+        <v>0</v>
       </c>
       <c r="H3" s="4">
         <f>IF(F3=0,0,G3/F3)</f>
-        <v>5.3074267159865594E-2</v>
+        <v>0</v>
       </c>
       <c r="I3" s="3">
         <f>I5+I6+I7+I8+I9</f>
-        <v>19429.786784833006</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3">
         <f>J5+J6+J7+J8+J9</f>
-        <v>1299.0325522563842</v>
+        <v>0</v>
       </c>
       <c r="K3" s="4">
         <f>IF(I3=0,0,J3/I3)</f>
-        <v>6.6857787305747263E-2</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>L5+L6+L7+L8+L9</f>
-        <v>73088.837013306678</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>M5+M6+M7+M8+M9</f>
-        <v>151.25588574661126</v>
+        <v>0</v>
       </c>
       <c r="N3" s="4">
         <f>IF(L3=0,0,M3/L3)</f>
-        <v>2.069479990755269E-3</v>
+        <v>0</v>
       </c>
       <c r="O3" s="3">
         <f>O5+O6+O7+O8+O9</f>
-        <v>2218.4421230582016</v>
+        <v>0</v>
       </c>
       <c r="P3" s="3">
         <f>P5+P6+P7+P8+P9</f>
-        <v>21.02886922457855</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="4">
         <f>IF(O3=0,0,P3/O3)</f>
-        <v>9.4791155496044693E-3</v>
+        <v>0</v>
       </c>
       <c r="S3" s="3">
         <f>S5+S6+S7+S8+S9</f>
-        <v>17581.869861191975</v>
+        <v>0</v>
       </c>
       <c r="T3" s="3">
         <f>T5+T6+T7+T8+T9</f>
-        <v>933.14485818289268</v>
+        <v>0</v>
       </c>
       <c r="U3" s="4">
         <f>IF(S3=0,0,T3/S3)</f>
-        <v>5.3074267159865636E-2</v>
+        <v>0</v>
       </c>
       <c r="V3" s="3">
         <f>V5+V6+V7+V8+V9</f>
-        <v>619844465.28808701</v>
+        <v>0</v>
       </c>
       <c r="W3" s="3">
         <f>W5+W6+W7+W8+W9</f>
-        <v>32672650.79602851</v>
+        <v>0</v>
       </c>
       <c r="X3" s="4">
         <f>IF(V3=0,0,W3/V3)</f>
-        <v>5.2711047086373745E-2</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="3">
         <f>Y5+Y6+Y7+Y8+Y9</f>
-        <v>23865851.045409296</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="3">
         <f>Z5+Z6+Z7+Z8+Z9</f>
-        <v>182259.01024660328</v>
+        <v>0</v>
       </c>
       <c r="AA3" s="4">
         <f>IF(Y3=0,0,Z3/Y3)</f>
-        <v>7.6368116896322301E-3</v>
+        <v>0</v>
       </c>
       <c r="AB3" s="3">
         <f>AB5+AB6+AB7+AB8+AB9</f>
-        <v>815643.03969645989</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="3">
         <f>AC5+AC6+AC7+AC8+AC9</f>
-        <v>1680.7280119055067</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="4">
         <f>IF(AB3=0,0,AC3/AB3)</f>
-        <v>2.0606171206107352E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30">
       <c r="A4" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30">
       <c r="B5" t="s">
         <v>30</v>
       </c>
       <c r="C5" s="3">
         <f>J5+M5+G5+P5</f>
-        <v>449.9915054404222</v>
+        <v>0</v>
       </c>
       <c r="D5" s="3">
         <f>G5</f>
-        <v>28.563180317425989</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3">
         <f>J5+M5+P5</f>
-        <v>421.42832512299623</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3">
-        <v>397.34111205252179</v>
+        <v>397.0902965307904</v>
       </c>
       <c r="G5" s="3">
-        <v>28.563180317425989</v>
+        <v>28.31236479569459</v>
       </c>
       <c r="H5" s="4">
         <f>IF(F5=0,0,G5/F5)</f>
-        <v>7.1885791454800216E-2</v>
+        <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>4596.9756107760377</v>
+        <v>4589.340725230151</v>
       </c>
       <c r="J5" s="3">
-        <v>361.18659869736899</v>
+        <v>353.7198939848701</v>
       </c>
       <c r="K5" s="4">
         <f>IF(I5=0,0,J5/I5)</f>
-        <v>7.8570484004894539E-2</v>
+        <v>0</v>
       </c>
       <c r="L5" s="3">
-        <v>18641.712679665659</v>
+        <v>18640.87579554441</v>
       </c>
       <c r="M5" s="3">
-        <v>53.864307028021663</v>
+        <v>53.02742290676385</v>
       </c>
       <c r="N5" s="4">
         <f>IF(L5=0,0,M5/L5)</f>
-        <v>2.8894505539062802E-3</v>
+        <v>0</v>
       </c>
       <c r="O5" s="3">
-        <v>597.84933727803173</v>
+        <v>597.8493190972089</v>
       </c>
       <c r="P5" s="3">
-        <v>6.3774193976055829</v>
+        <v>6.377401216782746</v>
       </c>
       <c r="Q5" s="4">
         <f>IF(O5=0,0,P5/O5)</f>
-        <v>1.0667268490488839E-2</v>
+        <v>0</v>
       </c>
       <c r="S5" s="3">
-        <v>4416.960542685817</v>
+        <v>4414.172403655204</v>
       </c>
       <c r="T5" s="3">
-        <v>317.51670443559402</v>
+        <v>314.7285654049811</v>
       </c>
       <c r="U5" s="4">
         <f>IF(S5=0,0,T5/S5)</f>
-        <v>7.1885791454800257E-2</v>
+        <v>0</v>
       </c>
       <c r="V5" s="3">
-        <v>139164134.1773752</v>
+        <v>139014089.4100596</v>
       </c>
       <c r="W5" s="3">
-        <v>8505845.6689952314</v>
+        <v>8355155.591834024</v>
       </c>
       <c r="X5" s="4">
         <f>IF(V5=0,0,W5/V5)</f>
-        <v>6.1120961368924906E-2</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="3">
-        <v>6122536.7016462469</v>
+        <v>6121894.332663051</v>
       </c>
       <c r="Z5" s="3">
-        <v>65974.70812917687</v>
+        <v>65332.33914598078</v>
       </c>
       <c r="AA5" s="4">
         <f>IF(Y5=0,0,Z5/Y5)</f>
-        <v>1.0775714600687878E-2</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="3">
-        <v>208025.75267651089</v>
+        <v>208016.4497539358</v>
       </c>
       <c r="AC5" s="3">
-        <v>598.48801899957471</v>
+        <v>589.1850964244513</v>
       </c>
       <c r="AD5" s="4">
         <f>IF(AB5=0,0,AC5/AB5)</f>
-        <v>2.876990042335045E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30">
       <c r="B6" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="3">
         <f>J6+M6+G6+P6</f>
-        <v>385.38777066778857</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3">
         <f>G6</f>
-        <v>21.234273115711929</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3">
         <f>J6+M6+P6</f>
-        <v>364.15349755207666</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3">
-        <v>347.01108902834721</v>
+        <v>346.9213241359736</v>
       </c>
       <c r="G6" s="3">
-        <v>21.234273115711929</v>
+        <v>21.14450822333828</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
-        <v>6.1191915149366623E-2</v>
+        <v>0</v>
       </c>
       <c r="I6" s="3">
-        <v>4120.9915624965133</v>
+        <v>4107.767741737073</v>
       </c>
       <c r="J6" s="3">
-        <v>324.67693416423162</v>
+        <v>311.7710410246919</v>
       </c>
       <c r="K6" s="4">
         <f>IF(I6=0,0,J6/I6)</f>
-        <v>7.8786119612324818E-2</v>
+        <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>15401.721838607329</v>
+        <v>15402.27975372651</v>
       </c>
       <c r="M6" s="3">
-        <v>34.045783631026737</v>
+        <v>34.60369875020162</v>
       </c>
       <c r="N6" s="4">
         <f>IF(L6=0,0,M6/L6)</f>
-        <v>2.2105180179065784E-3</v>
+        <v>0</v>
       </c>
       <c r="O6" s="3">
-        <v>474.66517473403837</v>
+        <v>474.6651801296223</v>
       </c>
       <c r="P6" s="3">
-        <v>5.4307797568183158</v>
+        <v>5.430785152402183</v>
       </c>
       <c r="Q6" s="4">
         <f>IF(O6=0,0,P6/O6)</f>
-        <v>1.1441285448972023E-2</v>
+        <v>0</v>
       </c>
       <c r="S6" s="3">
-        <v>3857.4772194981001</v>
+        <v>3856.479366581032</v>
       </c>
       <c r="T6" s="3">
-        <v>236.0464187061425</v>
+        <v>235.0485657890745</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
-        <v>6.1191915149366644E-2</v>
+        <v>0</v>
       </c>
       <c r="V6" s="3">
-        <v>129179305.0153213</v>
+        <v>128879655.4497555</v>
       </c>
       <c r="W6" s="3">
-        <v>8078008.1331280172</v>
+        <v>7779522.534546092</v>
       </c>
       <c r="X6" s="4">
         <f>IF(V6=0,0,W6/V6)</f>
-        <v>6.2533299216696717E-2</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="3">
-        <v>5177909.8376185223</v>
+        <v>5178418.767634194</v>
       </c>
       <c r="Z6" s="3">
-        <v>45114.783950233832</v>
+        <v>45623.71396590583</v>
       </c>
       <c r="AA6" s="4">
         <f>IF(Y6=0,0,Z6/Y6)</f>
-        <v>8.7129334741339343E-3</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="3">
-        <v>171862.19165281719</v>
+        <v>171868.3936012006</v>
       </c>
       <c r="AC6" s="3">
-        <v>378.31885138832149</v>
+        <v>384.5207997717371</v>
       </c>
       <c r="AD6" s="4">
         <f>IF(AB6=0,0,AC6/AB6)</f>
-        <v>2.2012919057413875E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30">
       <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="3">
         <f>J7+M7+G7+P7</f>
-        <v>328.27398788318089</v>
+        <v>0</v>
       </c>
       <c r="D7" s="3">
         <f>G7</f>
-        <v>16.09202406254137</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3">
         <f>J7+M7+P7</f>
-        <v>312.18196382063951</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3">
-        <v>308.5630389483282</v>
+        <v>308.4024677522138</v>
       </c>
       <c r="G7" s="3">
-        <v>16.09202406254137</v>
+        <v>15.93145286642702</v>
       </c>
       <c r="H7" s="4">
         <f>IF(F7=0,0,G7/F7)</f>
-        <v>5.2151495906274541E-2</v>
+        <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>3985.2760327157789</v>
+        <v>3973.118437255514</v>
       </c>
       <c r="J7" s="3">
-        <v>280.13566344122307</v>
+        <v>268.34160623975</v>
       </c>
       <c r="K7" s="4">
         <f>IF(I7=0,0,J7/I7)</f>
-        <v>7.0292662576329434E-2</v>
+        <v>0</v>
       </c>
       <c r="L7" s="3">
-        <v>13777.25618273796</v>
+        <v>13777.53512556912</v>
       </c>
       <c r="M7" s="3">
-        <v>27.90923734307103</v>
+        <v>28.18818017423339</v>
       </c>
       <c r="N7" s="4">
         <f>IF(L7=0,0,M7/L7)</f>
-        <v>2.0257471424563883E-3</v>
+        <v>0</v>
       </c>
       <c r="O7" s="3">
-        <v>416.35114676752949</v>
+        <v>416.3511559351928</v>
       </c>
       <c r="P7" s="3">
-        <v>4.1370630363454124</v>
+        <v>4.137072204008699</v>
       </c>
       <c r="Q7" s="4">
         <f>IF(O7=0,0,P7/O7)</f>
-        <v>9.936475661145111E-3</v>
+        <v>0</v>
       </c>
       <c r="S7" s="3">
-        <v>3430.077398549784</v>
+        <v>3428.292441957034</v>
       </c>
       <c r="T7" s="3">
-        <v>178.8836674086738</v>
+        <v>177.0987108159238</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
-        <v>5.2151495906274513E-2</v>
+        <v>0</v>
       </c>
       <c r="V7" s="3">
-        <v>125490666.0533599</v>
+        <v>125210935.1791828</v>
       </c>
       <c r="W7" s="3">
-        <v>7026848.5332566202</v>
+        <v>6749260.368166924</v>
       </c>
       <c r="X7" s="4">
         <f>IF(V7=0,0,W7/V7)</f>
-        <v>5.5994989541841567E-2</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="3">
-        <v>4635731.7964105764</v>
+        <v>4636445.539725238</v>
       </c>
       <c r="Z7" s="3">
-        <v>32670.824420694262</v>
+        <v>33384.56773535628</v>
       </c>
       <c r="AA7" s="4">
         <f>IF(Y7=0,0,Z7/Y7)</f>
-        <v>7.0476088469982488E-3</v>
+        <v>0</v>
       </c>
       <c r="AB7" s="3">
-        <v>153752.5023732449</v>
+        <v>153755.6033474366</v>
       </c>
       <c r="AC7" s="3">
-        <v>310.09741917075007</v>
+        <v>313.1983933624579</v>
       </c>
       <c r="AD7" s="4">
         <f>IF(AB7=0,0,AC7/AB7)</f>
-        <v>2.0168609576055353E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30">
       <c r="B8" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="3">
         <f>J8+M8+G8+P8</f>
-        <v>262.7394792518345</v>
+        <v>0</v>
       </c>
       <c r="D8" s="3">
         <f>G8</f>
-        <v>13.081033856759079</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3">
         <f>J8+M8+P8</f>
-        <v>249.6584453950754</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>288.86678736531792</v>
+        <v>288.7894998187962</v>
       </c>
       <c r="G8" s="3">
-        <v>13.081033856759079</v>
+        <v>13.00374631023745</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
-        <v>4.528396627410141E-2</v>
+        <v>0</v>
       </c>
       <c r="I8" s="3">
-        <v>3614.3317239066419</v>
+        <v>3607.833411572376</v>
       </c>
       <c r="J8" s="3">
-        <v>223.0981557032205</v>
+        <v>216.8494586088709</v>
       </c>
       <c r="K8" s="4">
         <f>IF(I8=0,0,J8/I8)</f>
-        <v>6.1725976679882395E-2</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3">
-        <v>12916.932829144929</v>
+        <v>12917.49073548635</v>
       </c>
       <c r="M8" s="3">
-        <v>22.595390879644079</v>
+        <v>23.15329722107202</v>
       </c>
       <c r="N8" s="4">
         <f>IF(L8=0,0,M8/L8)</f>
-        <v>1.7492845382505438E-3</v>
+        <v>0</v>
       </c>
       <c r="O8" s="3">
-        <v>380.99541784497882</v>
+        <v>380.9954098585719</v>
       </c>
       <c r="P8" s="3">
-        <v>3.9648988122108282</v>
+        <v>3.964890825803974</v>
       </c>
       <c r="Q8" s="4">
         <f>IF(O8=0,0,P8/O8)</f>
-        <v>1.0406683719813356E-2</v>
+        <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3211.1280790807491</v>
+        <v>3210.268928006087</v>
       </c>
       <c r="T8" s="3">
-        <v>145.41261563491341</v>
+        <v>144.553464560252</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
-        <v>4.5283966274101632E-2</v>
+        <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>117876445.53719731</v>
+        <v>117724986.5060492</v>
       </c>
       <c r="W8" s="3">
-        <v>5909428.3290538341</v>
+        <v>5759705.398426414</v>
       </c>
       <c r="X8" s="4">
         <f>IF(V8=0,0,W8/V8)</f>
-        <v>5.0132393304895204E-2</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="3">
-        <v>4171603.1382768038</v>
+        <v>4171333.157109953</v>
       </c>
       <c r="Z8" s="3">
-        <v>27643.588900032919</v>
+        <v>27373.60773318261</v>
       </c>
       <c r="AA8" s="4">
         <f>IF(Y8=0,0,Z8/Y8)</f>
-        <v>6.6266104381760222E-3</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="3">
-        <v>144164.29017248511</v>
+        <v>144170.4921208685</v>
       </c>
       <c r="AC8" s="3">
-        <v>251.178909528302</v>
+        <v>257.3808579117176</v>
       </c>
       <c r="AD8" s="4">
         <f>IF(AB8=0,0,AC8/AB8)</f>
-        <v>1.7423101742309378E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30">
       <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="3">
         <f>J9+M9+G9+P9</f>
-        <v>128.86844622492271</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3">
         <f>G9</f>
-        <v>4.9733708881363272</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3">
         <f>J9+M9+P9</f>
-        <v>123.89507533678638</v>
+        <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>239.84852037595849</v>
+        <v>239.8280399304447</v>
       </c>
       <c r="G9" s="3">
-        <v>4.9733708881363272</v>
+        <v>4.952890442622476</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
-        <v>2.0735466203171286E-2</v>
+        <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>3112.2118549380339</v>
+        <v>3109.42846045582</v>
       </c>
       <c r="J9" s="3">
-        <v>109.9352002503402</v>
+        <v>107.3276773510338</v>
       </c>
       <c r="K9" s="4">
         <f>IF(I9=0,0,J9/I9)</f>
-        <v>3.5323816428470316E-2</v>
+        <v>0</v>
       </c>
       <c r="L9" s="3">
-        <v>12351.213483150799</v>
+        <v>12350.65552086042</v>
       </c>
       <c r="M9" s="3">
-        <v>12.841166864847761</v>
+        <v>12.28320457446016</v>
       </c>
       <c r="N9" s="4">
         <f>IF(L9=0,0,M9/L9)</f>
-        <v>1.0396684408673967E-3</v>
+        <v>0</v>
       </c>
       <c r="O9" s="3">
-        <v>348.58104643362333</v>
+        <v>348.5810412050197</v>
       </c>
       <c r="P9" s="3">
-        <v>1.1187082215984121</v>
+        <v>1.118702992994746</v>
       </c>
       <c r="Q9" s="4">
         <f>IF(O9=0,0,P9/O9)</f>
-        <v>3.209320280158824E-3</v>
+        <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>2666.226621377526</v>
+        <v>2665.998954727921</v>
       </c>
       <c r="T9" s="3">
-        <v>55.285451997568998</v>
+        <v>55.057785347964</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
-        <v>2.0735466203171189E-2</v>
+        <v>0</v>
       </c>
       <c r="V9" s="3">
-        <v>108133914.5048333</v>
+        <v>108065359.9260122</v>
       </c>
       <c r="W9" s="3">
-        <v>3152520.1315948069</v>
+        <v>3085710.668220431</v>
       </c>
       <c r="X9" s="4">
         <f>IF(V9=0,0,W9/V9)</f>
-        <v>2.9153851925465046E-2</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="3">
-        <v>3758069.5714571462</v>
+        <v>3757886.480780777</v>
       </c>
       <c r="Z9" s="3">
-        <v>10855.1048464654</v>
+        <v>10672.01417009579</v>
       </c>
       <c r="AA9" s="4">
         <f>IF(Y9=0,0,Z9/Y9)</f>
-        <v>2.8884789491154801E-3</v>
+        <v>0</v>
       </c>
       <c r="AB9" s="3">
-        <v>137838.30282140171</v>
+        <v>137832.1008730183</v>
       </c>
       <c r="AC9" s="3">
-        <v>142.64481281855839</v>
+        <v>136.4428644351428</v>
       </c>
       <c r="AD9" s="4">
         <f>IF(AB9=0,0,AC9/AB9)</f>
-        <v>1.034870641169926E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30">
       <c r="B12" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="3">
         <f>C14+C15+C16+C17+C18</f>
-        <v>2069.0313075611234</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3">
         <f>D14+D15+D16+D17+D18</f>
-        <v>597.71400033354905</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3">
         <f>E14+E15+E16+E17+E18</f>
-        <v>1471.3173072275742</v>
+        <v>0</v>
       </c>
       <c r="F12" s="3">
         <f>F14+F15+F16+F17+F18</f>
-        <v>1581.6305477704739</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3">
         <f>G14+G15+G16+G17+G18</f>
-        <v>597.71400033354905</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4">
         <f>IF(F12=0,0,G12/F12)</f>
-        <v>0.37791000001619168</v>
+        <v>0</v>
       </c>
       <c r="I12" s="3">
         <f>I14+I15+I16+I17+I18</f>
-        <v>19429.786784833006</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3">
         <f>J14+J15+J16+J17+J18</f>
-        <v>1299.0325522563842</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
         <f>IF(I12=0,0,J12/I12)</f>
-        <v>6.6857787305747263E-2</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3">
         <f>L14+L15+L16+L17+L18</f>
-        <v>73088.837013306678</v>
+        <v>0</v>
       </c>
       <c r="M12" s="3">
         <f>M14+M15+M16+M17+M18</f>
-        <v>151.25588574661126</v>
+        <v>0</v>
       </c>
       <c r="N12" s="4">
         <f>IF(L12=0,0,M12/L12)</f>
-        <v>2.069479990755269E-3</v>
+        <v>0</v>
       </c>
       <c r="O12" s="3">
         <f>O14+O15+O16+O17+O18</f>
-        <v>2218.4421230582016</v>
+        <v>0</v>
       </c>
       <c r="P12" s="3">
         <f>P14+P15+P16+P17+P18</f>
-        <v>21.02886922457855</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="4">
         <f>IF(O12=0,0,P12/O12)</f>
-        <v>9.4791155496044693E-3</v>
+        <v>0</v>
       </c>
       <c r="S12" s="3">
         <f>S14+S15+S16+S17+S18</f>
-        <v>17581.869861191975</v>
+        <v>0</v>
       </c>
       <c r="T12" s="3">
         <f>T14+T15+T16+T17+T18</f>
-        <v>6644.3644395277415</v>
+        <v>0</v>
       </c>
       <c r="U12" s="4">
         <f>IF(S12=0,0,T12/S12)</f>
-        <v>0.37791000001619179</v>
+        <v>0</v>
       </c>
       <c r="V12" s="3">
         <f>V14+V15+V16+V17+V18</f>
-        <v>619844465.28808701</v>
+        <v>0</v>
       </c>
       <c r="W12" s="3">
         <f>W14+W15+W16+W17+W18</f>
-        <v>32672650.79602851</v>
+        <v>0</v>
       </c>
       <c r="X12" s="4">
         <f>IF(V12=0,0,W12/V12)</f>
-        <v>5.2711047086373745E-2</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="3">
         <f>Y14+Y15+Y16+Y17+Y18</f>
-        <v>23865851.045409296</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="3">
         <f>Z14+Z15+Z16+Z17+Z18</f>
-        <v>182259.01024660328</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="4">
         <f>IF(Y12=0,0,Z12/Y12)</f>
-        <v>7.6368116896322301E-3</v>
+        <v>0</v>
       </c>
       <c r="AB12" s="3">
         <f>AB14+AB15+AB16+AB17+AB18</f>
-        <v>815643.03969645989</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="3">
         <f>AC14+AC15+AC16+AC17+AC18</f>
-        <v>1680.7280119055067</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="4">
         <f>IF(AB12=0,0,AC12/AB12)</f>
-        <v>2.0606171206107352E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30">
       <c r="A13" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30">
       <c r="B14" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="3">
         <f>J14+M14+G14+P14</f>
-        <v>610.22389456206611</v>
+        <v>0</v>
       </c>
       <c r="D14" s="3">
         <f>G14</f>
-        <v>188.79556943906991</v>
+        <v>0</v>
       </c>
       <c r="E14" s="3">
         <f>J14+M14+P14</f>
-        <v>421.42832512299623</v>
+        <v>0</v>
       </c>
       <c r="F14" s="3">
-        <v>397.34111205252179</v>
+        <v>397.0902965307904</v>
       </c>
       <c r="G14" s="3">
-        <v>188.79556943906991</v>
+        <v>187.694679977468</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
-        <v>0.4751473323860691</v>
+        <v>0</v>
       </c>
       <c r="I14" s="3">
-        <v>4596.9756107760377</v>
+        <v>4589.340725230151</v>
       </c>
       <c r="J14" s="3">
-        <v>361.18659869736899</v>
+        <v>353.7198939848701</v>
       </c>
       <c r="K14" s="4">
         <f>IF(I14=0,0,J14/I14)</f>
-        <v>7.8570484004894539E-2</v>
+        <v>0</v>
       </c>
       <c r="L14" s="3">
-        <v>18641.712679665659</v>
+        <v>18640.87579554441</v>
       </c>
       <c r="M14" s="3">
-        <v>53.864307028021663</v>
+        <v>53.02742290676385</v>
       </c>
       <c r="N14" s="4">
         <f>IF(L14=0,0,M14/L14)</f>
-        <v>2.8894505539062802E-3</v>
+        <v>0</v>
       </c>
       <c r="O14" s="3">
-        <v>597.84933727803173</v>
+        <v>597.8493190972089</v>
       </c>
       <c r="P14" s="3">
-        <v>6.3774193976055829</v>
+        <v>6.377401216782746</v>
       </c>
       <c r="Q14" s="4">
         <f>IF(O14=0,0,P14/O14)</f>
-        <v>1.0667268490488839E-2</v>
+        <v>0</v>
       </c>
       <c r="S14" s="3">
-        <v>4416.960542685817</v>
+        <v>4414.172403655204</v>
       </c>
       <c r="T14" s="3">
-        <v>2098.7070191116909</v>
+        <v>2086.469208408852</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
-        <v>0.47514733238606927</v>
+        <v>0</v>
       </c>
       <c r="V14" s="3">
-        <v>139164134.1773752</v>
+        <v>139014089.4100596</v>
       </c>
       <c r="W14" s="3">
-        <v>8505845.6689952314</v>
+        <v>8355155.591834024</v>
       </c>
       <c r="X14" s="4">
         <f>IF(V14=0,0,W14/V14)</f>
-        <v>6.1120961368924906E-2</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="3">
-        <v>6122536.7016462469</v>
+        <v>6121894.332663051</v>
       </c>
       <c r="Z14" s="3">
-        <v>65974.70812917687</v>
+        <v>65332.33914598078</v>
       </c>
       <c r="AA14" s="4">
         <f>IF(Y14=0,0,Z14/Y14)</f>
-        <v>1.0775714600687878E-2</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="3">
-        <v>208025.75267651089</v>
+        <v>208016.4497539358</v>
       </c>
       <c r="AC14" s="3">
-        <v>598.48801899957471</v>
+        <v>589.1850964244513</v>
       </c>
       <c r="AD14" s="4">
         <f>IF(AB14=0,0,AC14/AB14)</f>
-        <v>2.876990042335045E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30">
       <c r="B15" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="3">
         <f>J15+M15+G15+P15</f>
-        <v>512.46692346363602</v>
+        <v>0</v>
       </c>
       <c r="D15" s="3">
         <f>G15</f>
-        <v>148.31342591155939</v>
+        <v>0</v>
       </c>
       <c r="E15" s="3">
         <f>J15+M15+P15</f>
-        <v>364.15349755207666</v>
+        <v>0</v>
       </c>
       <c r="F15" s="3">
-        <v>347.01108902834721</v>
+        <v>346.9213241359736</v>
       </c>
       <c r="G15" s="3">
-        <v>148.31342591155939</v>
+        <v>147.8750540550408</v>
       </c>
       <c r="H15" s="4">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.42740255456056542</v>
+        <v>0</v>
       </c>
       <c r="I15" s="3">
-        <v>4120.9915624965133</v>
+        <v>4107.767741737073</v>
       </c>
       <c r="J15" s="3">
-        <v>324.67693416423162</v>
+        <v>311.7710410246919</v>
       </c>
       <c r="K15" s="4">
         <f>IF(I15=0,0,J15/I15)</f>
-        <v>7.8786119612324818E-2</v>
+        <v>0</v>
       </c>
       <c r="L15" s="3">
-        <v>15401.721838607329</v>
+        <v>15402.27975372651</v>
       </c>
       <c r="M15" s="3">
-        <v>34.045783631026737</v>
+        <v>34.60369875020162</v>
       </c>
       <c r="N15" s="4">
         <f>IF(L15=0,0,M15/L15)</f>
-        <v>2.2105180179065784E-3</v>
+        <v>0</v>
       </c>
       <c r="O15" s="3">
-        <v>474.66517473403837</v>
+        <v>474.6651801296223</v>
       </c>
       <c r="P15" s="3">
-        <v>5.4307797568183158</v>
+        <v>5.430785152402183</v>
       </c>
       <c r="Q15" s="4">
         <f>IF(O15=0,0,P15/O15)</f>
-        <v>1.1441285448972023E-2</v>
+        <v>0</v>
       </c>
       <c r="S15" s="3">
-        <v>3857.4772194981001</v>
+        <v>3856.479366581032</v>
       </c>
       <c r="T15" s="3">
-        <v>1648.695617772675</v>
+        <v>1643.822547419435</v>
       </c>
       <c r="U15" s="4">
         <f>IF(S15=0,0,T15/S15)</f>
-        <v>0.42740255456056542</v>
+        <v>0</v>
       </c>
       <c r="V15" s="3">
-        <v>129179305.0153213</v>
+        <v>128879655.4497555</v>
       </c>
       <c r="W15" s="3">
-        <v>8078008.1331280172</v>
+        <v>7779522.534546092</v>
       </c>
       <c r="X15" s="4">
         <f>IF(V15=0,0,W15/V15)</f>
-        <v>6.2533299216696717E-2</v>
+        <v>0</v>
       </c>
       <c r="Y15" s="3">
-        <v>5177909.8376185223</v>
+        <v>5178418.767634194</v>
       </c>
       <c r="Z15" s="3">
-        <v>45114.783950233832</v>
+        <v>45623.71396590583</v>
       </c>
       <c r="AA15" s="4">
         <f>IF(Y15=0,0,Z15/Y15)</f>
-        <v>8.7129334741339343E-3</v>
+        <v>0</v>
       </c>
       <c r="AB15" s="3">
-        <v>171862.19165281719</v>
+        <v>171868.3936012006</v>
       </c>
       <c r="AC15" s="3">
-        <v>378.31885138832149</v>
+        <v>384.5207997717371</v>
       </c>
       <c r="AD15" s="4">
         <f>IF(AB15=0,0,AC15/AB15)</f>
-        <v>2.2012919057413875E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30">
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="3">
         <f>J16+M16+G16+P16</f>
-        <v>430.1225656507022</v>
+        <v>0</v>
       </c>
       <c r="D16" s="3">
         <f>G16</f>
-        <v>117.9406018300627</v>
+        <v>0</v>
       </c>
       <c r="E16" s="3">
         <f>J16+M16+P16</f>
-        <v>312.18196382063951</v>
+        <v>0</v>
       </c>
       <c r="F16" s="3">
-        <v>308.5630389483282</v>
+        <v>308.4024677522138</v>
       </c>
       <c r="G16" s="3">
-        <v>117.9406018300627</v>
+        <v>117.0752777047284</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
-        <v>0.38222530550657746</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3">
-        <v>3985.2760327157789</v>
+        <v>3973.118437255514</v>
       </c>
       <c r="J16" s="3">
-        <v>280.13566344122307</v>
+        <v>268.34160623975</v>
       </c>
       <c r="K16" s="4">
         <f>IF(I16=0,0,J16/I16)</f>
-        <v>7.0292662576329434E-2</v>
+        <v>0</v>
       </c>
       <c r="L16" s="3">
-        <v>13777.25618273796</v>
+        <v>13777.53512556912</v>
       </c>
       <c r="M16" s="3">
-        <v>27.90923734307103</v>
+        <v>28.18818017423339</v>
       </c>
       <c r="N16" s="4">
         <f>IF(L16=0,0,M16/L16)</f>
-        <v>2.0257471424563883E-3</v>
+        <v>0</v>
       </c>
       <c r="O16" s="3">
-        <v>416.35114676752949</v>
+        <v>416.3511559351928</v>
       </c>
       <c r="P16" s="3">
-        <v>4.1370630363454124</v>
+        <v>4.137072204008699</v>
       </c>
       <c r="Q16" s="4">
         <f>IF(O16=0,0,P16/O16)</f>
-        <v>9.936475661145111E-3</v>
+        <v>0</v>
       </c>
       <c r="S16" s="3">
-        <v>3430.077398549784</v>
+        <v>3428.292441957034</v>
       </c>
       <c r="T16" s="3">
-        <v>1311.062381571898</v>
+        <v>1301.443184357464</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
-        <v>0.38222530550657757</v>
+        <v>0</v>
       </c>
       <c r="V16" s="3">
-        <v>125490666.0533599</v>
+        <v>125210935.1791828</v>
       </c>
       <c r="W16" s="3">
-        <v>7026848.5332566202</v>
+        <v>6749260.368166924</v>
       </c>
       <c r="X16" s="4">
         <f>IF(V16=0,0,W16/V16)</f>
-        <v>5.5994989541841567E-2</v>
+        <v>0</v>
       </c>
       <c r="Y16" s="3">
-        <v>4635731.7964105764</v>
+        <v>4636445.539725238</v>
       </c>
       <c r="Z16" s="3">
-        <v>32670.824420694262</v>
+        <v>33384.56773535628</v>
       </c>
       <c r="AA16" s="4">
         <f>IF(Y16=0,0,Z16/Y16)</f>
-        <v>7.0476088469982488E-3</v>
+        <v>0</v>
       </c>
       <c r="AB16" s="3">
-        <v>153752.5023732449</v>
+        <v>153755.6033474366</v>
       </c>
       <c r="AC16" s="3">
-        <v>310.09741917075007</v>
+        <v>313.1983933624579</v>
       </c>
       <c r="AD16" s="4">
         <f>IF(AB16=0,0,AC16/AB16)</f>
-        <v>2.0168609576055353E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30">
       <c r="B17" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="3">
         <f>J17+M17+G17+P17</f>
-        <v>349.18065136433341</v>
+        <v>0</v>
       </c>
       <c r="D17" s="3">
         <f>G17</f>
-        <v>99.522205969258039</v>
+        <v>0</v>
       </c>
       <c r="E17" s="3">
         <f>J17+M17+P17</f>
-        <v>249.6584453950754</v>
+        <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>288.86678736531792</v>
+        <v>288.7894998187962</v>
       </c>
       <c r="G17" s="3">
-        <v>99.522205969258039</v>
+        <v>99.07282379826836</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
-        <v>0.3445263018188256</v>
+        <v>0</v>
       </c>
       <c r="I17" s="3">
-        <v>3614.3317239066419</v>
+        <v>3607.833411572376</v>
       </c>
       <c r="J17" s="3">
-        <v>223.0981557032205</v>
+        <v>216.8494586088709</v>
       </c>
       <c r="K17" s="4">
         <f>IF(I17=0,0,J17/I17)</f>
-        <v>6.1725976679882395E-2</v>
+        <v>0</v>
       </c>
       <c r="L17" s="3">
-        <v>12916.932829144929</v>
+        <v>12917.49073548635</v>
       </c>
       <c r="M17" s="3">
-        <v>22.595390879644079</v>
+        <v>23.15329722107202</v>
       </c>
       <c r="N17" s="4">
         <f>IF(L17=0,0,M17/L17)</f>
-        <v>1.7492845382505438E-3</v>
+        <v>0</v>
       </c>
       <c r="O17" s="3">
-        <v>380.99541784497882</v>
+        <v>380.9954098585719</v>
       </c>
       <c r="P17" s="3">
-        <v>3.9648988122108282</v>
+        <v>3.964890825803974</v>
       </c>
       <c r="Q17" s="4">
         <f>IF(O17=0,0,P17/O17)</f>
-        <v>1.0406683719813356E-2</v>
+        <v>0</v>
       </c>
       <c r="S17" s="3">
-        <v>3211.1280790807491</v>
+        <v>3210.268928006087</v>
       </c>
       <c r="T17" s="3">
-        <v>1106.3180817522791</v>
+        <v>1101.322617508485</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
-        <v>0.34452630181882538</v>
+        <v>0</v>
       </c>
       <c r="V17" s="3">
-        <v>117876445.53719731</v>
+        <v>117724986.5060492</v>
       </c>
       <c r="W17" s="3">
-        <v>5909428.3290538341</v>
+        <v>5759705.398426414</v>
       </c>
       <c r="X17" s="4">
         <f>IF(V17=0,0,W17/V17)</f>
-        <v>5.0132393304895204E-2</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="3">
-        <v>4171603.1382768038</v>
+        <v>4171333.157109953</v>
       </c>
       <c r="Z17" s="3">
-        <v>27643.588900032919</v>
+        <v>27373.60773318261</v>
       </c>
       <c r="AA17" s="4">
         <f>IF(Y17=0,0,Z17/Y17)</f>
-        <v>6.6266104381760222E-3</v>
+        <v>0</v>
       </c>
       <c r="AB17" s="3">
-        <v>144164.29017248511</v>
+        <v>144170.4921208685</v>
       </c>
       <c r="AC17" s="3">
-        <v>251.178909528302</v>
+        <v>257.3808579117176</v>
       </c>
       <c r="AD17" s="4">
         <f>IF(AB17=0,0,AC17/AB17)</f>
-        <v>1.7423101742309378E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30">
       <c r="B18" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="3">
         <f>J18+M18+G18+P18</f>
-        <v>167.03727252038544</v>
+        <v>0</v>
       </c>
       <c r="D18" s="3">
         <f>G18</f>
-        <v>43.142197183599052</v>
+        <v>0</v>
       </c>
       <c r="E18" s="3">
         <f>J18+M18+P18</f>
-        <v>123.89507533678638</v>
+        <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>239.84852037595849</v>
+        <v>239.8280399304447</v>
       </c>
       <c r="G18" s="3">
-        <v>43.142197183599052</v>
+        <v>42.98112288724334</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
-        <v>0.17987268429246256</v>
+        <v>0</v>
       </c>
       <c r="I18" s="3">
-        <v>3112.2118549380339</v>
+        <v>3109.42846045582</v>
       </c>
       <c r="J18" s="3">
-        <v>109.9352002503402</v>
+        <v>107.3276773510338</v>
       </c>
       <c r="K18" s="4">
         <f>IF(I18=0,0,J18/I18)</f>
-        <v>3.5323816428470316E-2</v>
+        <v>0</v>
       </c>
       <c r="L18" s="3">
-        <v>12351.213483150799</v>
+        <v>12350.65552086042</v>
       </c>
       <c r="M18" s="3">
-        <v>12.841166864847761</v>
+        <v>12.28320457446016</v>
       </c>
       <c r="N18" s="4">
         <f>IF(L18=0,0,M18/L18)</f>
-        <v>1.0396684408673967E-3</v>
+        <v>0</v>
       </c>
       <c r="O18" s="3">
-        <v>348.58104643362333</v>
+        <v>348.5810412050197</v>
       </c>
       <c r="P18" s="3">
-        <v>1.1187082215984121</v>
+        <v>1.118702992994746</v>
       </c>
       <c r="Q18" s="4">
         <f>IF(O18=0,0,P18/O18)</f>
-        <v>3.209320280158824E-3</v>
+        <v>0</v>
       </c>
       <c r="S18" s="3">
-        <v>2666.226621377526</v>
+        <v>2665.998954727921</v>
       </c>
       <c r="T18" s="3">
-        <v>479.58133931919878</v>
+        <v>477.7907901163517</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
-        <v>0.17987268429246253</v>
+        <v>0</v>
       </c>
       <c r="V18" s="3">
-        <v>108133914.5048333</v>
+        <v>108065359.9260122</v>
       </c>
       <c r="W18" s="3">
-        <v>3152520.1315948069</v>
+        <v>3085710.668220431</v>
       </c>
       <c r="X18" s="4">
         <f>IF(V18=0,0,W18/V18)</f>
-        <v>2.9153851925465046E-2</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="3">
-        <v>3758069.5714571462</v>
+        <v>3757886.480780777</v>
       </c>
       <c r="Z18" s="3">
-        <v>10855.1048464654</v>
+        <v>10672.01417009579</v>
       </c>
       <c r="AA18" s="4">
         <f>IF(Y18=0,0,Z18/Y18)</f>
-        <v>2.8884789491154801E-3</v>
+        <v>0</v>
       </c>
       <c r="AB18" s="3">
-        <v>137838.30282140171</v>
+        <v>137832.1008730183</v>
       </c>
       <c r="AC18" s="3">
-        <v>142.64481281855839</v>
+        <v>136.4428644351428</v>
       </c>
       <c r="AD18" s="4">
         <f>IF(AB18=0,0,AC18/AB18)</f>
-        <v>1.034870641169926E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30">
       <c r="A20" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30">
       <c r="B21" t="s">
         <v>28</v>
       </c>
       <c r="C21" s="3">
         <f>C23+C24+C25+C26+C27</f>
-        <v>2035.200376390321</v>
+        <v>0</v>
       </c>
       <c r="D21" s="3">
         <f>D23+D24+D25+D26+D27</f>
-        <v>1075.1027820881895</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3">
         <f>E23+E24+E25+E26+E27</f>
-        <v>960.09759430213182</v>
+        <v>0</v>
       </c>
       <c r="F21" s="3">
         <f>F23+F24+F25+F26+F27</f>
-        <v>1921.9196808294905</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3">
         <f>G23+G24+G25+G26+G27</f>
-        <v>1075.1027820881895</v>
+        <v>0</v>
       </c>
       <c r="H21" s="4">
         <f>IF(F21=0,0,G21/F21)</f>
-        <v>0.55939006859234652</v>
+        <v>0</v>
       </c>
       <c r="I21" s="3">
         <f>I23+I24+I25+I26+I27</f>
-        <v>3682.4352162782898</v>
+        <v>0</v>
       </c>
       <c r="J21" s="3">
         <f>J23+J24+J25+J26+J27</f>
-        <v>692.2560833897752</v>
+        <v>0</v>
       </c>
       <c r="K21" s="4">
         <f>IF(I21=0,0,J21/I21)</f>
-        <v>0.1879886658506961</v>
+        <v>0</v>
       </c>
       <c r="L21" s="3">
         <f>L23+L24+L25+L26+L27</f>
-        <v>75120.106151105079</v>
+        <v>0</v>
       </c>
       <c r="M21" s="3">
         <f>M23+M24+M25+M26+M27</f>
-        <v>207.94835208220408</v>
+        <v>0</v>
       </c>
       <c r="N21" s="4">
         <f>IF(L21=0,0,M21/L21)</f>
-        <v>2.7682116378258737E-3</v>
+        <v>0</v>
       </c>
       <c r="O21" s="3">
         <f>O23+O24+O25+O26+O27</f>
-        <v>1936.1737568351107</v>
+        <v>0</v>
       </c>
       <c r="P21" s="3">
         <f>P23+P24+P25+P26+P27</f>
-        <v>59.8931588301527</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="4">
         <f>IF(O21=0,0,P21/O21)</f>
-        <v>3.0933772663076824E-2</v>
+        <v>0</v>
       </c>
       <c r="S21" s="3">
         <f>S23+S24+S25+S26+S27</f>
-        <v>21364.623843185575</v>
+        <v>0</v>
       </c>
       <c r="T21" s="3">
         <f>T23+T24+T25+T26+T27</f>
-        <v>11951.158397089261</v>
+        <v>0</v>
       </c>
       <c r="U21" s="4">
         <f>IF(S21=0,0,T21/S21)</f>
-        <v>0.55939006859234652</v>
+        <v>0</v>
       </c>
       <c r="V21" s="3">
         <f>V23+V24+V25+V26+V27</f>
-        <v>106670224.92367341</v>
+        <v>0</v>
       </c>
       <c r="W21" s="3">
         <f>W23+W24+W25+W26+W27</f>
-        <v>16637355.760071689</v>
+        <v>0</v>
       </c>
       <c r="X21" s="4">
         <f>IF(V21=0,0,W21/V21)</f>
-        <v>0.15597000730031599</v>
+        <v>0</v>
       </c>
       <c r="Y21" s="3">
         <f>Y23+Y24+Y25+Y26+Y27</f>
-        <v>8082003.8383214176</v>
+        <v>0</v>
       </c>
       <c r="Z21" s="3">
         <f>Z23+Z24+Z25+Z26+Z27</f>
-        <v>258149.94787068455</v>
+        <v>0</v>
       </c>
       <c r="AA21" s="4">
         <f>IF(Y21=0,0,Z21/Y21)</f>
-        <v>3.1941329531006597E-2</v>
+        <v>0</v>
       </c>
       <c r="AB21" s="3">
         <f>AB23+AB24+AB25+AB26+AB27</f>
-        <v>844449.53447731666</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="3">
         <f>AC23+AC24+AC25+AC26+AC27</f>
-        <v>2308.9046278140158</v>
+        <v>0</v>
       </c>
       <c r="AD21" s="4">
         <f>IF(AB21=0,0,AC21/AB21)</f>
-        <v>2.7342126835834461E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30">
       <c r="A22" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30">
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="3">
         <f>J23+M23+G23+P23</f>
-        <v>532.13937442389363</v>
+        <v>0</v>
       </c>
       <c r="D23" s="3">
         <f>G23</f>
-        <v>277.48144279559938</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3">
         <f>J23+M23+P23</f>
-        <v>254.65793162829431</v>
+        <v>0</v>
       </c>
       <c r="F23" s="3">
-        <v>428.09244082133358</v>
+        <v>428.0924408213336</v>
       </c>
       <c r="G23" s="3">
-        <v>277.48144279559938</v>
+        <v>277.4814427955992</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
-        <v>0.64818113177431125</v>
+        <v>0</v>
       </c>
       <c r="I23" s="3">
-        <v>991.82050542122556</v>
+        <v>991.8205054212256</v>
       </c>
       <c r="J23" s="3">
-        <v>166.97305006018021</v>
+        <v>161.3467046339945</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
-        <v>0.16835006853308287</v>
+        <v>0</v>
       </c>
       <c r="L23" s="3">
-        <v>18248.150900694091</v>
+        <v>18248.15090069409</v>
       </c>
       <c r="M23" s="3">
-        <v>73.907573516033594</v>
+        <v>74.96112067504973</v>
       </c>
       <c r="N23" s="4">
         <f>IF(L23=0,0,M23/L23)</f>
-        <v>4.0501404179654407E-3</v>
+        <v>0</v>
       </c>
       <c r="O23" s="3">
-        <v>476.04818802351332</v>
+        <v>476.0481880235133</v>
       </c>
       <c r="P23" s="3">
-        <v>13.77730805208051</v>
+        <v>14.3034626128918</v>
       </c>
       <c r="Q23" s="4">
         <f>IF(O23=0,0,P23/O23)</f>
-        <v>2.894099462762793E-2</v>
+        <v>0</v>
       </c>
       <c r="S23" s="3">
-        <v>4758.8013481976486</v>
+        <v>4758.801348197649</v>
       </c>
       <c r="T23" s="3">
-        <v>3084.565243763871</v>
+        <v>3084.565243763868</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
-        <v>0.64818113177431147</v>
+        <v>0</v>
       </c>
       <c r="V23" s="3">
-        <v>25699987.560610589</v>
+        <v>25699987.56061059</v>
       </c>
       <c r="W23" s="3">
-        <v>3401420.686246444</v>
+        <v>3287127.85436815</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
-        <v>0.13235106352579232</v>
+        <v>0</v>
       </c>
       <c r="Y23" s="3">
-        <v>1959206.3612258229</v>
+        <v>1959206.361225823</v>
       </c>
       <c r="Z23" s="3">
-        <v>65082.608297784107</v>
+        <v>68388.33434051392</v>
       </c>
       <c r="AA23" s="4">
         <f>IF(Y23=0,0,Z23/Y23)</f>
-        <v>3.3218863303947042E-2</v>
+        <v>0</v>
       </c>
       <c r="AB23" s="3">
-        <v>205054.68928072241</v>
+        <v>205054.6892807224</v>
       </c>
       <c r="AC23" s="3">
-        <v>820.51982641321956</v>
+        <v>832.1809608971234</v>
       </c>
       <c r="AD23" s="4">
         <f>IF(AB23=0,0,AC23/AB23)</f>
-        <v>4.0014682389921735E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30">
       <c r="B24" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="3">
         <f>J24+M24+G24+P24</f>
-        <v>505.78668747185765</v>
+        <v>0</v>
       </c>
       <c r="D24" s="3">
         <f>G24</f>
-        <v>273.77050166811699</v>
+        <v>0</v>
       </c>
       <c r="E24" s="3">
         <f>J24+M24+P24</f>
-        <v>232.01618580374068</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>437.75116549754102</v>
+        <v>437.751165497541</v>
       </c>
       <c r="G24" s="3">
-        <v>273.77050166811699</v>
+        <v>273.7705016681168</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
-        <v>0.62540210796915596</v>
+        <v>0</v>
       </c>
       <c r="I24" s="3">
-        <v>847.52939170447485</v>
+        <v>847.5293917044748</v>
       </c>
       <c r="J24" s="3">
-        <v>153.3462496447697</v>
+        <v>150.8080230775032</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
-        <v>0.18093325275289099</v>
+        <v>0</v>
       </c>
       <c r="L24" s="3">
         <v>18442.648959675</v>
       </c>
       <c r="M24" s="3">
-        <v>61.556604397132993</v>
+        <v>61.83910950501263</v>
       </c>
       <c r="N24" s="4">
         <f>IF(L24=0,0,M24/L24)</f>
-        <v>3.3377311758048967E-3</v>
+        <v>0</v>
       </c>
       <c r="O24" s="3">
-        <v>476.56393826290048</v>
+        <v>476.5639382629005</v>
       </c>
       <c r="P24" s="3">
-        <v>17.113331761837991</v>
+        <v>17.72296783017885</v>
       </c>
       <c r="Q24" s="4">
         <f>IF(O24=0,0,P24/O24)</f>
-        <v>3.5909833681954502E-2</v>
+        <v>0</v>
       </c>
       <c r="S24" s="3">
-        <v>4866.1705694873763</v>
+        <v>4866.170569487376</v>
       </c>
       <c r="T24" s="3">
-        <v>3043.313331894874</v>
+        <v>3043.313331894871</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
-        <v>0.62540210796915607</v>
+        <v>0</v>
       </c>
       <c r="V24" s="3">
-        <v>23322467.600951109</v>
+        <v>23322467.60095111</v>
       </c>
       <c r="W24" s="3">
-        <v>3423888.8638618961</v>
+        <v>3365842.996704068</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
-        <v>0.14680645815206395</v>
+        <v>0</v>
       </c>
       <c r="Y24" s="3">
-        <v>2033978.1299748039</v>
+        <v>2033978.129974804</v>
       </c>
       <c r="Z24" s="3">
-        <v>70352.468004657887</v>
+        <v>72763.09209677344</v>
       </c>
       <c r="AA24" s="4">
         <f>IF(Y24=0,0,Z24/Y24)</f>
-        <v>3.4588605928387924E-2</v>
+        <v>0</v>
       </c>
       <c r="AB24" s="3">
-        <v>207305.28823611679</v>
+        <v>207305.2882361168</v>
       </c>
       <c r="AC24" s="3">
-        <v>683.76652201107936</v>
+        <v>686.9468314157566</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(AB24=0,0,AC24/AB24)</f>
-        <v>3.2983554246444609E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30">
       <c r="B25" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="3">
         <f>J25+M25+G25+P25</f>
-        <v>400.63814719596553</v>
+        <v>0</v>
       </c>
       <c r="D25" s="3">
         <f>G25</f>
-        <v>214.28435758159819</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3">
         <f>J25+M25+P25</f>
-        <v>186.35378961436732</v>
+        <v>0</v>
       </c>
       <c r="F25" s="3">
-        <v>396.28526128416758</v>
+        <v>396.2852612841676</v>
       </c>
       <c r="G25" s="3">
-        <v>214.28435758159819</v>
+        <v>214.2843575815979</v>
       </c>
       <c r="H25" s="4">
         <f>IF(F25=0,0,G25/F25)</f>
-        <v>0.54073259471524859</v>
+        <v>0</v>
       </c>
       <c r="I25" s="3">
-        <v>721.62080381298233</v>
+        <v>721.6208038129823</v>
       </c>
       <c r="J25" s="3">
-        <v>137.51098482848519</v>
+        <v>136.4734691339483</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
-        <v>0.19055850954114539</v>
+        <v>0</v>
       </c>
       <c r="L25" s="3">
-        <v>15355.961975565249</v>
+        <v>15355.96197556525</v>
       </c>
       <c r="M25" s="3">
-        <v>36.005612529100851</v>
+        <v>35.52823494572937</v>
       </c>
       <c r="N25" s="4">
         <f>IF(L25=0,0,M25/L25)</f>
-        <v>2.3447318107712033E-3</v>
+        <v>0</v>
       </c>
       <c r="O25" s="3">
         <v>391.5266582641886</v>
       </c>
       <c r="P25" s="3">
-        <v>12.83719225678127</v>
+        <v>12.97225060199702</v>
       </c>
       <c r="Q25" s="4">
         <f>IF(O25=0,0,P25/O25)</f>
-        <v>3.2787530518852123E-2</v>
+        <v>0</v>
       </c>
       <c r="S25" s="3">
-        <v>4405.2233953297473</v>
+        <v>4405.223395329747</v>
       </c>
       <c r="T25" s="3">
-        <v>2382.047876856971</v>
+        <v>2382.047876856968</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
-        <v>0.54073259471524848</v>
+        <v>0</v>
       </c>
       <c r="V25" s="3">
-        <v>21162807.846375171</v>
+        <v>21162807.84637517</v>
       </c>
       <c r="W25" s="3">
-        <v>3337513.1796382521</v>
+        <v>3312150.152959324</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
-        <v>0.15770653893688835</v>
+        <v>0</v>
       </c>
       <c r="Y25" s="3">
         <v>1664123.912966297</v>
       </c>
       <c r="Z25" s="3">
-        <v>53910.802672466729</v>
+        <v>54164.27348549617</v>
       </c>
       <c r="AA25" s="4">
         <f>IF(Y25=0,0,Z25/Y25)</f>
-        <v>3.2395906490142824E-2</v>
+        <v>0</v>
       </c>
       <c r="AB25" s="3">
         <v>172634.6152091868</v>
       </c>
       <c r="AC25" s="3">
-        <v>399.65888185758382</v>
+        <v>394.3583661830926</v>
       </c>
       <c r="AD25" s="4">
         <f>IF(AB25=0,0,AC25/AB25)</f>
-        <v>2.3150564640428838E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30">
       <c r="B26" t="s">
         <v>33</v>
       </c>
       <c r="C26" s="3">
         <f>J26+M26+G26+P26</f>
-        <v>331.14701605525443</v>
+        <v>0</v>
       </c>
       <c r="D26" s="3">
         <f>G26</f>
-        <v>169.09086715748001</v>
+        <v>0</v>
       </c>
       <c r="E26" s="3">
         <f>J26+M26+P26</f>
-        <v>162.05614889777445</v>
+        <v>0</v>
       </c>
       <c r="F26" s="3">
-        <v>351.26672270713158</v>
+        <v>351.2667227071316</v>
       </c>
       <c r="G26" s="3">
-        <v>169.09086715748001</v>
+        <v>169.09086715748</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
-        <v>0.48137456874461582</v>
+        <v>0</v>
       </c>
       <c r="I26" s="3">
-        <v>656.23600296293523</v>
+        <v>656.2360029629352</v>
       </c>
       <c r="J26" s="3">
-        <v>131.22809870126761</v>
+        <v>129.4537897061268</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
-        <v>0.19997089173523977</v>
+        <v>0</v>
       </c>
       <c r="L26" s="3">
-        <v>12320.893910346331</v>
+        <v>12320.89391034633</v>
       </c>
       <c r="M26" s="3">
-        <v>21.953041641423479</v>
+        <v>22.14377215228788</v>
       </c>
       <c r="N26" s="4">
         <f>IF(L26=0,0,M26/L26)</f>
-        <v>1.7817734493264861E-3</v>
+        <v>0</v>
       </c>
       <c r="O26" s="3">
-        <v>305.89771512841492</v>
+        <v>305.8977151284149</v>
       </c>
       <c r="P26" s="3">
-        <v>8.8750085550833617</v>
+        <v>8.938968257547996</v>
       </c>
       <c r="Q26" s="4">
         <f>IF(O26=0,0,P26/O26)</f>
-        <v>2.9012993939355382E-2</v>
+        <v>0</v>
       </c>
       <c r="S26" s="3">
-        <v>3904.7840938011818</v>
+        <v>3904.784093801182</v>
       </c>
       <c r="T26" s="3">
         <v>1879.66375919438</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
-        <v>0.48137456874461598</v>
+        <v>0</v>
       </c>
       <c r="V26" s="3">
-        <v>20232379.411657181</v>
+        <v>20232379.41165718</v>
       </c>
       <c r="W26" s="3">
-        <v>3377261.9696825258</v>
+        <v>3331387.450043749</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
-        <v>0.16692361787841262</v>
+        <v>0</v>
       </c>
       <c r="Y26" s="3">
-        <v>1291512.2728871789</v>
+        <v>1291512.272887179</v>
       </c>
       <c r="Z26" s="3">
-        <v>35946.191367430612</v>
+        <v>36162.54302373994</v>
       </c>
       <c r="AA26" s="4">
         <f>IF(Y26=0,0,Z26/Y26)</f>
-        <v>2.7832636299361533E-2</v>
+        <v>0</v>
       </c>
       <c r="AB26" s="3">
-        <v>138538.51808137319</v>
+        <v>138538.5180813732</v>
       </c>
       <c r="AC26" s="3">
-        <v>243.82372102720549</v>
+        <v>245.9439272969903</v>
       </c>
       <c r="AD26" s="4">
         <f>IF(AB26=0,0,AC26/AB26)</f>
-        <v>1.7599706161429494E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30">
       <c r="B27" t="s">
         <v>34</v>
       </c>
       <c r="C27" s="3">
         <f>J27+M27+G27+P27</f>
-        <v>265.48915124334991</v>
+        <v>0</v>
       </c>
       <c r="D27" s="3">
         <f>G27</f>
-        <v>140.47561288539481</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3">
         <f>J27+M27+P27</f>
-        <v>125.01353835795513</v>
+        <v>0</v>
       </c>
       <c r="F27" s="3">
-        <v>308.52409051931693</v>
+        <v>308.5240905193169</v>
       </c>
       <c r="G27" s="3">
-        <v>140.47561288539481</v>
+        <v>140.4756128853948</v>
       </c>
       <c r="H27" s="4">
         <f>IF(F27=0,0,G27/F27)</f>
-        <v>0.4553148917769827</v>
+        <v>0</v>
       </c>
       <c r="I27" s="3">
-        <v>465.22851237667129</v>
+        <v>465.2285123766713</v>
       </c>
       <c r="J27" s="3">
-        <v>103.1977001550724</v>
+        <v>101.8160884284314</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
-        <v>0.22182152944125358</v>
+        <v>0</v>
       </c>
       <c r="L27" s="3">
-        <v>10752.450404824391</v>
+        <v>10752.45040482439</v>
       </c>
       <c r="M27" s="3">
-        <v>14.525519998513159</v>
+        <v>14.61954391417466</v>
       </c>
       <c r="N27" s="4">
         <f>IF(L27=0,0,M27/L27)</f>
-        <v>1.3509032315085941E-3</v>
+        <v>0</v>
       </c>
       <c r="O27" s="3">
-        <v>286.13725715609343</v>
+        <v>286.1372571560934</v>
       </c>
       <c r="P27" s="3">
-        <v>7.2903182043695702</v>
+        <v>7.424886429645645</v>
       </c>
       <c r="Q27" s="4">
         <f>IF(O27=0,0,P27/O27)</f>
-        <v>2.5478395497418781E-2</v>
+        <v>0</v>
       </c>
       <c r="S27" s="3">
-        <v>3429.6444363696219</v>
+        <v>3429.644436369622</v>
       </c>
       <c r="T27" s="3">
         <v>1561.568185379165</v>
       </c>
       <c r="U27" s="4">
         <f>IF(S27=0,0,T27/S27)</f>
-        <v>0.45531489177698264</v>
+        <v>0</v>
       </c>
       <c r="V27" s="3">
-        <v>16252582.504079361</v>
+        <v>16252582.50407936</v>
       </c>
       <c r="W27" s="3">
-        <v>3097271.0606425721</v>
+        <v>3055534.524638651</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
-        <v>0.19057100986044306</v>
+        <v>0</v>
       </c>
       <c r="Y27" s="3">
         <v>1133183.161267315</v>
       </c>
       <c r="Z27" s="3">
-        <v>32857.877528345212</v>
+        <v>33166.49680278706</v>
       </c>
       <c r="AA27" s="4">
         <f>IF(Y27=0,0,Z27/Y27)</f>
-        <v>2.8996086997620081E-2</v>
+        <v>0</v>
       </c>
       <c r="AB27" s="3">
-        <v>120916.42366991749</v>
+        <v>120916.4236699175</v>
       </c>
       <c r="AC27" s="3">
-        <v>161.13567650492769</v>
+        <v>162.1957796398201</v>
       </c>
       <c r="AD27" s="4">
         <f>IF(AB27=0,0,AC27/AB27)</f>
-        <v>1.3326202645953401E-3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30">
       <c r="A29" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30">
       <c r="B30" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="3">
         <f>C32+C33+C34+C35+C36</f>
-        <v>252.98081722758172</v>
+        <v>0</v>
       </c>
       <c r="D30" s="3">
         <f>D32+D33+D34+D35+D36</f>
-        <v>252.98081722758172</v>
+        <v>0</v>
       </c>
       <c r="E30" s="3">
         <f>E32+E33+E34+E35+E36</f>
@@ -2595,27 +2569,27 @@
       </c>
       <c r="F30" s="3">
         <f>F32+F33+F34+F35+F36</f>
-        <v>660.80113298361266</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3">
         <f>G32+G33+G34+G35+G36</f>
-        <v>245.1322541365746</v>
+        <v>0</v>
       </c>
       <c r="H30" s="4">
         <f>IF(F30=0,0,G30/F30)</f>
-        <v>0.37096221828459497</v>
+        <v>0</v>
       </c>
       <c r="I30" s="3">
         <f>I32+I33+I34+I35+I36</f>
-        <v>814.53034621778045</v>
-      </c>
-      <c r="J30" s="6">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3">
         <f>J32+J33+J34+J35+J36</f>
-        <v>7.8485630910071178</v>
-      </c>
-      <c r="K30" s="7">
+        <v>0</v>
+      </c>
+      <c r="K30" s="4">
         <f>IF(I30=0,0,J30/I30)</f>
-        <v>9.6356914477789789E-3</v>
+        <v>0</v>
       </c>
       <c r="L30" s="3">
         <f>L32+L33+L34+L35+L36</f>
@@ -2643,27 +2617,27 @@
       </c>
       <c r="S30" s="3">
         <f>S32+S33+S34+S35+S36</f>
-        <v>7345.6595414292105</v>
+        <v>0</v>
       </c>
       <c r="T30" s="3">
         <f>T32+T33+T34+T35+T36</f>
-        <v>2724.9621582519808</v>
+        <v>0</v>
       </c>
       <c r="U30" s="4">
         <f>IF(S30=0,0,T30/S30)</f>
-        <v>0.37096221828459497</v>
+        <v>0</v>
       </c>
       <c r="V30" s="3">
         <f>V32+V33+V34+V35+V36</f>
-        <v>26890169.836246081</v>
-      </c>
-      <c r="W30" s="6">
+        <v>0</v>
+      </c>
+      <c r="W30" s="3">
         <f>W32+W33+W34+W35+W36</f>
-        <v>292255.43316228967</v>
-      </c>
-      <c r="X30" s="7">
+        <v>0</v>
+      </c>
+      <c r="X30" s="4">
         <f>IF(V30=0,0,W30/V30)</f>
-        <v>1.086848595386518E-2</v>
+        <v>0</v>
       </c>
       <c r="Y30" s="3">
         <f>Y32+Y33+Y34+Y35+Y36</f>
@@ -2690,512 +2664,512 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30">
       <c r="A31" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30">
       <c r="B32" t="s">
         <v>30</v>
       </c>
       <c r="C32" s="3">
         <f>J32+M32+G32+P32</f>
-        <v>73.82106874493499</v>
+        <v>0</v>
       </c>
       <c r="D32" s="3">
-        <f>G32+J32</f>
-        <v>73.82106874493499</v>
+        <f>G32</f>
+        <v>0</v>
       </c>
       <c r="E32" s="3">
-        <f>M32+P32</f>
+        <f>J32+M32+P32</f>
         <v>0</v>
       </c>
       <c r="F32" s="3">
-        <v>158.01636350616181</v>
+        <v>428.0924408213336</v>
       </c>
       <c r="G32" s="3">
-        <v>71.120547266421269</v>
+        <v>17.02603595398361</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
-        <v>0.45008343242659132</v>
+        <v>0</v>
       </c>
       <c r="I32" s="3">
-        <v>289.90090139463632</v>
-      </c>
-      <c r="J32" s="6">
-        <v>2.7005214785137208</v>
-      </c>
-      <c r="K32" s="7">
+        <v>991.8205054212256</v>
+      </c>
+      <c r="J32" s="3">
+        <v>13.27426398876158</v>
+      </c>
+      <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
-        <v>9.3153262563939205E-3</v>
+        <v>0</v>
       </c>
       <c r="L32" s="3">
-        <v>0</v>
+        <v>18248.15090069409</v>
       </c>
       <c r="M32" s="3">
-        <v>0</v>
+        <v>1.053563024971634</v>
       </c>
       <c r="N32" s="4">
         <f>IF(L32=0,0,M32/L32)</f>
         <v>0</v>
       </c>
       <c r="O32" s="3">
-        <v>0</v>
+        <v>476.0481880235133</v>
       </c>
       <c r="P32" s="3">
-        <v>0</v>
+        <v>4.400421166792512E-07</v>
       </c>
       <c r="Q32" s="4">
         <f>IF(O32=0,0,P32/O32)</f>
         <v>0</v>
       </c>
       <c r="S32" s="3">
-        <v>1756.5563228532919</v>
+        <v>4758.801348197649</v>
       </c>
       <c r="T32" s="3">
-        <v>790.59689904044183</v>
+        <v>189.2664180120255</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
-        <v>0.4500834324265916</v>
+        <v>0</v>
       </c>
       <c r="V32" s="3">
-        <v>7917202.4300766056</v>
-      </c>
-      <c r="W32" s="6">
-        <v>79522.935220028274</v>
-      </c>
-      <c r="X32" s="7">
+        <v>25699987.56061059</v>
+      </c>
+      <c r="W32" s="3">
+        <v>265621.4381604269</v>
+      </c>
+      <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
-        <v>1.004432259025349E-2</v>
+        <v>0</v>
       </c>
       <c r="Y32" s="3">
-        <v>0</v>
+        <v>1959206.361225823</v>
       </c>
       <c r="Z32" s="3">
-        <v>0</v>
+        <v>16.96875735768117</v>
       </c>
       <c r="AA32" s="4">
         <f>IF(Y32=0,0,Z32/Y32)</f>
         <v>0</v>
       </c>
       <c r="AB32" s="3">
-        <v>0</v>
+        <v>205054.6892807224</v>
       </c>
       <c r="AC32" s="3">
-        <v>0</v>
+        <v>11.66113448393298</v>
       </c>
       <c r="AD32" s="4">
         <f>IF(AB32=0,0,AC32/AB32)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30">
       <c r="B33" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="3">
         <f>J33+M33+G33+P33</f>
-        <v>66.051288895629042</v>
+        <v>0</v>
       </c>
       <c r="D33" s="3">
-        <f>G33+J33</f>
-        <v>66.051288895629042</v>
+        <f>G33</f>
+        <v>0</v>
       </c>
       <c r="E33" s="3">
-        <f>M33+P33</f>
+        <f>J33+M33+P33</f>
         <v>0</v>
       </c>
       <c r="F33" s="3">
-        <v>150.30970532381971</v>
+        <v>437.751165497541</v>
       </c>
       <c r="G33" s="3">
-        <v>64.218379853471717</v>
+        <v>33.74848177556315</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
-        <v>0.42724040816341735</v>
+        <v>0</v>
       </c>
       <c r="I33" s="3">
-        <v>172.51020331953049</v>
-      </c>
-      <c r="J33" s="6">
-        <v>1.83290904215732</v>
-      </c>
-      <c r="K33" s="7">
+        <v>847.5293917044748</v>
+      </c>
+      <c r="J33" s="3">
+        <v>15.93424343309703</v>
+      </c>
+      <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
-        <v>1.0624931203416012E-2</v>
+        <v>0</v>
       </c>
       <c r="L33" s="3">
-        <v>0</v>
+        <v>18442.648959675</v>
       </c>
       <c r="M33" s="3">
-        <v>0</v>
+        <v>1.708336847607046</v>
       </c>
       <c r="N33" s="4">
         <f>IF(L33=0,0,M33/L33)</f>
         <v>0</v>
       </c>
       <c r="O33" s="3">
-        <v>0</v>
+        <v>476.5639382629005</v>
       </c>
       <c r="P33" s="3">
-        <v>0</v>
+        <v>2.734852547291666E-06</v>
       </c>
       <c r="Q33" s="4">
         <f>IF(O33=0,0,P33/O33)</f>
         <v>0</v>
       </c>
       <c r="S33" s="3">
-        <v>1670.8868462377629</v>
+        <v>4866.170569487376</v>
       </c>
       <c r="T33" s="3">
-        <v>713.87037818150714</v>
+        <v>375.1580389157161</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
-        <v>0.42724040816341741</v>
+        <v>0</v>
       </c>
       <c r="V33" s="3">
-        <v>5775458.9344058</v>
-      </c>
-      <c r="W33" s="6">
-        <v>71151.412156144157</v>
-      </c>
-      <c r="X33" s="7">
+        <v>23322467.60095111</v>
+      </c>
+      <c r="W33" s="3">
+        <v>353266.0783004276</v>
+      </c>
+      <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
-        <v>1.2319611820331379E-2</v>
+        <v>0</v>
       </c>
       <c r="Y33" s="3">
-        <v>0</v>
+        <v>2033978.129974804</v>
       </c>
       <c r="Z33" s="3">
-        <v>0</v>
+        <v>101.8125441458542</v>
       </c>
       <c r="AA33" s="4">
         <f>IF(Y33=0,0,Z33/Y33)</f>
         <v>0</v>
       </c>
       <c r="AB33" s="3">
-        <v>0</v>
+        <v>207305.2882361168</v>
       </c>
       <c r="AC33" s="3">
-        <v>0</v>
+        <v>19.08185642829631</v>
       </c>
       <c r="AD33" s="4">
         <f>IF(AB33=0,0,AC33/AB33)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30">
       <c r="B34" t="s">
         <v>32</v>
       </c>
       <c r="C34" s="3">
         <f>J34+M34+G34+P34</f>
-        <v>65.437886901995398</v>
+        <v>0</v>
       </c>
       <c r="D34" s="3">
-        <f>G34+J34</f>
-        <v>65.437886901995398</v>
+        <f>G34</f>
+        <v>0</v>
       </c>
       <c r="E34" s="3">
-        <f>M34+P34</f>
+        <f>J34+M34+P34</f>
         <v>0</v>
       </c>
       <c r="F34" s="3">
-        <v>136.8081181206467</v>
+        <v>396.2852612841676</v>
       </c>
       <c r="G34" s="3">
-        <v>63.504190897818653</v>
+        <v>42.55442586053192</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
-        <v>0.46418437568022347</v>
+        <v>0</v>
       </c>
       <c r="I34" s="3">
-        <v>135.45605543604131</v>
-      </c>
-      <c r="J34" s="6">
-        <v>1.933696004176745</v>
-      </c>
-      <c r="K34" s="7">
+        <v>721.6208038129823</v>
+      </c>
+      <c r="J34" s="3">
+        <v>17.59058517312794</v>
+      </c>
+      <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
-        <v>1.4275448948753598E-2</v>
+        <v>0</v>
       </c>
       <c r="L34" s="3">
-        <v>0</v>
+        <v>15355.96197556525</v>
       </c>
       <c r="M34" s="3">
-        <v>0</v>
+        <v>1.813587757010013</v>
       </c>
       <c r="N34" s="4">
         <f>IF(L34=0,0,M34/L34)</f>
         <v>0</v>
       </c>
       <c r="O34" s="3">
-        <v>0</v>
+        <v>391.5266582641886</v>
       </c>
       <c r="P34" s="3">
-        <v>0</v>
+        <v>8.800494251772761E-07</v>
       </c>
       <c r="Q34" s="4">
         <f>IF(O34=0,0,P34/O34)</f>
         <v>0</v>
       </c>
       <c r="S34" s="3">
-        <v>1520.7992360431149</v>
+        <v>4405.223395329747</v>
       </c>
       <c r="T34" s="3">
-        <v>705.93124391763399</v>
+        <v>473.0475006013803</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
-        <v>0.46418437568022342</v>
+        <v>0</v>
       </c>
       <c r="V34" s="3">
-        <v>4941006.3189266957</v>
-      </c>
-      <c r="W34" s="6">
-        <v>79056.746527970769</v>
-      </c>
-      <c r="X34" s="7">
+        <v>21162807.84637517</v>
+      </c>
+      <c r="W34" s="3">
+        <v>423351.1303020306</v>
+      </c>
+      <c r="X34" s="4">
         <f>IF(V34=0,0,W34/V34)</f>
-        <v>1.6000130626253436E-2</v>
+        <v>0</v>
       </c>
       <c r="Y34" s="3">
-        <v>0</v>
+        <v>1664123.912966297</v>
       </c>
       <c r="Z34" s="3">
-        <v>0</v>
+        <v>34.99806205020286</v>
       </c>
       <c r="AA34" s="4">
         <f>IF(Y34=0,0,Z34/Y34)</f>
         <v>0</v>
       </c>
       <c r="AB34" s="3">
-        <v>0</v>
+        <v>172634.6152091868</v>
       </c>
       <c r="AC34" s="3">
-        <v>0</v>
+        <v>20.14195956310141</v>
       </c>
       <c r="AD34" s="4">
         <f>IF(AB34=0,0,AC34/AB34)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30">
       <c r="B35" t="s">
         <v>33</v>
       </c>
       <c r="C35" s="3">
         <f>J35+M35+G35+P35</f>
-        <v>29.385977025459027</v>
+        <v>0</v>
       </c>
       <c r="D35" s="3">
-        <f>G35+J35</f>
-        <v>29.385977025459027</v>
+        <f>G35</f>
+        <v>0</v>
       </c>
       <c r="E35" s="3">
-        <f>M35+P35</f>
+        <f>J35+M35+P35</f>
         <v>0</v>
       </c>
       <c r="F35" s="3">
-        <v>120.55842024780129</v>
+        <v>351.2667227071316</v>
       </c>
       <c r="G35" s="3">
-        <v>28.61946098787946</v>
+        <v>50.15844948604295</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
-        <v>0.23739080960959599</v>
+        <v>0</v>
       </c>
       <c r="I35" s="3">
-        <v>131.31388542968341</v>
-      </c>
-      <c r="J35" s="6">
-        <v>0.76651603757956766</v>
-      </c>
-      <c r="K35" s="7">
+        <v>656.2360029629352</v>
+      </c>
+      <c r="J35" s="3">
+        <v>19.57495471003908</v>
+      </c>
+      <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
-        <v>5.8372809171808818E-3</v>
+        <v>0</v>
       </c>
       <c r="L35" s="3">
-        <v>0</v>
+        <v>12320.89391034633</v>
       </c>
       <c r="M35" s="3">
-        <v>0</v>
+        <v>0.7611593206617981</v>
       </c>
       <c r="N35" s="4">
         <f>IF(L35=0,0,M35/L35)</f>
         <v>0</v>
       </c>
       <c r="O35" s="3">
-        <v>0</v>
+        <v>305.8977151284149</v>
       </c>
       <c r="P35" s="3">
-        <v>0</v>
+        <v>0.07876691888418282</v>
       </c>
       <c r="Q35" s="4">
         <f>IF(O35=0,0,P35/O35)</f>
         <v>0</v>
       </c>
       <c r="S35" s="3">
-        <v>1340.1628202336269</v>
+        <v>3904.784093801182</v>
       </c>
       <c r="T35" s="3">
-        <v>318.14233690394002</v>
+        <v>557.5760613285502</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
-        <v>0.23739080960959591</v>
+        <v>0</v>
       </c>
       <c r="V35" s="3">
-        <v>4714339.9302510964</v>
-      </c>
-      <c r="W35" s="6">
-        <v>33401.84311571531</v>
-      </c>
-      <c r="X35" s="7">
+        <v>20232379.41165718</v>
+      </c>
+      <c r="W35" s="3">
+        <v>498928.1711215638</v>
+      </c>
+      <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
-        <v>7.0851579669470831E-3</v>
+        <v>0</v>
       </c>
       <c r="Y35" s="3">
-        <v>0</v>
+        <v>1291512.272887179</v>
       </c>
       <c r="Z35" s="3">
-        <v>0</v>
+        <v>3.181642004521564</v>
       </c>
       <c r="AA35" s="4">
         <f>IF(Y35=0,0,Z35/Y35)</f>
         <v>0</v>
       </c>
       <c r="AB35" s="3">
-        <v>0</v>
+        <v>138538.5180813732</v>
       </c>
       <c r="AC35" s="3">
-        <v>0</v>
+        <v>8.480825079226634</v>
       </c>
       <c r="AD35" s="4">
         <f>IF(AB35=0,0,AC35/AB35)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30">
       <c r="B36" t="s">
         <v>34</v>
       </c>
       <c r="C36" s="3">
         <f>J36+M36+G36+P36</f>
-        <v>18.284595659563276</v>
+        <v>0</v>
       </c>
       <c r="D36" s="3">
-        <f>G36+J36</f>
-        <v>18.284595659563276</v>
+        <f>G36</f>
+        <v>0</v>
       </c>
       <c r="E36" s="3">
-        <f>M36+P36</f>
+        <f>J36+M36+P36</f>
         <v>0</v>
       </c>
       <c r="F36" s="3">
-        <v>95.10852578518319</v>
+        <v>308.5240905193169</v>
       </c>
       <c r="G36" s="3">
-        <v>17.66967513098351</v>
+        <v>48.89042151910646</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
-        <v>0.18578434462219623</v>
+        <v>0</v>
       </c>
       <c r="I36" s="3">
-        <v>85.349300637888987</v>
-      </c>
-      <c r="J36" s="6">
-        <v>0.6149205285797652</v>
-      </c>
-      <c r="K36" s="7">
+        <v>465.2285123766713</v>
+      </c>
+      <c r="J36" s="3">
+        <v>16.59646397136233</v>
+      </c>
+      <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
-        <v>7.2047518138278034E-3</v>
+        <v>0</v>
       </c>
       <c r="L36" s="3">
-        <v>0</v>
+        <v>10752.45040482439</v>
       </c>
       <c r="M36" s="3">
-        <v>0</v>
+        <v>2.380907366001979</v>
       </c>
       <c r="N36" s="4">
         <f>IF(L36=0,0,M36/L36)</f>
         <v>0</v>
       </c>
       <c r="O36" s="3">
-        <v>0</v>
+        <v>286.1372571560934</v>
       </c>
       <c r="P36" s="3">
-        <v>0</v>
+        <v>2.980956342071295E-07</v>
       </c>
       <c r="Q36" s="4">
         <f>IF(O36=0,0,P36/O36)</f>
         <v>0</v>
       </c>
       <c r="S36" s="3">
-        <v>1057.2543160614141</v>
+        <v>3429.644436369622</v>
       </c>
       <c r="T36" s="3">
-        <v>196.42130020845809</v>
+        <v>543.4802898941557</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
-        <v>0.1857843446221962</v>
+        <v>0</v>
       </c>
       <c r="V36" s="3">
-        <v>3542162.2225858839</v>
-      </c>
-      <c r="W36" s="6">
-        <v>29122.496142431159</v>
-      </c>
-      <c r="X36" s="7">
+        <v>16252582.50407936</v>
+      </c>
+      <c r="W36" s="3">
+        <v>494248.2701021787</v>
+      </c>
+      <c r="X36" s="4">
         <f>IF(V36=0,0,W36/V36)</f>
-        <v>8.2216720501216544E-3</v>
+        <v>0</v>
       </c>
       <c r="Y36" s="3">
-        <v>0</v>
+        <v>1133183.161267315</v>
       </c>
       <c r="Z36" s="3">
-        <v>0</v>
+        <v>8.484378678957</v>
       </c>
       <c r="AA36" s="4">
         <f>IF(Y36=0,0,Z36/Y36)</f>
         <v>0</v>
       </c>
       <c r="AB36" s="3">
-        <v>0</v>
+        <v>120916.4236699175</v>
       </c>
       <c r="AC36" s="3">
-        <v>0</v>
+        <v>26.50257837252866</v>
       </c>
       <c r="AD36" s="4">
         <f>IF(AB36=0,0,AC36/AB36)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30">
       <c r="A38" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30">
       <c r="B39" t="s">
         <v>28</v>
       </c>
       <c r="C39" s="3">
         <f>C41+C42+C43+C44+C45</f>
-        <v>509.8785426179017</v>
+        <v>0</v>
       </c>
       <c r="D39" s="3">
         <f>D41+D42+D43+D44+D45</f>
-        <v>509.8785426179017</v>
+        <v>0</v>
       </c>
       <c r="E39" s="3">
         <f>E41+E42+E43+E44+E45</f>
@@ -3203,27 +3177,27 @@
       </c>
       <c r="F39" s="3">
         <f>F41+F42+F43+F44+F45</f>
-        <v>660.80113298361266</v>
+        <v>0</v>
       </c>
       <c r="G39" s="3">
         <f>G41+G42+G43+G44+G45</f>
-        <v>480.83763185909783</v>
+        <v>0</v>
       </c>
       <c r="H39" s="4">
         <f>IF(F39=0,0,G39/F39)</f>
-        <v>0.72765860689137496</v>
+        <v>0</v>
       </c>
       <c r="I39" s="3">
         <f>I41+I42+I43+I44+I45</f>
-        <v>814.53034621778045</v>
+        <v>0</v>
       </c>
       <c r="J39" s="6">
         <f>J41+J42+J43+J44+J45</f>
-        <v>29.040910758803861</v>
+        <v>0</v>
       </c>
       <c r="K39" s="7">
         <f>IF(I39=0,0,J39/I39)</f>
-        <v>3.5653565141745142E-2</v>
+        <v>0</v>
       </c>
       <c r="L39" s="3">
         <f>L41+L42+L43+L44+L45</f>
@@ -3251,27 +3225,27 @@
       </c>
       <c r="S39" s="3">
         <f>S41+S42+S43+S44+S45</f>
-        <v>7345.6595414292105</v>
+        <v>0</v>
       </c>
       <c r="T39" s="3">
         <f>T41+T42+T43+T44+T45</f>
-        <v>5345.1323886147175</v>
+        <v>0</v>
       </c>
       <c r="U39" s="4">
         <f>IF(S39=0,0,T39/S39)</f>
-        <v>0.72765860689137518</v>
+        <v>0</v>
       </c>
       <c r="V39" s="3">
         <f>V41+V42+V43+V44+V45</f>
-        <v>26890169.836246081</v>
+        <v>0</v>
       </c>
       <c r="W39" s="6">
         <f>W41+W42+W43+W44+W45</f>
-        <v>1105374.7651894097</v>
+        <v>0</v>
       </c>
       <c r="X39" s="7">
         <f>IF(V39=0,0,W39/V39)</f>
-        <v>4.1107020592314795E-2</v>
+        <v>0</v>
       </c>
       <c r="Y39" s="3">
         <f>Y41+Y42+Y43+Y44+Y45</f>
@@ -3298,46 +3272,46 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30">
       <c r="A40" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30">
       <c r="B41" t="s">
         <v>30</v>
       </c>
       <c r="C41" s="3">
         <f>J41+M41+G41+P41</f>
-        <v>138.65122217384757</v>
+        <v>0</v>
       </c>
       <c r="D41" s="3">
         <f>G41+J41</f>
-        <v>138.65122217384757</v>
+        <v>0</v>
       </c>
       <c r="E41" s="3">
         <f>M41+P41</f>
         <v>0</v>
       </c>
       <c r="F41" s="3">
-        <v>158.01636350616181</v>
+        <v>158.0163635061618</v>
       </c>
       <c r="G41" s="3">
-        <v>128.62683418279411</v>
+        <v>73.07670608966366</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
-        <v>0.81400958311370286</v>
+        <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>289.90090139463632</v>
+        <v>289.9009013946363</v>
       </c>
       <c r="J41" s="6">
-        <v>10.024387991053461</v>
+        <v>2.468307550160215</v>
       </c>
       <c r="K41" s="7">
         <f>IF(I41=0,0,J41/I41)</f>
-        <v>3.4578671341926812E-2</v>
+        <v>0</v>
       </c>
       <c r="L41" s="3">
         <v>0</v>
@@ -3360,24 +3334,24 @@
         <v>0</v>
       </c>
       <c r="S41" s="3">
-        <v>1756.5563228532919</v>
+        <v>1756.556322853292</v>
       </c>
       <c r="T41" s="3">
-        <v>1429.8536800815471</v>
+        <v>812.3421352503464</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
-        <v>0.81400958311370286</v>
+        <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>7917202.4300766056</v>
+        <v>7917202.430076606</v>
       </c>
       <c r="W41" s="6">
-        <v>303590.13104824722</v>
+        <v>72642.66277817823</v>
       </c>
       <c r="X41" s="7">
         <f>IF(V41=0,0,W41/V41)</f>
-        <v>3.8345632024632939E-2</v>
+        <v>0</v>
       </c>
       <c r="Y41" s="3">
         <v>0</v>
@@ -3400,41 +3374,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30">
       <c r="B42" t="s">
         <v>31</v>
       </c>
       <c r="C42" s="3">
         <f>J42+M42+G42+P42</f>
-        <v>126.52920136922393</v>
+        <v>0</v>
       </c>
       <c r="D42" s="3">
         <f>G42+J42</f>
-        <v>126.52920136922393</v>
+        <v>0</v>
       </c>
       <c r="E42" s="3">
         <f>M42+P42</f>
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>150.30970532381971</v>
+        <v>150.3097053238197</v>
       </c>
       <c r="G42" s="3">
-        <v>119.80575138365791</v>
+        <v>73.84732358370334</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
-        <v>0.79705931912749339</v>
+        <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>172.51020331953049</v>
+        <v>172.5102033195305</v>
       </c>
       <c r="J42" s="6">
-        <v>6.7234499855660248</v>
+        <v>1.675697128445114</v>
       </c>
       <c r="K42" s="7">
         <f>IF(I42=0,0,J42/I42)</f>
-        <v>3.8974216343091166E-2</v>
+        <v>0</v>
       </c>
       <c r="L42" s="3">
         <v>0</v>
@@ -3457,24 +3431,24 @@
         <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>1670.8868462377629</v>
+        <v>1670.886846237763</v>
       </c>
       <c r="T42" s="3">
-        <v>1331.795932001357</v>
+        <v>820.908545725955</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
-        <v>0.79705931912749395</v>
+        <v>0</v>
       </c>
       <c r="V42" s="3">
         <v>5775458.9344058</v>
       </c>
       <c r="W42" s="6">
-        <v>266981.41794837551</v>
+        <v>65017.80318323709</v>
       </c>
       <c r="X42" s="7">
         <f>IF(V42=0,0,W42/V42)</f>
-        <v>4.6226874951513015E-2</v>
+        <v>0</v>
       </c>
       <c r="Y42" s="3">
         <v>0</v>
@@ -3497,17 +3471,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30">
       <c r="B43" t="s">
         <v>32</v>
       </c>
       <c r="C43" s="3">
         <f>J43+M43+G43+P43</f>
-        <v>119.70614589422573</v>
+        <v>0</v>
       </c>
       <c r="D43" s="3">
         <f>G43+J43</f>
-        <v>119.70614589422573</v>
+        <v>0</v>
       </c>
       <c r="E43" s="3">
         <f>M43+P43</f>
@@ -3517,21 +3491,21 @@
         <v>136.8081181206467</v>
       </c>
       <c r="G43" s="3">
-        <v>112.71169114408799</v>
+        <v>73.91268637921716</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
-        <v>0.82386698020866833</v>
+        <v>0</v>
       </c>
       <c r="I43" s="3">
-        <v>135.45605543604131</v>
+        <v>135.4560554360413</v>
       </c>
       <c r="J43" s="6">
-        <v>6.9944547501377379</v>
+        <v>1.768331189597433</v>
       </c>
       <c r="K43" s="7">
         <f>IF(I43=0,0,J43/I43)</f>
-        <v>5.1636338645933262E-2</v>
+        <v>0</v>
       </c>
       <c r="L43" s="3">
         <v>0</v>
@@ -3554,24 +3528,24 @@
         <v>0</v>
       </c>
       <c r="S43" s="3">
-        <v>1520.7992360431149</v>
+        <v>1520.799236043115</v>
       </c>
       <c r="T43" s="3">
-        <v>1252.9362741024911</v>
+        <v>821.6351377648527</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
-        <v>0.82386698020866844</v>
+        <v>0</v>
       </c>
       <c r="V43" s="3">
-        <v>4941006.3189266957</v>
+        <v>4941006.318926696</v>
       </c>
       <c r="W43" s="6">
-        <v>292834.59484026668</v>
+        <v>72259.68524401821</v>
       </c>
       <c r="X43" s="7">
         <f>IF(V43=0,0,W43/V43)</f>
-        <v>5.9266185051930341E-2</v>
+        <v>0</v>
       </c>
       <c r="Y43" s="3">
         <v>0</v>
@@ -3594,41 +3568,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30">
       <c r="B44" t="s">
         <v>33</v>
       </c>
       <c r="C44" s="3">
         <f>J44+M44+G44+P44</f>
-        <v>74.321153627583328</v>
+        <v>0</v>
       </c>
       <c r="D44" s="3">
         <f>G44+J44</f>
-        <v>74.321153627583328</v>
+        <v>0</v>
       </c>
       <c r="E44" s="3">
         <f>M44+P44</f>
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>120.55842024780129</v>
+        <v>120.5584202478013</v>
       </c>
       <c r="G44" s="3">
-        <v>71.388793624683842</v>
+        <v>33.53727064413405</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
-        <v>0.59215103746339781</v>
+        <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>131.31388542968341</v>
+        <v>131.3138854296834</v>
       </c>
       <c r="J44" s="6">
-        <v>2.9323600028994838</v>
+        <v>0.7001932129434426</v>
       </c>
       <c r="K44" s="7">
         <f>IF(I44=0,0,J44/I44)</f>
-        <v>2.2330921008880802E-2</v>
+        <v>0</v>
       </c>
       <c r="L44" s="3">
         <v>0</v>
@@ -3651,24 +3625,24 @@
         <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>1340.1628202336269</v>
+        <v>1340.162820233627</v>
       </c>
       <c r="T44" s="3">
-        <v>793.57880437121526</v>
+        <v>372.8101539237017</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
-        <v>0.59215103746339781</v>
+        <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>4714339.9302510964</v>
+        <v>4714339.930251096</v>
       </c>
       <c r="W44" s="6">
-        <v>129073.88777256011</v>
+        <v>30505.50398644246</v>
       </c>
       <c r="X44" s="7">
         <f>IF(V44=0,0,W44/V44)</f>
-        <v>2.7378994659319218E-2</v>
+        <v>0</v>
       </c>
       <c r="Y44" s="3">
         <v>0</v>
@@ -3691,17 +3665,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30">
       <c r="B45" t="s">
         <v>34</v>
       </c>
       <c r="C45" s="3">
         <f>J45+M45+G45+P45</f>
-        <v>50.670819553021161</v>
+        <v>0</v>
       </c>
       <c r="D45" s="3">
         <f>G45+J45</f>
-        <v>50.670819553021161</v>
+        <v>0</v>
       </c>
       <c r="E45" s="3">
         <f>M45+P45</f>
@@ -3711,21 +3685,21 @@
         <v>95.10852578518319</v>
       </c>
       <c r="G45" s="3">
-        <v>48.304561523874007</v>
+        <v>19.22102452952165</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
-        <v>0.50788886827009672</v>
+        <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>85.349300637888987</v>
+        <v>85.34930063788899</v>
       </c>
       <c r="J45" s="6">
-        <v>2.3662580291471529</v>
+        <v>0.5616501875193062</v>
       </c>
       <c r="K45" s="7">
         <f>IF(I45=0,0,J45/I45)</f>
-        <v>2.7724398576931087E-2</v>
+        <v>0</v>
       </c>
       <c r="L45" s="3">
         <v>0</v>
@@ -3748,24 +3722,24 @@
         <v>0</v>
       </c>
       <c r="S45" s="3">
-        <v>1057.2543160614141</v>
+        <v>1057.254316061414</v>
       </c>
       <c r="T45" s="3">
-        <v>536.96769805810709</v>
+        <v>213.6665559180072</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
-        <v>0.50788886827009705</v>
+        <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>3542162.2225858839</v>
+        <v>3542162.222585884</v>
       </c>
       <c r="W45" s="6">
-        <v>112894.7335799602</v>
+        <v>26595.64490665263</v>
       </c>
       <c r="X45" s="7">
         <f>IF(V45=0,0,W45/V45)</f>
-        <v>3.1871700528030497E-2</v>
+        <v>0</v>
       </c>
       <c r="Y45" s="3">
         <v>0</v>
@@ -3785,6 +3759,614 @@
       </c>
       <c r="AD45" s="4">
         <f>IF(AB45=0,0,AC45/AB45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:30">
+      <c r="A47" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:30">
+      <c r="B48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" s="3">
+        <f>C50+C51+C52+C53+C54</f>
+        <v>0</v>
+      </c>
+      <c r="D48" s="3">
+        <f>D50+D51+D52+D53+D54</f>
+        <v>0</v>
+      </c>
+      <c r="E48" s="3">
+        <f>E50+E51+E52+E53+E54</f>
+        <v>0</v>
+      </c>
+      <c r="F48" s="3">
+        <f>F50+F51+F52+F53+F54</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="3">
+        <f>G50+G51+G52+G53+G54</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="4">
+        <f>IF(F48=0,0,G48/F48)</f>
+        <v>0</v>
+      </c>
+      <c r="I48" s="3">
+        <f>I50+I51+I52+I53+I54</f>
+        <v>0</v>
+      </c>
+      <c r="J48" s="6">
+        <f>J50+J51+J52+J53+J54</f>
+        <v>0</v>
+      </c>
+      <c r="K48" s="7">
+        <f>IF(I48=0,0,J48/I48)</f>
+        <v>0</v>
+      </c>
+      <c r="L48" s="3">
+        <f>L50+L51+L52+L53+L54</f>
+        <v>0</v>
+      </c>
+      <c r="M48" s="3">
+        <f>M50+M51+M52+M53+M54</f>
+        <v>0</v>
+      </c>
+      <c r="N48" s="4">
+        <f>IF(L48=0,0,M48/L48)</f>
+        <v>0</v>
+      </c>
+      <c r="O48" s="3">
+        <f>O50+O51+O52+O53+O54</f>
+        <v>0</v>
+      </c>
+      <c r="P48" s="3">
+        <f>P50+P51+P52+P53+P54</f>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="4">
+        <f>IF(O48=0,0,P48/O48)</f>
+        <v>0</v>
+      </c>
+      <c r="S48" s="3">
+        <f>S50+S51+S52+S53+S54</f>
+        <v>0</v>
+      </c>
+      <c r="T48" s="3">
+        <f>T50+T51+T52+T53+T54</f>
+        <v>0</v>
+      </c>
+      <c r="U48" s="4">
+        <f>IF(S48=0,0,T48/S48)</f>
+        <v>0</v>
+      </c>
+      <c r="V48" s="3">
+        <f>V50+V51+V52+V53+V54</f>
+        <v>0</v>
+      </c>
+      <c r="W48" s="6">
+        <f>W50+W51+W52+W53+W54</f>
+        <v>0</v>
+      </c>
+      <c r="X48" s="7">
+        <f>IF(V48=0,0,W48/V48)</f>
+        <v>0</v>
+      </c>
+      <c r="Y48" s="3">
+        <f>Y50+Y51+Y52+Y53+Y54</f>
+        <v>0</v>
+      </c>
+      <c r="Z48" s="3">
+        <f>Z50+Z51+Z52+Z53+Z54</f>
+        <v>0</v>
+      </c>
+      <c r="AA48" s="4">
+        <f>IF(Y48=0,0,Z48/Y48)</f>
+        <v>0</v>
+      </c>
+      <c r="AB48" s="3">
+        <f>AB50+AB51+AB52+AB53+AB54</f>
+        <v>0</v>
+      </c>
+      <c r="AC48" s="3">
+        <f>AC50+AC51+AC52+AC53+AC54</f>
+        <v>0</v>
+      </c>
+      <c r="AD48" s="4">
+        <f>IF(AB48=0,0,AC48/AB48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:30">
+      <c r="A49" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="50" spans="1:30">
+      <c r="B50" t="s">
+        <v>30</v>
+      </c>
+      <c r="C50" s="3">
+        <f>J50+M50+G50+P50</f>
+        <v>0</v>
+      </c>
+      <c r="D50" s="3">
+        <f>G50+J50</f>
+        <v>0</v>
+      </c>
+      <c r="E50" s="3">
+        <f>M50+P50</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="3">
+        <v>158.0163635061618</v>
+      </c>
+      <c r="G50" s="3">
+        <v>129.998056574341</v>
+      </c>
+      <c r="H50" s="4">
+        <f>IF(F50=0,0,G50/F50)</f>
+        <v>0</v>
+      </c>
+      <c r="I50" s="3">
+        <v>289.9009013946363</v>
+      </c>
+      <c r="J50" s="6">
+        <v>9.20320339849731</v>
+      </c>
+      <c r="K50" s="7">
+        <f>IF(I50=0,0,J50/I50)</f>
+        <v>0</v>
+      </c>
+      <c r="L50" s="3">
+        <v>0</v>
+      </c>
+      <c r="M50" s="3">
+        <v>0</v>
+      </c>
+      <c r="N50" s="4">
+        <f>IF(L50=0,0,M50/L50)</f>
+        <v>0</v>
+      </c>
+      <c r="O50" s="3">
+        <v>0</v>
+      </c>
+      <c r="P50" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="4">
+        <f>IF(O50=0,0,P50/O50)</f>
+        <v>0</v>
+      </c>
+      <c r="S50" s="3">
+        <v>1756.556322853292</v>
+      </c>
+      <c r="T50" s="3">
+        <v>1445.096591059028</v>
+      </c>
+      <c r="U50" s="4">
+        <f>IF(S50=0,0,T50/S50)</f>
+        <v>0</v>
+      </c>
+      <c r="V50" s="3">
+        <v>7917202.430076606</v>
+      </c>
+      <c r="W50" s="6">
+        <v>278133.0844278978</v>
+      </c>
+      <c r="X50" s="7">
+        <f>IF(V50=0,0,W50/V50)</f>
+        <v>0</v>
+      </c>
+      <c r="Y50" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z50" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA50" s="4">
+        <f>IF(Y50=0,0,Z50/Y50)</f>
+        <v>0</v>
+      </c>
+      <c r="AB50" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC50" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD50" s="4">
+        <f>IF(AB50=0,0,AC50/AB50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:30">
+      <c r="B51" t="s">
+        <v>31</v>
+      </c>
+      <c r="C51" s="3">
+        <f>J51+M51+G51+P51</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="3">
+        <f>G51+J51</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="3">
+        <f>M51+P51</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="3">
+        <v>150.3097053238197</v>
+      </c>
+      <c r="G51" s="3">
+        <v>126.503663964271</v>
+      </c>
+      <c r="H51" s="4">
+        <f>IF(F51=0,0,G51/F51)</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="3">
+        <v>172.5102033195305</v>
+      </c>
+      <c r="J51" s="6">
+        <v>6.178369900404912</v>
+      </c>
+      <c r="K51" s="7">
+        <f>IF(I51=0,0,J51/I51)</f>
+        <v>0</v>
+      </c>
+      <c r="L51" s="3">
+        <v>0</v>
+      </c>
+      <c r="M51" s="3">
+        <v>0</v>
+      </c>
+      <c r="N51" s="4">
+        <f>IF(L51=0,0,M51/L51)</f>
+        <v>0</v>
+      </c>
+      <c r="O51" s="3">
+        <v>0</v>
+      </c>
+      <c r="P51" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="4">
+        <f>IF(O51=0,0,P51/O51)</f>
+        <v>0</v>
+      </c>
+      <c r="S51" s="3">
+        <v>1670.886846237763</v>
+      </c>
+      <c r="T51" s="3">
+        <v>1406.251896132791</v>
+      </c>
+      <c r="U51" s="4">
+        <f>IF(S51=0,0,T51/S51)</f>
+        <v>0</v>
+      </c>
+      <c r="V51" s="3">
+        <v>5775458.9344058</v>
+      </c>
+      <c r="W51" s="6">
+        <v>244923.1724868985</v>
+      </c>
+      <c r="X51" s="7">
+        <f>IF(V51=0,0,W51/V51)</f>
+        <v>0</v>
+      </c>
+      <c r="Y51" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="4">
+        <f>IF(Y51=0,0,Z51/Y51)</f>
+        <v>0</v>
+      </c>
+      <c r="AB51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD51" s="4">
+        <f>IF(AB51=0,0,AC51/AB51)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:30">
+      <c r="B52" t="s">
+        <v>32</v>
+      </c>
+      <c r="C52" s="3">
+        <f>J52+M52+G52+P52</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="3">
+        <f>G52+J52</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="3">
+        <f>M52+P52</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="3">
+        <v>136.8081181206467</v>
+      </c>
+      <c r="G52" s="3">
+        <v>119.0323549228301</v>
+      </c>
+      <c r="H52" s="4">
+        <f>IF(F52=0,0,G52/F52)</f>
+        <v>0</v>
+      </c>
+      <c r="I52" s="3">
+        <v>135.4560554360413</v>
+      </c>
+      <c r="J52" s="6">
+        <v>6.434434707193577</v>
+      </c>
+      <c r="K52" s="7">
+        <f>IF(I52=0,0,J52/I52)</f>
+        <v>0</v>
+      </c>
+      <c r="L52" s="3">
+        <v>0</v>
+      </c>
+      <c r="M52" s="3">
+        <v>0</v>
+      </c>
+      <c r="N52" s="4">
+        <f>IF(L52=0,0,M52/L52)</f>
+        <v>0</v>
+      </c>
+      <c r="O52" s="3">
+        <v>0</v>
+      </c>
+      <c r="P52" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="4">
+        <f>IF(O52=0,0,P52/O52)</f>
+        <v>0</v>
+      </c>
+      <c r="S52" s="3">
+        <v>1520.799236043115</v>
+      </c>
+      <c r="T52" s="3">
+        <v>1323.198629714454</v>
+      </c>
+      <c r="U52" s="4">
+        <f>IF(S52=0,0,T52/S52)</f>
+        <v>0</v>
+      </c>
+      <c r="V52" s="3">
+        <v>4941006.318926696</v>
+      </c>
+      <c r="W52" s="6">
+        <v>268918.3009289764</v>
+      </c>
+      <c r="X52" s="7">
+        <f>IF(V52=0,0,W52/V52)</f>
+        <v>0</v>
+      </c>
+      <c r="Y52" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="4">
+        <f>IF(Y52=0,0,Z52/Y52)</f>
+        <v>0</v>
+      </c>
+      <c r="AB52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD52" s="4">
+        <f>IF(AB52=0,0,AC52/AB52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:30">
+      <c r="B53" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" s="3">
+        <f>J53+M53+G53+P53</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="3">
+        <f>G53+J53</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="3">
+        <f>M53+P53</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="3">
+        <v>120.5584202478013</v>
+      </c>
+      <c r="G53" s="3">
+        <v>78.15395060100447</v>
+      </c>
+      <c r="H53" s="4">
+        <f>IF(F53=0,0,G53/F53)</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="3">
+        <v>131.3138854296834</v>
+      </c>
+      <c r="J53" s="6">
+        <v>2.685703846483724</v>
+      </c>
+      <c r="K53" s="7">
+        <f>IF(I53=0,0,J53/I53)</f>
+        <v>0</v>
+      </c>
+      <c r="L53" s="3">
+        <v>0</v>
+      </c>
+      <c r="M53" s="3">
+        <v>0</v>
+      </c>
+      <c r="N53" s="4">
+        <f>IF(L53=0,0,M53/L53)</f>
+        <v>0</v>
+      </c>
+      <c r="O53" s="3">
+        <v>0</v>
+      </c>
+      <c r="P53" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="4">
+        <f>IF(O53=0,0,P53/O53)</f>
+        <v>0</v>
+      </c>
+      <c r="S53" s="3">
+        <v>1340.162820233627</v>
+      </c>
+      <c r="T53" s="3">
+        <v>868.7822769621262</v>
+      </c>
+      <c r="U53" s="4">
+        <f>IF(S53=0,0,T53/S53)</f>
+        <v>0</v>
+      </c>
+      <c r="V53" s="3">
+        <v>4714339.930251096</v>
+      </c>
+      <c r="W53" s="6">
+        <v>118125.7799676377</v>
+      </c>
+      <c r="X53" s="7">
+        <f>IF(V53=0,0,W53/V53)</f>
+        <v>0</v>
+      </c>
+      <c r="Y53" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="4">
+        <f>IF(Y53=0,0,Z53/Y53)</f>
+        <v>0</v>
+      </c>
+      <c r="AB53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD53" s="4">
+        <f>IF(AB53=0,0,AC53/AB53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:30">
+      <c r="B54" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54" s="3">
+        <f>J54+M54+G54+P54</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="3">
+        <f>G54+J54</f>
+        <v>0</v>
+      </c>
+      <c r="E54" s="3">
+        <f>M54+P54</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="3">
+        <v>95.10852578518319</v>
+      </c>
+      <c r="G54" s="3">
+        <v>51.0082429912127</v>
+      </c>
+      <c r="H54" s="4">
+        <f>IF(F54=0,0,G54/F54)</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="3">
+        <v>85.34930063788899</v>
+      </c>
+      <c r="J54" s="6">
+        <v>2.166210930921327</v>
+      </c>
+      <c r="K54" s="7">
+        <f>IF(I54=0,0,J54/I54)</f>
+        <v>0</v>
+      </c>
+      <c r="L54" s="3">
+        <v>0</v>
+      </c>
+      <c r="M54" s="3">
+        <v>0</v>
+      </c>
+      <c r="N54" s="4">
+        <f>IF(L54=0,0,M54/L54)</f>
+        <v>0</v>
+      </c>
+      <c r="O54" s="3">
+        <v>0</v>
+      </c>
+      <c r="P54" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="4">
+        <f>IF(O54=0,0,P54/O54)</f>
+        <v>0</v>
+      </c>
+      <c r="S54" s="3">
+        <v>1057.254316061414</v>
+      </c>
+      <c r="T54" s="3">
+        <v>567.0226156062497</v>
+      </c>
+      <c r="U54" s="4">
+        <f>IF(S54=0,0,T54/S54)</f>
+        <v>0</v>
+      </c>
+      <c r="V54" s="3">
+        <v>3542162.222585884</v>
+      </c>
+      <c r="W54" s="6">
+        <v>103292.0565680326</v>
+      </c>
+      <c r="X54" s="7">
+        <f>IF(V54=0,0,W54/V54)</f>
+        <v>0</v>
+      </c>
+      <c r="Y54" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA54" s="4">
+        <f>IF(Y54=0,0,Z54/Y54)</f>
+        <v>0</v>
+      </c>
+      <c r="AB54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD54" s="4">
+        <f>IF(AB54=0,0,AC54/AB54)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use baseline effectiveness for baseline calibration
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\src\vivarium_gates_lsff_by_wealth_quintile\5000_analyze_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE965AA-1BBB-40DA-B9E8-7171382D249F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A28911-9E96-42C2-BCCF-169F1DB65925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1470,11 +1470,11 @@
       </c>
       <c r="AC12" s="3">
         <f>AC14+AC15+AC16+AC17+AC18</f>
-        <v>1680.7280119055358</v>
+        <v>1680.7280119055067</v>
       </c>
       <c r="AD12" s="4">
         <f>IF(AB12=0,0,AC12/AB12)</f>
-        <v>2.0606171206107712E-3</v>
+        <v>2.0606171206107356E-3</v>
       </c>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.25">
@@ -1669,11 +1669,11 @@
         <v>171868.3936012006</v>
       </c>
       <c r="AC15" s="3">
-        <v>384.52079977176618</v>
+        <v>384.52079977173707</v>
       </c>
       <c r="AD15" s="4">
         <f>IF(AB15=0,0,AC15/AB15)</f>
-        <v>2.2372979214782167E-3</v>
+        <v>2.2372979214780476E-3</v>
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.25">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C21" s="3">
         <f>C23+C24+C25+C26+C27</f>
-        <v>1975.7745733977658</v>
+        <v>2111.7120178026412</v>
       </c>
       <c r="D21" s="3">
         <f>D23+D24+D25+D26+D27</f>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="E21" s="3">
         <f>E23+E24+E25+E26+E27</f>
-        <v>900.67179130957709</v>
+        <v>1036.6092357144523</v>
       </c>
       <c r="F21" s="3">
         <f>F23+F24+F25+F26+F27</f>
@@ -2006,11 +2006,11 @@
       </c>
       <c r="J21" s="3">
         <f>J23+J24+J25+J26+J27</f>
-        <v>664.88986387520163</v>
+        <v>686.2475247770335</v>
       </c>
       <c r="K21" s="4">
         <f>IF(I21=0,0,J21/I21)</f>
-        <v>0.18055711094007593</v>
+        <v>0.18635698511231386</v>
       </c>
       <c r="L21" s="3">
         <f>L23+L24+L25+L26+L27</f>
@@ -2018,11 +2018,11 @@
       </c>
       <c r="M21" s="3">
         <f>M23+M24+M25+M26+M27</f>
-        <v>209.09178119225427</v>
+        <v>270.09622799380867</v>
       </c>
       <c r="N21" s="4">
         <f>IF(L21=0,0,M21/L21)</f>
-        <v>2.7834329835964744E-3</v>
+        <v>3.5955251108206179E-3</v>
       </c>
       <c r="O21" s="3">
         <f>O23+O24+O25+O26+O27</f>
@@ -2030,11 +2030,11 @@
       </c>
       <c r="P21" s="3">
         <f>P23+P24+P25+P26+P27</f>
-        <v>26.690146242121234</v>
+        <v>80.265482943610337</v>
       </c>
       <c r="Q21" s="4">
         <f>IF(O21=0,0,P21/O21)</f>
-        <v>1.3784995353799867E-2</v>
+        <v>4.1455723000198653E-2</v>
       </c>
       <c r="S21" s="3">
         <f>S23+S24+S25+S26+S27</f>
@@ -2054,11 +2054,11 @@
       </c>
       <c r="W21" s="3">
         <f>W23+W24+W25+W26+W27</f>
-        <v>16036047.728803257</v>
+        <v>16489023.35117919</v>
       </c>
       <c r="X21" s="4">
         <f>IF(V21=0,0,W21/V21)</f>
-        <v>0.15033293255243116</v>
+        <v>0.15457943735449806</v>
       </c>
       <c r="Y21" s="3">
         <f>Y23+Y24+Y25+Y26+Y27</f>
@@ -2066,11 +2066,11 @@
       </c>
       <c r="Z21" s="3">
         <f>Z23+Z24+Z25+Z26+Z27</f>
-        <v>103232.61702703497</v>
+        <v>334084.07649866142</v>
       </c>
       <c r="AA21" s="4">
         <f>IF(Y21=0,0,Z21/Y21)</f>
-        <v>1.2773146250877771E-2</v>
+        <v>4.1336787655875284E-2</v>
       </c>
       <c r="AB21" s="3">
         <f>AB23+AB24+AB25+AB26+AB27</f>
@@ -2078,11 +2078,11 @@
       </c>
       <c r="AC21" s="3">
         <f>AC23+AC24+AC25+AC26+AC27</f>
-        <v>2321.625865432783</v>
+        <v>2999.0317686344206</v>
       </c>
       <c r="AD21" s="4">
         <f>IF(AB21=0,0,AC21/AB21)</f>
-        <v>2.7492772162753154E-3</v>
+        <v>3.5514635821200509E-3</v>
       </c>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.25">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="C23" s="3">
         <f>J23+M23+G23+P23</f>
-        <v>518.61713209248273</v>
+        <v>550.58183910185278</v>
       </c>
       <c r="D23" s="3">
         <f>G23</f>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="E23" s="3">
         <f>J23+M23+P23</f>
-        <v>241.1356892968835</v>
+        <v>273.10039630625363</v>
       </c>
       <c r="F23" s="3">
         <v>428.09244082133358</v>
@@ -2120,31 +2120,31 @@
         <v>991.82050542122556</v>
       </c>
       <c r="J23" s="3">
-        <v>158.0066388873833</v>
+        <v>162.60977052226261</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
-        <v>0.15930971181149151</v>
+        <v>0.16395080524494937</v>
       </c>
       <c r="L23" s="3">
         <v>18248.150900694091</v>
       </c>
       <c r="M23" s="3">
-        <v>74.961120675049727</v>
+        <v>92.706822166558354</v>
       </c>
       <c r="N23" s="4">
         <f>IF(L23=0,0,M23/L23)</f>
-        <v>4.1078748791034212E-3</v>
+        <v>5.0803406148418103E-3</v>
       </c>
       <c r="O23" s="3">
         <v>476.04818802351332</v>
       </c>
       <c r="P23" s="3">
-        <v>8.1679297344504747</v>
+        <v>17.78380361743271</v>
       </c>
       <c r="Q23" s="4">
         <f>IF(O23=0,0,P23/O23)</f>
-        <v>1.7157779275166651E-2</v>
+        <v>3.7357150105472768E-2</v>
       </c>
       <c r="S23" s="3">
         <v>4758.8013481976486</v>
@@ -2160,31 +2160,31 @@
         <v>25699987.560610589</v>
       </c>
       <c r="W23" s="3">
-        <v>3216996.2172383629</v>
+        <v>3313562.2441319791</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
-        <v>0.12517501067467179</v>
+        <v>0.12893244544641541</v>
       </c>
       <c r="Y23" s="3">
         <v>1959206.3612258229</v>
       </c>
       <c r="Z23" s="3">
-        <v>32813.334540281438</v>
+        <v>81685.476824872196</v>
       </c>
       <c r="AA23" s="4">
         <f>IF(Y23=0,0,Z23/Y23)</f>
-        <v>1.6748278889698487E-2</v>
+        <v>4.1693145980683619E-2</v>
       </c>
       <c r="AB23" s="3">
         <v>205054.68928072241</v>
       </c>
       <c r="AC23" s="3">
-        <v>832.18096089712344</v>
+        <v>1029.3601439886841</v>
       </c>
       <c r="AD23" s="4">
         <f>IF(AB23=0,0,AC23/AB23)</f>
-        <v>4.0583366506574126E-3</v>
+        <v>5.0199297933610151E-3</v>
       </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.25">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="C24" s="3">
         <f>J24+M24+G24+P24</f>
-        <v>489.435021452032</v>
+        <v>524.38521669671627</v>
       </c>
       <c r="D24" s="3">
         <f>G24</f>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E24" s="3">
         <f>J24+M24+P24</f>
-        <v>215.66451978391521</v>
+        <v>250.61471502859939</v>
       </c>
       <c r="F24" s="3">
         <v>437.75116549754102</v>
@@ -2217,31 +2217,31 @@
         <v>847.52939170447485</v>
       </c>
       <c r="J24" s="3">
-        <v>146.2972280304503</v>
+        <v>151.9237102732427</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
-        <v>0.17261611156190168</v>
+        <v>0.17925479842971276</v>
       </c>
       <c r="L24" s="3">
         <v>18442.648959675</v>
       </c>
       <c r="M24" s="3">
-        <v>61.83910950501263</v>
+        <v>78.360818720057608</v>
       </c>
       <c r="N24" s="4">
         <f>IF(L24=0,0,M24/L24)</f>
-        <v>3.3530492089408814E-3</v>
+        <v>4.2488917341209588E-3</v>
       </c>
       <c r="O24" s="3">
         <v>476.56393826290048</v>
       </c>
       <c r="P24" s="3">
-        <v>7.5281822484522696</v>
+        <v>20.330186035299089</v>
       </c>
       <c r="Q24" s="4">
         <f>IF(O24=0,0,P24/O24)</f>
-        <v>1.5796793764741981E-2</v>
+        <v>4.2659933752863553E-2</v>
       </c>
       <c r="S24" s="3">
         <v>4866.1705694873763</v>
@@ -2257,31 +2257,31 @@
         <v>23322467.600951109</v>
       </c>
       <c r="W24" s="3">
-        <v>3280613.24423252</v>
+        <v>3386920.8556735781</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
-        <v>0.14066321370294171</v>
+        <v>0.14522137681243716</v>
       </c>
       <c r="Y24" s="3">
         <v>2033978.1299748039</v>
       </c>
       <c r="Z24" s="3">
-        <v>28335.70369254192</v>
+        <v>83922.171154072974</v>
       </c>
       <c r="AA24" s="4">
         <f>IF(Y24=0,0,Z24/Y24)</f>
-        <v>1.3931174222061537E-2</v>
+        <v>4.1260114805222889E-2</v>
       </c>
       <c r="AB24" s="3">
         <v>207305.28823611679</v>
       </c>
       <c r="AC24" s="3">
-        <v>686.94683141575661</v>
+        <v>870.34467375359964</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(AB24=0,0,AC24/AB24)</f>
-        <v>3.3136966126659402E-3</v>
+        <v>4.1983717885782706E-3</v>
       </c>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.25">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C25" s="3">
         <f>J25+M25+G25+P25</f>
-        <v>387.91812187613897</v>
+        <v>417.64037577601232</v>
       </c>
       <c r="D25" s="3">
         <f>G25</f>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="E25" s="3">
         <f>J25+M25+P25</f>
-        <v>173.63376429454109</v>
+        <v>203.35601819441447</v>
       </c>
       <c r="F25" s="3">
         <v>396.28526128416758</v>
@@ -2314,31 +2314,31 @@
         <v>721.62080381298233</v>
       </c>
       <c r="J25" s="3">
-        <v>133.25111545387341</v>
+        <v>137.9599041540084</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
-        <v>0.18465531308103364</v>
+        <v>0.19118060818790161</v>
       </c>
       <c r="L25" s="3">
         <v>15355.961975565249</v>
       </c>
       <c r="M25" s="3">
-        <v>35.528234945729373</v>
+        <v>48.616281052693722</v>
       </c>
       <c r="N25" s="4">
         <f>IF(L25=0,0,M25/L25)</f>
-        <v>2.3136443683738407E-3</v>
+        <v>3.1659547692325001E-3</v>
       </c>
       <c r="O25" s="3">
         <v>391.5266582641886</v>
       </c>
       <c r="P25" s="3">
-        <v>4.8544138949383049</v>
+        <v>16.77983298771235</v>
       </c>
       <c r="Q25" s="4">
         <f>IF(O25=0,0,P25/O25)</f>
-        <v>1.2398680377116786E-2</v>
+        <v>4.2857446954199227E-2</v>
       </c>
       <c r="S25" s="3">
         <v>4405.2233953297473</v>
@@ -2354,31 +2354,31 @@
         <v>21162807.846375171</v>
       </c>
       <c r="W25" s="3">
-        <v>3244311.4196785842</v>
+        <v>3343728.0163370739</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
-        <v>0.1533025032986953</v>
+        <v>0.15800020680666899</v>
       </c>
       <c r="Y25" s="3">
         <v>1664123.912966297</v>
       </c>
       <c r="Z25" s="3">
-        <v>19414.379511777312</v>
+        <v>70162.630031719338</v>
       </c>
       <c r="AA25" s="4">
         <f>IF(Y25=0,0,Z25/Y25)</f>
-        <v>1.1666426616736265E-2</v>
+        <v>4.2161902419066026E-2</v>
       </c>
       <c r="AB25" s="3">
         <v>172634.6152091868</v>
       </c>
       <c r="AC25" s="3">
-        <v>394.35836618309258</v>
+        <v>539.59249566448852</v>
       </c>
       <c r="AD25" s="4">
         <f>IF(AB25=0,0,AC25/AB25)</f>
-        <v>2.2843527974110876E-3</v>
+        <v>3.1256332631242425E-3</v>
       </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.25">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C26" s="3">
         <f>J26+M26+G26+P26</f>
-        <v>322.24592078576092</v>
+        <v>344.40259067183274</v>
       </c>
       <c r="D26" s="3">
         <f>G26</f>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="E26" s="3">
         <f>J26+M26+P26</f>
-        <v>153.15505362828097</v>
+        <v>175.31172351435274</v>
       </c>
       <c r="F26" s="3">
         <v>351.26672270713158</v>
@@ -2411,31 +2411,31 @@
         <v>656.23600296293523</v>
       </c>
       <c r="J26" s="3">
-        <v>127.3969180751008</v>
+        <v>130.83245085781229</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
-        <v>0.19413277768957807</v>
+        <v>0.19936798692406063</v>
       </c>
       <c r="L26" s="3">
         <v>12320.893910346331</v>
       </c>
       <c r="M26" s="3">
-        <v>22.14377215228788</v>
+        <v>30.922360504940151</v>
       </c>
       <c r="N26" s="4">
         <f>IF(L26=0,0,M26/L26)</f>
-        <v>1.7972536987509403E-3</v>
+        <v>2.5097497576026888E-3</v>
       </c>
       <c r="O26" s="3">
         <v>305.89771512841492</v>
       </c>
       <c r="P26" s="3">
-        <v>3.6143634008922958</v>
+        <v>13.55691215160029</v>
       </c>
       <c r="Q26" s="4">
         <f>IF(O26=0,0,P26/O26)</f>
-        <v>1.1815594632261301E-2</v>
+        <v>4.4318448556927403E-2</v>
       </c>
       <c r="S26" s="3">
         <v>3904.7840938011818</v>
@@ -2451,31 +2451,31 @@
         <v>20232379.411657181</v>
       </c>
       <c r="W26" s="3">
-        <v>3285780.5653708731</v>
+        <v>3361820.0850684568</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
-        <v>0.16240208324077407</v>
+        <v>0.16616039155194445</v>
       </c>
       <c r="Y26" s="3">
         <v>1291512.2728871789</v>
       </c>
       <c r="Z26" s="3">
-        <v>12960.948979210571</v>
+        <v>51650.776301899918</v>
       </c>
       <c r="AA26" s="4">
         <f>IF(Y26=0,0,Z26/Y26)</f>
-        <v>1.0035482628621358E-2</v>
+        <v>3.9992478109739119E-2</v>
       </c>
       <c r="AB26" s="3">
         <v>138538.51808137319</v>
       </c>
       <c r="AC26" s="3">
-        <v>245.9439272969903</v>
+        <v>343.4734157078783</v>
       </c>
       <c r="AD26" s="4">
         <f>IF(AB26=0,0,AC26/AB26)</f>
-        <v>1.7752747084571131E-3</v>
+        <v>2.479262954914335E-3</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.25">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="C27" s="3">
         <f>J27+M27+G27+P27</f>
-        <v>257.55837719135116</v>
+        <v>274.70199555622702</v>
       </c>
       <c r="D27" s="3">
         <f>G27</f>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="E27" s="3">
         <f>J27+M27+P27</f>
-        <v>117.08276430595636</v>
+        <v>134.22638267083227</v>
       </c>
       <c r="F27" s="3">
         <v>308.52409051931693</v>
@@ -2508,31 +2508,31 @@
         <v>465.22851237667129</v>
       </c>
       <c r="J27" s="3">
-        <v>99.937963428393815</v>
+        <v>102.9216889697075</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
-        <v>0.21481478621731431</v>
+        <v>0.22122824855235265</v>
       </c>
       <c r="L27" s="3">
         <v>10752.450404824391</v>
       </c>
       <c r="M27" s="3">
-        <v>14.61954391417466</v>
+        <v>19.489945549558851</v>
       </c>
       <c r="N27" s="4">
         <f>IF(L27=0,0,M27/L27)</f>
-        <v>1.3596476490247459E-3</v>
+        <v>1.8126050170679359E-3</v>
       </c>
       <c r="O27" s="3">
         <v>286.13725715609343</v>
       </c>
       <c r="P27" s="3">
-        <v>2.5252569633878879</v>
+        <v>11.814748151565899</v>
       </c>
       <c r="Q27" s="4">
         <f>IF(O27=0,0,P27/O27)</f>
-        <v>8.8253343464822238E-3</v>
+        <v>4.12904920840865E-2</v>
       </c>
       <c r="S27" s="3">
         <v>3429.6444363696219</v>
@@ -2548,31 +2548,31 @@
         <v>16252582.504079361</v>
       </c>
       <c r="W27" s="3">
-        <v>3008346.2822829168</v>
+        <v>3082992.149968103</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
-        <v>0.18509958534453394</v>
+        <v>0.18969244728917875</v>
       </c>
       <c r="Y27" s="3">
         <v>1133183.161267315</v>
       </c>
       <c r="Z27" s="3">
-        <v>9708.2503032237291</v>
+        <v>46663.02218609699</v>
       </c>
       <c r="AA27" s="4">
         <f>IF(Y27=0,0,Z27/Y27)</f>
-        <v>8.5672384086314338E-3</v>
+        <v>4.1178711245506497E-2</v>
       </c>
       <c r="AB27" s="3">
         <v>120916.42366991749</v>
       </c>
       <c r="AC27" s="3">
-        <v>162.1957796398201</v>
+        <v>216.26103951976981</v>
       </c>
       <c r="AD27" s="4">
         <f>IF(AB27=0,0,AC27/AB27)</f>
-        <v>1.3413875031781345E-3</v>
+        <v>1.7885166709042592E-3</v>
       </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Change non-pregnant anemia model to an approach based on distributions, add results plots
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\src\vivarium_gates_lsff_by_wealth_quintile\5000_analyze_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A28911-9E96-42C2-BCCF-169F1DB65925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5AD325F-8559-4870-A355-6119A5DEDD2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Model Results" sheetId="1" r:id="rId1"/>
@@ -762,7 +762,7 @@
       </c>
       <c r="C3" s="3">
         <f>C5+C6+C7+C8+C9</f>
-        <v>1550.4769535986134</v>
+        <v>1391.4362330092995</v>
       </c>
       <c r="D3" s="3">
         <f>D5+D6+D7+D8+D9</f>
@@ -770,7 +770,7 @@
       </c>
       <c r="E3" s="3">
         <f>E5+E6+E7+E8+E9</f>
-        <v>1467.1319909602937</v>
+        <v>1308.0912703709794</v>
       </c>
       <c r="F3" s="3">
         <f>F5+F6+F7+F8+F9</f>
@@ -786,15 +786,15 @@
       </c>
       <c r="I3" s="3">
         <f>I5+I6+I7+I8+I9</f>
-        <v>19407.709538433905</v>
+        <v>18088.403478171738</v>
       </c>
       <c r="J3" s="3">
         <f>J5+J6+J7+J8+J9</f>
-        <v>1278.2304393921872</v>
+        <v>1119.1897188028731</v>
       </c>
       <c r="K3" s="4">
         <f>IF(I3=0,0,J3/I3)</f>
-        <v>6.5861993495979196E-2</v>
+        <v>6.1873327856350635E-2</v>
       </c>
       <c r="L3" s="3">
         <f>L5+L6+L7+L8+L9</f>
@@ -834,15 +834,15 @@
       </c>
       <c r="V3" s="3">
         <f>V5+V6+V7+V8+V9</f>
-        <v>619265330.3877759</v>
+        <v>586984476.54622817</v>
       </c>
       <c r="W3" s="3">
         <f>W5+W6+W7+W8+W9</f>
-        <v>32099658.477910429</v>
+        <v>28560841.837795049</v>
       </c>
       <c r="X3" s="4">
         <f>IF(V3=0,0,W3/V3)</f>
-        <v>5.1835064717429026E-2</v>
+        <v>4.8656894652214421E-2</v>
       </c>
       <c r="Y3" s="3">
         <f>Y5+Y6+Y7+Y8+Y9</f>
@@ -880,7 +880,7 @@
       </c>
       <c r="C5" s="3">
         <f>J5+M5+G5+P5</f>
-        <v>453.17794864394864</v>
+        <v>406.30987716553807</v>
       </c>
       <c r="D5" s="3">
         <f>G5</f>
@@ -888,7 +888,7 @@
       </c>
       <c r="E5" s="3">
         <f>J5+M5+P5</f>
-        <v>424.86558384825406</v>
+        <v>377.99751236984349</v>
       </c>
       <c r="F5" s="3">
         <v>397.0902965307904</v>
@@ -901,14 +901,14 @@
         <v>7.1299563457097093E-2</v>
       </c>
       <c r="I5" s="3">
-        <v>4595.3272879255064</v>
+        <v>4229.0317579039856</v>
       </c>
       <c r="J5" s="3">
-        <v>359.70645668022428</v>
+        <v>312.83838520181371</v>
       </c>
       <c r="K5" s="4">
         <f>IF(I5=0,0,J5/I5)</f>
-        <v>7.8276569685335404E-2</v>
+        <v>7.3973997621825438E-2</v>
       </c>
       <c r="L5" s="3">
         <v>18640.875795544409</v>
@@ -941,14 +941,14 @@
         <v>7.1299563457097107E-2</v>
       </c>
       <c r="V5" s="3">
-        <v>139111960.55532151</v>
+        <v>130721936.6657657</v>
       </c>
       <c r="W5" s="3">
-        <v>8453026.7370958477</v>
+        <v>7530151.3682035357</v>
       </c>
       <c r="X5" s="4">
         <f>IF(V5=0,0,W5/V5)</f>
-        <v>6.076419815630648E-2</v>
+        <v>5.7604343695250498E-2</v>
       </c>
       <c r="Y5" s="3">
         <v>6174245.853177595</v>
@@ -977,7 +977,7 @@
       </c>
       <c r="C6" s="3">
         <f>J6+M6+G6+P6</f>
-        <v>380.08640040355482</v>
+        <v>338.69031697899226</v>
       </c>
       <c r="D6" s="3">
         <f>G6</f>
@@ -985,7 +985,7 @@
       </c>
       <c r="E6" s="3">
         <f>J6+M6+P6</f>
-        <v>358.94189218021654</v>
+        <v>317.54580875565398</v>
       </c>
       <c r="F6" s="3">
         <v>346.92132413597358</v>
@@ -998,14 +998,14 @@
         <v>6.0949001264191033E-2</v>
       </c>
       <c r="I6" s="3">
-        <v>4112.5343319715366</v>
+        <v>3787.0627176324879</v>
       </c>
       <c r="J6" s="3">
-        <v>316.53763125915589</v>
+        <v>275.14154783459333</v>
       </c>
       <c r="K6" s="4">
         <f>IF(I6=0,0,J6/I6)</f>
-        <v>7.6968994227802276E-2</v>
+        <v>7.2653021180119307E-2</v>
       </c>
       <c r="L6" s="3">
         <v>15402.279753726511</v>
@@ -1038,14 +1038,14 @@
         <v>6.0949001264191172E-2</v>
       </c>
       <c r="V6" s="3">
-        <v>128962196.4271194</v>
+        <v>121072766.34225529</v>
       </c>
       <c r="W6" s="3">
-        <v>7862063.5119100511</v>
+        <v>6967680.9027350992</v>
       </c>
       <c r="X6" s="4">
         <f>IF(V6=0,0,W6/V6)</f>
-        <v>6.0964094360420967E-2</v>
+        <v>5.7549530858479497E-2</v>
       </c>
       <c r="Y6" s="3">
         <v>5221398.5281040482</v>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C7" s="3">
         <f>J7+M7+G7+P7</f>
-        <v>323.46818905339939</v>
+        <v>289.54899421135423</v>
       </c>
       <c r="D7" s="3">
         <f>G7</f>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E7" s="3">
         <f>J7+M7+P7</f>
-        <v>307.53673618697235</v>
+        <v>273.61754134492719</v>
       </c>
       <c r="F7" s="3">
         <v>308.40246775221379</v>
@@ -1095,14 +1095,14 @@
         <v>5.1657994122236262E-2</v>
       </c>
       <c r="I7" s="3">
-        <v>3977.0165003595712</v>
+        <v>3695.2568384953711</v>
       </c>
       <c r="J7" s="3">
-        <v>272.23966934380729</v>
+        <v>238.32047450176211</v>
       </c>
       <c r="K7" s="4">
         <f>IF(I7=0,0,J7/I7)</f>
-        <v>6.8453241096483625E-2</v>
+        <v>6.44936157127311E-2</v>
       </c>
       <c r="L7" s="3">
         <v>13777.53512556912</v>
@@ -1135,14 +1135,14 @@
         <v>5.1657994122236359E-2</v>
       </c>
       <c r="V7" s="3">
-        <v>125283725.8487372</v>
+        <v>118411700.21523701</v>
       </c>
       <c r="W7" s="3">
-        <v>6822051.0377212912</v>
+        <v>6061904.1303865612</v>
       </c>
       <c r="X7" s="4">
         <f>IF(V7=0,0,W7/V7)</f>
-        <v>5.4452810941765704E-2</v>
+        <v>5.1193455708919262E-2</v>
       </c>
       <c r="Y7" s="3">
         <v>4674292.5547931315</v>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C8" s="3">
         <f>J8+M8+G8+P8</f>
-        <v>262.79886093455542</v>
+        <v>236.55437705627074</v>
       </c>
       <c r="D8" s="3">
         <f>G8</f>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="E8" s="3">
         <f>J8+M8+P8</f>
-        <v>249.79511462431799</v>
+        <v>223.55063074603328</v>
       </c>
       <c r="F8" s="3">
         <v>288.78949981879617</v>
@@ -1192,14 +1192,14 @@
         <v>4.5028459547167672E-2</v>
       </c>
       <c r="I8" s="3">
-        <v>3611.250304222594</v>
+        <v>3381.6786244094469</v>
       </c>
       <c r="J8" s="3">
-        <v>220.2663512590895</v>
+        <v>194.02186738080479</v>
       </c>
       <c r="K8" s="4">
         <f>IF(I8=0,0,J8/I8)</f>
-        <v>6.0994484653011882E-2</v>
+        <v>5.7374425227851876E-2</v>
       </c>
       <c r="L8" s="3">
         <v>12917.49073548635</v>
@@ -1232,14 +1232,14 @@
         <v>4.5028459547167853E-2</v>
       </c>
       <c r="V8" s="3">
-        <v>117793026.48660821</v>
+        <v>111883027.5327851</v>
       </c>
       <c r="W8" s="3">
-        <v>5827745.3789854348</v>
+        <v>5178772.0582784116</v>
       </c>
       <c r="X8" s="4">
         <f>IF(V8=0,0,W8/V8)</f>
-        <v>4.9474451525769958E-2</v>
+        <v>4.6287378635341943E-2</v>
       </c>
       <c r="Y8" s="3">
         <v>4206781.3739942238</v>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="C9" s="3">
         <f>J9+M9+G9+P9</f>
-        <v>130.9455545631551</v>
+        <v>120.33266759714401</v>
       </c>
       <c r="D9" s="3">
         <f>G9</f>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="E9" s="3">
         <f>J9+M9+P9</f>
-        <v>125.99266412053261</v>
+        <v>115.37977715452153</v>
       </c>
       <c r="F9" s="3">
         <v>239.8280399304447</v>
@@ -1289,14 +1289,14 @@
         <v>2.065184056067389E-2</v>
       </c>
       <c r="I9" s="3">
-        <v>3111.5811139546959</v>
+        <v>2995.3735397304449</v>
       </c>
       <c r="J9" s="3">
-        <v>109.4803308499102</v>
+        <v>98.867443883899128</v>
       </c>
       <c r="K9" s="4">
         <f>IF(I9=0,0,J9/I9)</f>
-        <v>3.5184790895830147E-2</v>
+        <v>3.3006716048108065E-2</v>
       </c>
       <c r="L9" s="3">
         <v>12350.65552086042</v>
@@ -1329,14 +1329,14 @@
         <v>2.0651840560673786E-2</v>
       </c>
       <c r="V9" s="3">
-        <v>108114421.06998961</v>
+        <v>104895045.790185</v>
       </c>
       <c r="W9" s="3">
-        <v>3134771.812197804</v>
+        <v>2822333.3781914408</v>
       </c>
       <c r="X9" s="4">
         <f>IF(V9=0,0,W9/V9)</f>
-        <v>2.8994946105926601E-2</v>
+        <v>2.6906260032878746E-2</v>
       </c>
       <c r="Y9" s="3">
         <v>3782982.3163706479</v>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C12" s="3">
         <f>C14+C15+C16+C17+C18</f>
-        <v>2061.8309493830425</v>
+        <v>1902.7902287937284</v>
       </c>
       <c r="D12" s="3">
         <f>D14+D15+D16+D17+D18</f>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="E12" s="3">
         <f>E14+E15+E16+E17+E18</f>
-        <v>1467.1319909602937</v>
+        <v>1308.0912703709794</v>
       </c>
       <c r="F12" s="3">
         <f>F14+F15+F16+F17+F18</f>
@@ -1394,15 +1394,15 @@
       </c>
       <c r="I12" s="3">
         <f>I14+I15+I16+I17+I18</f>
-        <v>19407.709538433905</v>
+        <v>18088.403478171738</v>
       </c>
       <c r="J12" s="3">
         <f>J14+J15+J16+J17+J18</f>
-        <v>1278.2304393921872</v>
+        <v>1119.1897188028731</v>
       </c>
       <c r="K12" s="4">
         <f>IF(I12=0,0,J12/I12)</f>
-        <v>6.5861993495979196E-2</v>
+        <v>6.1873327856350635E-2</v>
       </c>
       <c r="L12" s="3">
         <f>L14+L15+L16+L17+L18</f>
@@ -1442,15 +1442,15 @@
       </c>
       <c r="V12" s="3">
         <f>V14+V15+V16+V17+V18</f>
-        <v>619265330.3877759</v>
+        <v>586984476.54622817</v>
       </c>
       <c r="W12" s="3">
         <f>W14+W15+W16+W17+W18</f>
-        <v>32099658.477910429</v>
+        <v>28560841.837795049</v>
       </c>
       <c r="X12" s="4">
         <f>IF(V12=0,0,W12/V12)</f>
-        <v>5.1835064717429026E-2</v>
+        <v>4.8656894652214421E-2</v>
       </c>
       <c r="Y12" s="3">
         <f>Y14+Y15+Y16+Y17+Y18</f>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="C14" s="3">
         <f>J14+M14+G14+P14</f>
-        <v>612.56026382572202</v>
+        <v>565.69219234731145</v>
       </c>
       <c r="D14" s="3">
         <f>G14</f>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="E14" s="3">
         <f>J14+M14+P14</f>
-        <v>424.86558384825406</v>
+        <v>377.99751236984349</v>
       </c>
       <c r="F14" s="3">
         <v>397.0902965307904</v>
@@ -1509,14 +1509,14 @@
         <v>0.47267506060278197</v>
       </c>
       <c r="I14" s="3">
-        <v>4595.3272879255064</v>
+        <v>4229.0317579039856</v>
       </c>
       <c r="J14" s="3">
-        <v>359.70645668022428</v>
+        <v>312.83838520181371</v>
       </c>
       <c r="K14" s="4">
         <f>IF(I14=0,0,J14/I14)</f>
-        <v>7.8276569685335404E-2</v>
+        <v>7.3973997621825438E-2</v>
       </c>
       <c r="L14" s="3">
         <v>18640.875795544409</v>
@@ -1549,14 +1549,14 @@
         <v>0.47267506060278208</v>
       </c>
       <c r="V14" s="3">
-        <v>139111960.55532151</v>
+        <v>130721936.6657657</v>
       </c>
       <c r="W14" s="3">
-        <v>8453026.7370958477</v>
+        <v>7530151.3682035357</v>
       </c>
       <c r="X14" s="4">
         <f>IF(V14=0,0,W14/V14)</f>
-        <v>6.076419815630648E-2</v>
+        <v>5.7604343695250498E-2</v>
       </c>
       <c r="Y14" s="3">
         <v>6174245.853177595</v>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C15" s="3">
         <f>J15+M15+G15+P15</f>
-        <v>506.81694623525732</v>
+        <v>465.42086281069476</v>
       </c>
       <c r="D15" s="3">
         <f>G15</f>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="E15" s="3">
         <f>J15+M15+P15</f>
-        <v>358.94189218021654</v>
+        <v>317.54580875565398</v>
       </c>
       <c r="F15" s="3">
         <v>346.92132413597358</v>
@@ -1606,14 +1606,14 @@
         <v>0.42624953776863289</v>
       </c>
       <c r="I15" s="3">
-        <v>4112.5343319715366</v>
+        <v>3787.0627176324879</v>
       </c>
       <c r="J15" s="3">
-        <v>316.53763125915589</v>
+        <v>275.14154783459333</v>
       </c>
       <c r="K15" s="4">
         <f>IF(I15=0,0,J15/I15)</f>
-        <v>7.6968994227802276E-2</v>
+        <v>7.2653021180119307E-2</v>
       </c>
       <c r="L15" s="3">
         <v>15402.279753726511</v>
@@ -1646,14 +1646,14 @@
         <v>0.42624953776863289</v>
       </c>
       <c r="V15" s="3">
-        <v>128962196.4271194</v>
+        <v>121072766.34225529</v>
       </c>
       <c r="W15" s="3">
-        <v>7862063.5119100511</v>
+        <v>6967680.9027350992</v>
       </c>
       <c r="X15" s="4">
         <f>IF(V15=0,0,W15/V15)</f>
-        <v>6.0964094360420967E-2</v>
+        <v>5.7549530858479497E-2</v>
       </c>
       <c r="Y15" s="3">
         <v>5221398.5281040482</v>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C16" s="3">
         <f>J16+M16+G16+P16</f>
-        <v>424.61201389170077</v>
+        <v>390.69281904965561</v>
       </c>
       <c r="D16" s="3">
         <f>G16</f>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="E16" s="3">
         <f>J16+M16+P16</f>
-        <v>307.53673618697235</v>
+        <v>273.61754134492719</v>
       </c>
       <c r="F16" s="3">
         <v>308.40246775221379</v>
@@ -1703,14 +1703,14 @@
         <v>0.37961848540976212</v>
       </c>
       <c r="I16" s="3">
-        <v>3977.0165003595712</v>
+        <v>3695.2568384953711</v>
       </c>
       <c r="J16" s="3">
-        <v>272.23966934380729</v>
+        <v>238.32047450176211</v>
       </c>
       <c r="K16" s="4">
         <f>IF(I16=0,0,J16/I16)</f>
-        <v>6.8453241096483625E-2</v>
+        <v>6.44936157127311E-2</v>
       </c>
       <c r="L16" s="3">
         <v>13777.53512556912</v>
@@ -1743,14 +1743,14 @@
         <v>0.37961848540976206</v>
       </c>
       <c r="V16" s="3">
-        <v>125283725.8487372</v>
+        <v>118411700.21523701</v>
       </c>
       <c r="W16" s="3">
-        <v>6822051.0377212912</v>
+        <v>6061904.1303865612</v>
       </c>
       <c r="X16" s="4">
         <f>IF(V16=0,0,W16/V16)</f>
-        <v>5.4452810941765704E-2</v>
+        <v>5.1193455708919262E-2</v>
       </c>
       <c r="Y16" s="3">
         <v>4674292.5547931315</v>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="C17" s="3">
         <f>J17+M17+G17+P17</f>
-        <v>348.86793842258635</v>
+        <v>322.62345454430164</v>
       </c>
       <c r="D17" s="3">
         <f>G17</f>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="E17" s="3">
         <f>J17+M17+P17</f>
-        <v>249.79511462431799</v>
+        <v>223.55063074603328</v>
       </c>
       <c r="F17" s="3">
         <v>288.78949981879617</v>
@@ -1800,14 +1800,14 @@
         <v>0.3430624169522527</v>
       </c>
       <c r="I17" s="3">
-        <v>3611.250304222594</v>
+        <v>3381.6786244094469</v>
       </c>
       <c r="J17" s="3">
-        <v>220.2663512590895</v>
+        <v>194.02186738080479</v>
       </c>
       <c r="K17" s="4">
         <f>IF(I17=0,0,J17/I17)</f>
-        <v>6.0994484653011882E-2</v>
+        <v>5.7374425227851876E-2</v>
       </c>
       <c r="L17" s="3">
         <v>12917.49073548635</v>
@@ -1840,14 +1840,14 @@
         <v>0.34306241695225254</v>
       </c>
       <c r="V17" s="3">
-        <v>117793026.48660821</v>
+        <v>111883027.5327851</v>
       </c>
       <c r="W17" s="3">
-        <v>5827745.3789854348</v>
+        <v>5178772.0582784116</v>
       </c>
       <c r="X17" s="4">
         <f>IF(V17=0,0,W17/V17)</f>
-        <v>4.9474451525769958E-2</v>
+        <v>4.6287378635341943E-2</v>
       </c>
       <c r="Y17" s="3">
         <v>4206781.3739942238</v>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C18" s="3">
         <f>J18+M18+G18+P18</f>
-        <v>168.97378700777597</v>
+        <v>158.36090004176489</v>
       </c>
       <c r="D18" s="3">
         <f>G18</f>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E18" s="3">
         <f>J18+M18+P18</f>
-        <v>125.99266412053261</v>
+        <v>115.37977715452153</v>
       </c>
       <c r="F18" s="3">
         <v>239.8280399304447</v>
@@ -1897,14 +1897,14 @@
         <v>0.17921642064751389</v>
       </c>
       <c r="I18" s="3">
-        <v>3111.5811139546959</v>
+        <v>2995.3735397304449</v>
       </c>
       <c r="J18" s="3">
-        <v>109.4803308499102</v>
+        <v>98.867443883899128</v>
       </c>
       <c r="K18" s="4">
         <f>IF(I18=0,0,J18/I18)</f>
-        <v>3.5184790895830147E-2</v>
+        <v>3.3006716048108065E-2</v>
       </c>
       <c r="L18" s="3">
         <v>12350.65552086042</v>
@@ -1937,14 +1937,14 @@
         <v>0.17921642064751397</v>
       </c>
       <c r="V18" s="3">
-        <v>108114421.06998961</v>
+        <v>104895045.790185</v>
       </c>
       <c r="W18" s="3">
-        <v>3134771.812197804</v>
+        <v>2822333.3781914408</v>
       </c>
       <c r="X18" s="4">
         <f>IF(V18=0,0,W18/V18)</f>
-        <v>2.8994946105926601E-2</v>
+        <v>2.6906260032878746E-2</v>
       </c>
       <c r="Y18" s="3">
         <v>3782982.3163706479</v>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C21" s="3">
         <f>C23+C24+C25+C26+C27</f>
-        <v>2111.7120178026412</v>
+        <v>2011.3640256098345</v>
       </c>
       <c r="D21" s="3">
         <f>D23+D24+D25+D26+D27</f>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="E21" s="3">
         <f>E23+E24+E25+E26+E27</f>
-        <v>1036.6092357144523</v>
+        <v>936.26124352164572</v>
       </c>
       <c r="F21" s="3">
         <f>F23+F24+F25+F26+F27</f>
@@ -2006,11 +2006,11 @@
       </c>
       <c r="J21" s="3">
         <f>J23+J24+J25+J26+J27</f>
-        <v>686.2475247770335</v>
+        <v>585.89953258422668</v>
       </c>
       <c r="K21" s="4">
         <f>IF(I21=0,0,J21/I21)</f>
-        <v>0.18635698511231386</v>
+        <v>0.15910654177818098</v>
       </c>
       <c r="L21" s="3">
         <f>L23+L24+L25+L26+L27</f>
@@ -2054,11 +2054,11 @@
       </c>
       <c r="W21" s="3">
         <f>W23+W24+W25+W26+W27</f>
-        <v>16489023.35117919</v>
+        <v>13782093.295542261</v>
       </c>
       <c r="X21" s="4">
         <f>IF(V21=0,0,W21/V21)</f>
-        <v>0.15457943735449806</v>
+        <v>0.12920281461301755</v>
       </c>
       <c r="Y21" s="3">
         <f>Y23+Y24+Y25+Y26+Y27</f>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="C23" s="3">
         <f>J23+M23+G23+P23</f>
-        <v>550.58183910185278</v>
+        <v>525.35232482572508</v>
       </c>
       <c r="D23" s="3">
         <f>G23</f>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="E23" s="3">
         <f>J23+M23+P23</f>
-        <v>273.10039630625363</v>
+        <v>247.87088203012584</v>
       </c>
       <c r="F23" s="3">
         <v>428.09244082133358</v>
@@ -2120,11 +2120,11 @@
         <v>991.82050542122556</v>
       </c>
       <c r="J23" s="3">
-        <v>162.60977052226261</v>
+        <v>137.38025624613479</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
-        <v>0.16395080524494937</v>
+        <v>0.13851322441432029</v>
       </c>
       <c r="L23" s="3">
         <v>18248.150900694091</v>
@@ -2160,11 +2160,11 @@
         <v>25699987.560610589</v>
       </c>
       <c r="W23" s="3">
-        <v>3313562.2441319791</v>
+        <v>2724438.1987594548</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
-        <v>0.12893244544641541</v>
+        <v>0.10600931974516203</v>
       </c>
       <c r="Y23" s="3">
         <v>1959206.3612258229</v>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="C24" s="3">
         <f>J24+M24+G24+P24</f>
-        <v>524.38521669671627</v>
+        <v>502.10011734093223</v>
       </c>
       <c r="D24" s="3">
         <f>G24</f>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E24" s="3">
         <f>J24+M24+P24</f>
-        <v>250.61471502859939</v>
+        <v>228.32961567281538</v>
       </c>
       <c r="F24" s="3">
         <v>437.75116549754102</v>
@@ -2217,11 +2217,11 @@
         <v>847.52939170447485</v>
       </c>
       <c r="J24" s="3">
-        <v>151.9237102732427</v>
+        <v>129.63861091745869</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
-        <v>0.17925479842971276</v>
+        <v>0.15296060784009058</v>
       </c>
       <c r="L24" s="3">
         <v>18442.648959675</v>
@@ -2257,11 +2257,11 @@
         <v>23322467.600951109</v>
       </c>
       <c r="W24" s="3">
-        <v>3386920.8556735781</v>
+        <v>2821008.1417387952</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
-        <v>0.14522137681243716</v>
+        <v>0.12095667534012362</v>
       </c>
       <c r="Y24" s="3">
         <v>2033978.1299748039</v>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C25" s="3">
         <f>J25+M25+G25+P25</f>
-        <v>417.64037577601232</v>
+        <v>397.67985371592215</v>
       </c>
       <c r="D25" s="3">
         <f>G25</f>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="E25" s="3">
         <f>J25+M25+P25</f>
-        <v>203.35601819441447</v>
+        <v>183.39549613432428</v>
       </c>
       <c r="F25" s="3">
         <v>396.28526128416758</v>
@@ -2314,11 +2314,11 @@
         <v>721.62080381298233</v>
       </c>
       <c r="J25" s="3">
-        <v>137.9599041540084</v>
+        <v>117.9993820939182</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
-        <v>0.19118060818790161</v>
+        <v>0.16351992829255976</v>
       </c>
       <c r="L25" s="3">
         <v>15355.961975565249</v>
@@ -2354,11 +2354,11 @@
         <v>21162807.846375171</v>
       </c>
       <c r="W25" s="3">
-        <v>3343728.0163370739</v>
+        <v>2800683.8604466021</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
-        <v>0.15800020680666899</v>
+        <v>0.13233989935443805</v>
       </c>
       <c r="Y25" s="3">
         <v>1664123.912966297</v>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C26" s="3">
         <f>J26+M26+G26+P26</f>
-        <v>344.40259067183274</v>
+        <v>325.4816190604223</v>
       </c>
       <c r="D26" s="3">
         <f>G26</f>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="E26" s="3">
         <f>J26+M26+P26</f>
-        <v>175.31172351435274</v>
+        <v>156.39075190294236</v>
       </c>
       <c r="F26" s="3">
         <v>351.26672270713158</v>
@@ -2411,11 +2411,11 @@
         <v>656.23600296293523</v>
       </c>
       <c r="J26" s="3">
-        <v>130.83245085781229</v>
+        <v>111.9114792464019</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
-        <v>0.19936798692406063</v>
+        <v>0.17053541521817839</v>
       </c>
       <c r="L26" s="3">
         <v>12320.893910346331</v>
@@ -2451,11 +2451,11 @@
         <v>20232379.411657181</v>
       </c>
       <c r="W26" s="3">
-        <v>3361820.0850684568</v>
+        <v>2815905.181914039</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
-        <v>0.16616039155194445</v>
+        <v>0.13917815223905963</v>
       </c>
       <c r="Y26" s="3">
         <v>1291512.2728871789</v>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="C27" s="3">
         <f>J27+M27+G27+P27</f>
-        <v>274.70199555622702</v>
+        <v>260.75011066683265</v>
       </c>
       <c r="D27" s="3">
         <f>G27</f>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="E27" s="3">
         <f>J27+M27+P27</f>
-        <v>134.22638267083227</v>
+        <v>120.27449778143787</v>
       </c>
       <c r="F27" s="3">
         <v>308.52409051931693</v>
@@ -2508,11 +2508,11 @@
         <v>465.22851237667129</v>
       </c>
       <c r="J27" s="3">
-        <v>102.9216889697075</v>
+        <v>88.969804080313125</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
-        <v>0.22122824855235265</v>
+        <v>0.19123893251039376</v>
       </c>
       <c r="L27" s="3">
         <v>10752.450404824391</v>
@@ -2548,11 +2548,11 @@
         <v>16252582.504079361</v>
       </c>
       <c r="W27" s="3">
-        <v>3082992.149968103</v>
+        <v>2620057.9126833701</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
-        <v>0.18969244728917875</v>
+        <v>0.16120871326299938</v>
       </c>
       <c r="Y27" s="3">
         <v>1133183.161267315</v>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="C30" s="3">
         <f>C32+C33+C34+C35+C36</f>
-        <v>295.99211166518984</v>
+        <v>283.3332129957933</v>
       </c>
       <c r="D30" s="3">
         <f>D32+D33+D34+D35+D36</f>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="E30" s="3">
         <f>E32+E33+E34+E35+E36</f>
-        <v>103.61429706996172</v>
+        <v>90.955398400565215</v>
       </c>
       <c r="F30" s="3">
         <f>F32+F33+F34+F35+F36</f>
@@ -2614,11 +2614,11 @@
       </c>
       <c r="J30" s="3">
         <f>J32+J33+J34+J35+J36</f>
-        <v>86.645889706201388</v>
+        <v>73.986991036804866</v>
       </c>
       <c r="K30" s="4">
         <f>IF(I30=0,0,J30/I30)</f>
-        <v>2.3529508224117899E-2</v>
+        <v>2.0091864945714095E-2</v>
       </c>
       <c r="L30" s="3">
         <f>L32+L33+L34+L35+L36</f>
@@ -2662,11 +2662,11 @@
       </c>
       <c r="W30" s="3">
         <f>W32+W33+W34+W35+W36</f>
-        <v>2113147.9465661086</v>
+        <v>1767252.4081023186</v>
       </c>
       <c r="X30" s="4">
         <f>IF(V30=0,0,W30/V30)</f>
-        <v>1.9810101160639214E-2</v>
+        <v>1.6567438658415267E-2</v>
       </c>
       <c r="Y30" s="3">
         <f>Y32+Y33+Y34+Y35+Y36</f>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C32" s="3">
         <f>J32+M32+G32+P32</f>
-        <v>33.333098332242749</v>
+        <v>31.154475954145141</v>
       </c>
       <c r="D32" s="3">
         <f>G32</f>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="E32" s="3">
         <f>J32+M32+P32</f>
-        <v>16.30706237825914</v>
+        <v>14.128440000161532</v>
       </c>
       <c r="F32" s="3">
         <v>428.09244082133358</v>
@@ -2728,11 +2728,11 @@
         <v>991.82050542122556</v>
       </c>
       <c r="J32" s="3">
-        <v>13.849887789733589</v>
+        <v>11.67126541163598</v>
       </c>
       <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
-        <v>1.3964107128286838E-2</v>
+        <v>1.1767517759354251E-2</v>
       </c>
       <c r="L32" s="3">
         <v>18248.150900694091</v>
@@ -2768,11 +2768,11 @@
         <v>25699987.560610589</v>
       </c>
       <c r="W32" s="3">
-        <v>277309.83426191658</v>
+        <v>227272.75268540901</v>
       </c>
       <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
-        <v>1.0790271147326896E-2</v>
+        <v>8.8433020502212793E-3</v>
       </c>
       <c r="Y32" s="3">
         <v>1959206.3612258229</v>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="C33" s="3">
         <f>J33+M33+G33+P33</f>
-        <v>53.94667240773223</v>
+        <v>51.454722558748443</v>
       </c>
       <c r="D33" s="3">
         <f>G33</f>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="E33" s="3">
         <f>J33+M33+P33</f>
-        <v>20.198190632169077</v>
+        <v>17.706240783185294</v>
       </c>
       <c r="F33" s="3">
         <v>437.75116549754102</v>
@@ -2825,11 +2825,11 @@
         <v>847.52939170447485</v>
       </c>
       <c r="J33" s="3">
-        <v>16.815069467100081</v>
+        <v>14.3231196181163</v>
       </c>
       <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
-        <v>1.9840101867479931E-2</v>
+        <v>1.6899850032706158E-2</v>
       </c>
       <c r="L33" s="3">
         <v>18442.648959675</v>
@@ -2865,11 +2865,11 @@
         <v>23322467.600951109</v>
       </c>
       <c r="W33" s="3">
-        <v>369838.35950630158</v>
+        <v>307442.101903148</v>
       </c>
       <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
-        <v>1.5857599883265322E-2</v>
+        <v>1.3182228705962926E-2</v>
       </c>
       <c r="Y33" s="3">
         <v>2033978.1299748039</v>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C34" s="3">
         <f>J34+M34+G34+P34</f>
-        <v>65.031316955350277</v>
+        <v>62.342351079779156</v>
       </c>
       <c r="D34" s="3">
         <f>G34</f>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="E34" s="3">
         <f>J34+M34+P34</f>
-        <v>22.47689109481836</v>
+        <v>19.787925219247239</v>
       </c>
       <c r="F34" s="3">
         <v>396.28526128416758</v>
@@ -2922,11 +2922,11 @@
         <v>721.62080381298233</v>
       </c>
       <c r="J34" s="3">
-        <v>18.469011170364681</v>
+        <v>15.78004529479356</v>
       </c>
       <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
-        <v>2.5593789803143165E-2</v>
+        <v>2.1867503280688632E-2</v>
       </c>
       <c r="L34" s="3">
         <v>15355.961975565249</v>
@@ -2962,11 +2962,11 @@
         <v>21162807.846375171</v>
       </c>
       <c r="W34" s="3">
-        <v>441593.2794682458</v>
+        <v>369371.39764320478</v>
       </c>
       <c r="X34" s="4">
         <f>IF(V34=0,0,W34/V34)</f>
-        <v>2.0866478714632531E-2</v>
+        <v>1.7453799152009584E-2</v>
       </c>
       <c r="Y34" s="3">
         <v>1664123.912966297</v>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="C35" s="3">
         <f>J35+M35+G35+P35</f>
-        <v>73.367237213514912</v>
+        <v>70.415390099069029</v>
       </c>
       <c r="D35" s="3">
         <f>G35</f>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="E35" s="3">
         <f>J35+M35+P35</f>
-        <v>23.208787727471961</v>
+        <v>20.256940613026089</v>
       </c>
       <c r="F35" s="3">
         <v>351.26672270713158</v>
@@ -3019,11 +3019,11 @@
         <v>656.23600296293523</v>
       </c>
       <c r="J35" s="3">
-        <v>20.289220375396191</v>
+        <v>17.337373260950319</v>
       </c>
       <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
-        <v>3.0917566673863431E-2</v>
+        <v>2.6419417987844761E-2</v>
       </c>
       <c r="L35" s="3">
         <v>12320.893910346331</v>
@@ -3059,11 +3059,11 @@
         <v>20232379.411657181</v>
       </c>
       <c r="W35" s="3">
-        <v>514684.47839863971</v>
+        <v>430534.00670235232</v>
       </c>
       <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
-        <v>2.5438652959527675E-2</v>
+        <v>2.1279454973758244E-2</v>
       </c>
       <c r="Y35" s="3">
         <v>1291512.2728871789</v>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C36" s="3">
         <f>J36+M36+G36+P36</f>
-        <v>70.313786756349657</v>
+        <v>67.966273304051526</v>
       </c>
       <c r="D36" s="3">
         <f>G36</f>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="E36" s="3">
         <f>J36+M36+P36</f>
-        <v>21.423365237243186</v>
+        <v>19.075851784945058</v>
       </c>
       <c r="F36" s="3">
         <v>308.52409051931693</v>
@@ -3116,11 +3116,11 @@
         <v>465.22851237667129</v>
       </c>
       <c r="J36" s="3">
-        <v>17.222700903606839</v>
+        <v>14.87518745130871</v>
       </c>
       <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
-        <v>3.7019873987565309E-2</v>
+        <v>3.1973937657683901E-2</v>
       </c>
       <c r="L36" s="3">
         <v>10752.450404824391</v>
@@ -3156,11 +3156,11 @@
         <v>16252582.504079361</v>
       </c>
       <c r="W36" s="3">
-        <v>509721.99493100488</v>
+        <v>432632.14916820452</v>
       </c>
       <c r="X36" s="4">
         <f>IF(V36=0,0,W36/V36)</f>
-        <v>3.1362523143818273E-2</v>
+        <v>2.6619286446299524E-2</v>
       </c>
       <c r="Y36" s="3">
         <v>1133183.161267315</v>

</xml_diff>

<commit_message>
Apply India baseline changes to all modeled pathways, make some other small fixes
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
@@ -1,44 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\src\vivarium_gates_lsff_by_wealth_quintile\5000_analyze_results\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5AD325F-8559-4870-A355-6119A5DEDD2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Model Results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="J39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="J39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -51,7 +32,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="K39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -64,7 +45,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="W39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -77,7 +58,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="X39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -90,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="J48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -103,7 +84,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="K48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -116,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="W48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -129,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="X48" authorId="0">
       <text>
         <r>
           <rPr>
@@ -272,12 +253,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0%;\-0.0%;&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0%;-0.0%;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,21 +340,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -411,7 +384,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -445,7 +418,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -480,10 +452,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -656,9 +627,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AD54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
@@ -667,7 +638,7 @@
     <col min="19" max="30" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30">
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
@@ -751,1584 +722,1584 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30">
       <c r="B3" t="s">
         <v>28</v>
       </c>
       <c r="C3" s="3">
         <f>C5+C6+C7+C8+C9</f>
-        <v>1391.4362330092995</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3">
         <f>D5+D6+D7+D8+D9</f>
-        <v>83.344962638319814</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3">
         <f>E5+E6+E7+E8+E9</f>
-        <v>1308.0912703709794</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3">
         <f>F5+F6+F7+F8+F9</f>
-        <v>1581.0316281682187</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3">
         <f>G5+G6+G7+G8+G9</f>
-        <v>83.344962638319814</v>
+        <v>0</v>
       </c>
       <c r="H3" s="4">
         <f>IF(F3=0,0,G3/F3)</f>
-        <v>5.27155568259461E-2</v>
+        <v>0</v>
       </c>
       <c r="I3" s="3">
         <f>I5+I6+I7+I8+I9</f>
-        <v>18088.403478171738</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3">
         <f>J5+J6+J7+J8+J9</f>
-        <v>1119.1897188028731</v>
+        <v>0</v>
       </c>
       <c r="K3" s="4">
         <f>IF(I3=0,0,J3/I3)</f>
-        <v>6.1873327856350635E-2</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>L5+L6+L7+L8+L9</f>
-        <v>73088.836931186815</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>M5+M6+M7+M8+M9</f>
-        <v>151.25580362673105</v>
+        <v>0</v>
       </c>
       <c r="N3" s="4">
         <f>IF(L3=0,0,M3/L3)</f>
-        <v>2.0694788695179056E-3</v>
+        <v>0</v>
       </c>
       <c r="O3" s="3">
         <f>O5+O6+O7+O8+O9</f>
-        <v>2235.0590017749987</v>
+        <v>0</v>
       </c>
       <c r="P3" s="3">
         <f>P5+P6+P7+P8+P9</f>
-        <v>37.645747941375426</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="4">
         <f>IF(O3=0,0,P3/O3)</f>
-        <v>1.6843290450712312E-2</v>
+        <v>0</v>
       </c>
       <c r="S3" s="3">
         <f>S5+S6+S7+S8+S9</f>
-        <v>17575.212094927279</v>
+        <v>0</v>
       </c>
       <c r="T3" s="3">
         <f>T5+T6+T7+T8+T9</f>
-        <v>926.48709191819546</v>
+        <v>0</v>
       </c>
       <c r="U3" s="4">
         <f>IF(S3=0,0,T3/S3)</f>
-        <v>5.2715556825946169E-2</v>
+        <v>0</v>
       </c>
       <c r="V3" s="3">
         <f>V5+V6+V7+V8+V9</f>
-        <v>586984476.54622817</v>
+        <v>0</v>
       </c>
       <c r="W3" s="3">
         <f>W5+W6+W7+W8+W9</f>
-        <v>28560841.837795049</v>
+        <v>0</v>
       </c>
       <c r="X3" s="4">
         <f>IF(V3=0,0,W3/V3)</f>
-        <v>4.8656894652214421E-2</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="3">
         <f>Y5+Y6+Y7+Y8+Y9</f>
-        <v>24059700.626439646</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="3">
         <f>Z5+Z6+Z7+Z8+Z9</f>
-        <v>376108.59127695486</v>
+        <v>0</v>
       </c>
       <c r="AA3" s="4">
         <f>IF(Y3=0,0,Z3/Y3)</f>
-        <v>1.5632305535158746E-2</v>
+        <v>0</v>
       </c>
       <c r="AB3" s="3">
         <f>AB5+AB6+AB7+AB8+AB9</f>
-        <v>815643.03969645977</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="3">
         <f>AC5+AC6+AC7+AC8+AC9</f>
-        <v>1680.7280119055067</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="4">
         <f>IF(AB3=0,0,AC3/AB3)</f>
-        <v>2.0606171206107356E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30">
       <c r="A4" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30">
       <c r="B5" t="s">
         <v>30</v>
       </c>
       <c r="C5" s="3">
         <f>J5+M5+G5+P5</f>
-        <v>406.30987716553807</v>
+        <v>0</v>
       </c>
       <c r="D5" s="3">
         <f>G5</f>
-        <v>28.312364795694592</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3">
         <f>J5+M5+P5</f>
-        <v>377.99751236984349</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3">
-        <v>397.0902965307904</v>
+        <v>363.1566259346982</v>
       </c>
       <c r="G5" s="3">
-        <v>28.312364795694592</v>
+        <v>25.60632743086544</v>
       </c>
       <c r="H5" s="4">
         <f>IF(F5=0,0,G5/F5)</f>
-        <v>7.1299563457097093E-2</v>
+        <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>4229.0317579039856</v>
+        <v>4215.705028068518</v>
       </c>
       <c r="J5" s="3">
-        <v>312.83838520181371</v>
+        <v>311.1262929552929</v>
       </c>
       <c r="K5" s="4">
         <f>IF(I5=0,0,J5/I5)</f>
-        <v>7.3973997621825438E-2</v>
+        <v>0</v>
       </c>
       <c r="L5" s="3">
-        <v>18640.875795544409</v>
+        <v>18587.84837263764</v>
       </c>
       <c r="M5" s="3">
-        <v>53.027422906763853</v>
+        <v>48.27357658215985</v>
       </c>
       <c r="N5" s="4">
         <f>IF(L5=0,0,M5/L5)</f>
-        <v>2.8446851686785343E-3</v>
+        <v>0</v>
       </c>
       <c r="O5" s="3">
-        <v>603.60362214169209</v>
+        <v>591.4719178804262</v>
       </c>
       <c r="P5" s="3">
-        <v>12.131704261265931</v>
+        <v>9.426500014935039</v>
       </c>
       <c r="Q5" s="4">
         <f>IF(O5=0,0,P5/O5)</f>
-        <v>2.0098793009592129E-2</v>
+        <v>0</v>
       </c>
       <c r="S5" s="3">
-        <v>4414.1724036552041</v>
+        <v>4036.955751400944</v>
       </c>
       <c r="T5" s="3">
-        <v>314.72856540498111</v>
+        <v>284.647459008158</v>
       </c>
       <c r="U5" s="4">
         <f>IF(S5=0,0,T5/S5)</f>
-        <v>7.1299563457097107E-2</v>
+        <v>0</v>
       </c>
       <c r="V5" s="3">
-        <v>130721936.6657657</v>
+        <v>130504106.3683567</v>
       </c>
       <c r="W5" s="3">
-        <v>7530151.3682035357</v>
+        <v>7529815.832129106</v>
       </c>
       <c r="X5" s="4">
         <f>IF(V5=0,0,W5/V5)</f>
-        <v>5.7604343695250498E-2</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="3">
-        <v>6174245.853177595</v>
+        <v>6056561.99351707</v>
       </c>
       <c r="Z5" s="3">
-        <v>117683.8596605249</v>
+        <v>113528.6322764717</v>
       </c>
       <c r="AA5" s="4">
         <f>IF(Y5=0,0,Z5/Y5)</f>
-        <v>1.9060442758358664E-2</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="3">
-        <v>208016.4497539358</v>
+        <v>207427.2646575113</v>
       </c>
       <c r="AC5" s="3">
-        <v>589.18509642445133</v>
+        <v>536.4685351653607</v>
       </c>
       <c r="AD5" s="4">
         <f>IF(AB5=0,0,AC5/AB5)</f>
-        <v>2.8323966547905356E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30">
       <c r="B6" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="3">
         <f>J6+M6+G6+P6</f>
-        <v>338.69031697899226</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3">
         <f>G6</f>
-        <v>21.144508223338281</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3">
         <f>J6+M6+P6</f>
-        <v>317.54580875565398</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3">
-        <v>346.92132413597358</v>
+        <v>320.8109788943828</v>
       </c>
       <c r="G6" s="3">
-        <v>21.144508223338281</v>
+        <v>19.29712236727314</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
-        <v>6.0949001264191033E-2</v>
+        <v>0</v>
       </c>
       <c r="I6" s="3">
-        <v>3787.0627176324879</v>
+        <v>3777.348955767648</v>
       </c>
       <c r="J6" s="3">
-        <v>275.14154783459333</v>
+        <v>273.8748450018219</v>
       </c>
       <c r="K6" s="4">
         <f>IF(I6=0,0,J6/I6)</f>
-        <v>7.2653021180119307E-2</v>
+        <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>15402.279753726511</v>
+        <v>15367.67605497631</v>
       </c>
       <c r="M6" s="3">
-        <v>34.603698750201623</v>
+        <v>30.71036729697697</v>
       </c>
       <c r="N6" s="4">
         <f>IF(L6=0,0,M6/L6)</f>
-        <v>2.2466608387520957E-3</v>
+        <v>0</v>
       </c>
       <c r="O6" s="3">
-        <v>477.03495714807917</v>
+        <v>469.2343949772201</v>
       </c>
       <c r="P6" s="3">
-        <v>7.8005621708590773</v>
+        <v>6.561405479874811</v>
       </c>
       <c r="Q6" s="4">
         <f>IF(O6=0,0,P6/O6)</f>
-        <v>1.6352181436543361E-2</v>
+        <v>0</v>
       </c>
       <c r="S6" s="3">
-        <v>3856.4793665810321</v>
+        <v>3566.229097505511</v>
       </c>
       <c r="T6" s="3">
-        <v>235.0485657890745</v>
+        <v>214.5124818404361</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
-        <v>6.0949001264191172E-2</v>
+        <v>0</v>
       </c>
       <c r="V6" s="3">
-        <v>121072766.34225529</v>
+        <v>120904784.0220684</v>
       </c>
       <c r="W6" s="3">
-        <v>6967680.9027350992</v>
+        <v>6963839.795960322</v>
       </c>
       <c r="X6" s="4">
         <f>IF(V6=0,0,W6/V6)</f>
-        <v>5.7549530858479497E-2</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="3">
-        <v>5221398.5281040482</v>
+        <v>5132795.053668289</v>
       </c>
       <c r="Z6" s="3">
-        <v>88603.474435759708</v>
+        <v>85655.40422302578</v>
       </c>
       <c r="AA6" s="4">
         <f>IF(Y6=0,0,Z6/Y6)</f>
-        <v>1.6969299309151312E-2</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="3">
-        <v>171868.3936012006</v>
+        <v>171483.8728014289</v>
       </c>
       <c r="AC6" s="3">
-        <v>384.52079977173707</v>
+        <v>341.1071610878571</v>
       </c>
       <c r="AD6" s="4">
         <f>IF(AB6=0,0,AC6/AB6)</f>
-        <v>2.2372979214780476E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30">
       <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="3">
         <f>J7+M7+G7+P7</f>
-        <v>289.54899421135423</v>
+        <v>0</v>
       </c>
       <c r="D7" s="3">
         <f>G7</f>
-        <v>15.931452866427019</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3">
         <f>J7+M7+P7</f>
-        <v>273.61754134492719</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3">
-        <v>308.40246775221379</v>
+        <v>288.0128603408813</v>
       </c>
       <c r="G7" s="3">
-        <v>15.931452866427019</v>
+        <v>14.64607722620195</v>
       </c>
       <c r="H7" s="4">
         <f>IF(F7=0,0,G7/F7)</f>
-        <v>5.1657994122236262E-2</v>
+        <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>3695.2568384953711</v>
+        <v>3687.87367156503</v>
       </c>
       <c r="J7" s="3">
-        <v>238.32047450176211</v>
+        <v>237.3412499570018</v>
       </c>
       <c r="K7" s="4">
         <f>IF(I7=0,0,J7/I7)</f>
-        <v>6.44936157127311E-2</v>
+        <v>0</v>
       </c>
       <c r="L7" s="3">
-        <v>13777.53512556912</v>
+        <v>13749.34694539489</v>
       </c>
       <c r="M7" s="3">
-        <v>28.188180174233391</v>
+        <v>26.21495619864762</v>
       </c>
       <c r="N7" s="4">
         <f>IF(L7=0,0,M7/L7)</f>
-        <v>2.0459523359820865E-3</v>
+        <v>0</v>
       </c>
       <c r="O7" s="3">
-        <v>419.32297040011582</v>
+        <v>412.2140837311841</v>
       </c>
       <c r="P7" s="3">
-        <v>7.1088866689316932</v>
+        <v>3.678403565003595</v>
       </c>
       <c r="Q7" s="4">
         <f>IF(O7=0,0,P7/O7)</f>
-        <v>1.6953248857672715E-2</v>
+        <v>0</v>
       </c>
       <c r="S7" s="3">
-        <v>3428.292441957034</v>
+        <v>3201.635575388428</v>
       </c>
       <c r="T7" s="3">
-        <v>177.09871081592379</v>
+        <v>162.8100975484062</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
-        <v>5.1657994122236359E-2</v>
+        <v>0</v>
       </c>
       <c r="V7" s="3">
-        <v>118411700.21523701</v>
+        <v>118273982.4631039</v>
       </c>
       <c r="W7" s="3">
-        <v>6061904.1303865612</v>
+        <v>6057749.0648617</v>
       </c>
       <c r="X7" s="4">
         <f>IF(V7=0,0,W7/V7)</f>
-        <v>5.1193455708919262E-2</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="3">
-        <v>4674292.5547931315</v>
+        <v>4603060.971989882</v>
       </c>
       <c r="Z7" s="3">
-        <v>71231.58280325029</v>
+        <v>67998.01526465267</v>
       </c>
       <c r="AA7" s="4">
         <f>IF(Y7=0,0,Z7/Y7)</f>
-        <v>1.5239008249538792E-2</v>
+        <v>0</v>
       </c>
       <c r="AB7" s="3">
-        <v>153755.60334743661</v>
+        <v>153442.4049540742</v>
       </c>
       <c r="AC7" s="3">
-        <v>313.19839336245792</v>
+        <v>291.4915740205033</v>
       </c>
       <c r="AD7" s="4">
         <f>IF(AB7=0,0,AC7/AB7)</f>
-        <v>2.036988483956149E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30">
       <c r="B8" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="3">
         <f>J8+M8+G8+P8</f>
-        <v>236.55437705627074</v>
+        <v>0</v>
       </c>
       <c r="D8" s="3">
         <f>G8</f>
-        <v>13.00374631023745</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3">
         <f>J8+M8+P8</f>
-        <v>223.55063074603328</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>288.78949981879617</v>
+        <v>271.5819334790612</v>
       </c>
       <c r="G8" s="3">
-        <v>13.00374631023745</v>
+        <v>12.00853732205968</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
-        <v>4.5028459547167672E-2</v>
+        <v>0</v>
       </c>
       <c r="I8" s="3">
-        <v>3381.6786244094469</v>
+        <v>3375.640124395373</v>
       </c>
       <c r="J8" s="3">
-        <v>194.02186738080479</v>
+        <v>193.1881464041606</v>
       </c>
       <c r="K8" s="4">
         <f>IF(I8=0,0,J8/I8)</f>
-        <v>5.7374425227851876E-2</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3">
-        <v>12917.49073548635</v>
+        <v>12894.33743826528</v>
       </c>
       <c r="M8" s="3">
-        <v>23.15329722107202</v>
+        <v>21.20628217103705</v>
       </c>
       <c r="N8" s="4">
         <f>IF(L8=0,0,M8/L8)</f>
-        <v>1.7923989802033551E-3</v>
+        <v>0</v>
       </c>
       <c r="O8" s="3">
-        <v>383.40598517692439</v>
+        <v>377.0305190327679</v>
       </c>
       <c r="P8" s="3">
-        <v>6.3754661441564684</v>
+        <v>7.029277368942742</v>
       </c>
       <c r="Q8" s="4">
         <f>IF(O8=0,0,P8/O8)</f>
-        <v>1.6628499268769841E-2</v>
+        <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3210.2689280060872</v>
+        <v>3018.984564891375</v>
       </c>
       <c r="T8" s="3">
-        <v>144.553464560252</v>
+        <v>133.4904290495269</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
-        <v>4.5028459547167853E-2</v>
+        <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>111883027.5327851</v>
+        <v>111762860.6181328</v>
       </c>
       <c r="W8" s="3">
-        <v>5178772.0582784116</v>
+        <v>5173153.551915213</v>
       </c>
       <c r="X8" s="4">
         <f>IF(V8=0,0,W8/V8)</f>
-        <v>4.6287378635341943E-2</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="3">
-        <v>4206781.3739942238</v>
+        <v>4143959.549376771</v>
       </c>
       <c r="Z8" s="3">
-        <v>62821.824617452919</v>
+        <v>58840.37821436115</v>
       </c>
       <c r="AA8" s="4">
         <f>IF(Y8=0,0,Z8/Y8)</f>
-        <v>1.4933465524452799E-2</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="3">
-        <v>144170.4921208685</v>
+        <v>143913.1112629568</v>
       </c>
       <c r="AC8" s="3">
-        <v>257.38085791171761</v>
+        <v>235.6740385697631</v>
       </c>
       <c r="AD8" s="4">
         <f>IF(AB8=0,0,AC8/AB8)</f>
-        <v>1.7852533769249863E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30">
       <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="3">
         <f>J9+M9+G9+P9</f>
-        <v>120.33266759714401</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3">
         <f>G9</f>
-        <v>4.9528904426224756</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3">
         <f>J9+M9+P9</f>
-        <v>115.37977715452153</v>
+        <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>239.8280399304447</v>
+        <v>231.2949324342337</v>
       </c>
       <c r="G9" s="3">
-        <v>4.9528904426224756</v>
+        <v>4.584187797725841</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
-        <v>2.065184056067389E-2</v>
+        <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>2995.3735397304449</v>
+        <v>2992.321625738417</v>
       </c>
       <c r="J9" s="3">
-        <v>98.867443883899128</v>
+        <v>98.31675622033933</v>
       </c>
       <c r="K9" s="4">
         <f>IF(I9=0,0,J9/I9)</f>
-        <v>3.3006716048108065E-2</v>
+        <v>0</v>
       </c>
       <c r="L9" s="3">
-        <v>12350.65552086042</v>
+        <v>12338.37231628596</v>
       </c>
       <c r="M9" s="3">
-        <v>12.283204574460161</v>
+        <v>7.532925860725343</v>
       </c>
       <c r="N9" s="4">
         <f>IF(L9=0,0,M9/L9)</f>
-        <v>9.9453867478642454E-4</v>
+        <v>0</v>
       </c>
       <c r="O9" s="3">
-        <v>351.69146690818718</v>
+        <v>347.4623382120249</v>
       </c>
       <c r="P9" s="3">
-        <v>4.2291286961622534</v>
+        <v>4.333501334440312</v>
       </c>
       <c r="Q9" s="4">
         <f>IF(O9=0,0,P9/O9)</f>
-        <v>1.2025110342715004E-2</v>
+        <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>2665.998954727921</v>
+        <v>2571.142424723851</v>
       </c>
       <c r="T9" s="3">
-        <v>55.057785347964</v>
+        <v>50.95917842033032</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
-        <v>2.0651840560673786E-2</v>
+        <v>0</v>
       </c>
       <c r="V9" s="3">
-        <v>104895045.790185</v>
+        <v>104825402.4579278</v>
       </c>
       <c r="W9" s="3">
-        <v>2822333.3781914408</v>
+        <v>2816078.964827821</v>
       </c>
       <c r="X9" s="4">
         <f>IF(V9=0,0,W9/V9)</f>
-        <v>2.6906260032878746E-2</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="3">
-        <v>3782982.3163706479</v>
+        <v>3747214.466610681</v>
       </c>
       <c r="Z9" s="3">
-        <v>35767.849759967074</v>
+        <v>31907.42939718673</v>
       </c>
       <c r="AA9" s="4">
         <f>IF(Y9=0,0,Z9/Y9)</f>
-        <v>9.4549344323349525E-3</v>
+        <v>0</v>
       </c>
       <c r="AB9" s="3">
-        <v>137832.10087301829</v>
+        <v>137695.6580085831</v>
       </c>
       <c r="AC9" s="3">
-        <v>136.44286443514281</v>
+        <v>83.72630317611038</v>
       </c>
       <c r="AD9" s="4">
         <f>IF(AB9=0,0,AC9/AB9)</f>
-        <v>9.8992080633556216E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30">
       <c r="B12" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="3">
         <f>C14+C15+C16+C17+C18</f>
-        <v>1902.7902287937284</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3">
         <f>D14+D15+D16+D17+D18</f>
-        <v>594.698958422749</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3">
         <f>E14+E15+E16+E17+E18</f>
-        <v>1308.0912703709794</v>
+        <v>0</v>
       </c>
       <c r="F12" s="3">
         <f>F14+F15+F16+F17+F18</f>
-        <v>1581.0316281682187</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3">
         <f>G14+G15+G16+G17+G18</f>
-        <v>594.698958422749</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4">
         <f>IF(F12=0,0,G12/F12)</f>
-        <v>0.37614614902534649</v>
+        <v>0</v>
       </c>
       <c r="I12" s="3">
         <f>I14+I15+I16+I17+I18</f>
-        <v>18088.403478171738</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3">
         <f>J14+J15+J16+J17+J18</f>
-        <v>1119.1897188028731</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
         <f>IF(I12=0,0,J12/I12)</f>
-        <v>6.1873327856350635E-2</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3">
         <f>L14+L15+L16+L17+L18</f>
-        <v>73088.836931186815</v>
+        <v>0</v>
       </c>
       <c r="M12" s="3">
         <f>M14+M15+M16+M17+M18</f>
-        <v>151.25580362673105</v>
+        <v>0</v>
       </c>
       <c r="N12" s="4">
         <f>IF(L12=0,0,M12/L12)</f>
-        <v>2.0694788695179056E-3</v>
+        <v>0</v>
       </c>
       <c r="O12" s="3">
         <f>O14+O15+O16+O17+O18</f>
-        <v>2235.0590017749987</v>
+        <v>0</v>
       </c>
       <c r="P12" s="3">
         <f>P14+P15+P16+P17+P18</f>
-        <v>37.645747941375426</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="4">
         <f>IF(O12=0,0,P12/O12)</f>
-        <v>1.6843290450712312E-2</v>
+        <v>0</v>
       </c>
       <c r="S12" s="3">
         <f>S14+S15+S16+S17+S18</f>
-        <v>17575.212094927279</v>
+        <v>0</v>
       </c>
       <c r="T12" s="3">
         <f>T14+T15+T16+T17+T18</f>
-        <v>6610.8483478105873</v>
+        <v>0</v>
       </c>
       <c r="U12" s="4">
         <f>IF(S12=0,0,T12/S12)</f>
-        <v>0.37614614902534643</v>
+        <v>0</v>
       </c>
       <c r="V12" s="3">
         <f>V14+V15+V16+V17+V18</f>
-        <v>586984476.54622817</v>
+        <v>0</v>
       </c>
       <c r="W12" s="3">
         <f>W14+W15+W16+W17+W18</f>
-        <v>28560841.837795049</v>
+        <v>0</v>
       </c>
       <c r="X12" s="4">
         <f>IF(V12=0,0,W12/V12)</f>
-        <v>4.8656894652214421E-2</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="3">
         <f>Y14+Y15+Y16+Y17+Y18</f>
-        <v>24059700.626439646</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="3">
         <f>Z14+Z15+Z16+Z17+Z18</f>
-        <v>376108.59127695486</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="4">
         <f>IF(Y12=0,0,Z12/Y12)</f>
-        <v>1.5632305535158746E-2</v>
+        <v>0</v>
       </c>
       <c r="AB12" s="3">
         <f>AB14+AB15+AB16+AB17+AB18</f>
-        <v>815643.03969645977</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="3">
         <f>AC14+AC15+AC16+AC17+AC18</f>
-        <v>1680.7280119055067</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="4">
         <f>IF(AB12=0,0,AC12/AB12)</f>
-        <v>2.0606171206107356E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30">
       <c r="A13" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30">
       <c r="B14" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="3">
         <f>J14+M14+G14+P14</f>
-        <v>565.69219234731145</v>
+        <v>0</v>
       </c>
       <c r="D14" s="3">
         <f>G14</f>
-        <v>187.69467997746801</v>
+        <v>0</v>
       </c>
       <c r="E14" s="3">
         <f>J14+M14+P14</f>
-        <v>377.99751236984349</v>
+        <v>0</v>
       </c>
       <c r="F14" s="3">
-        <v>397.0902965307904</v>
+        <v>363.1566259346982</v>
       </c>
       <c r="G14" s="3">
-        <v>187.69467997746801</v>
+        <v>171.6550801719853</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
-        <v>0.47267506060278197</v>
+        <v>0</v>
       </c>
       <c r="I14" s="3">
-        <v>4229.0317579039856</v>
+        <v>4215.705028068518</v>
       </c>
       <c r="J14" s="3">
-        <v>312.83838520181371</v>
+        <v>311.1262929552929</v>
       </c>
       <c r="K14" s="4">
         <f>IF(I14=0,0,J14/I14)</f>
-        <v>7.3973997621825438E-2</v>
+        <v>0</v>
       </c>
       <c r="L14" s="3">
-        <v>18640.875795544409</v>
+        <v>18587.84837263764</v>
       </c>
       <c r="M14" s="3">
-        <v>53.027422906763853</v>
+        <v>48.27357658215985</v>
       </c>
       <c r="N14" s="4">
         <f>IF(L14=0,0,M14/L14)</f>
-        <v>2.8446851686785343E-3</v>
+        <v>0</v>
       </c>
       <c r="O14" s="3">
-        <v>603.60362214169209</v>
+        <v>591.4719178804262</v>
       </c>
       <c r="P14" s="3">
-        <v>12.131704261265931</v>
+        <v>9.426500014935039</v>
       </c>
       <c r="Q14" s="4">
         <f>IF(O14=0,0,P14/O14)</f>
-        <v>2.0098793009592129E-2</v>
+        <v>0</v>
       </c>
       <c r="S14" s="3">
-        <v>4414.1724036552041</v>
+        <v>4036.955751400944</v>
       </c>
       <c r="T14" s="3">
-        <v>2086.469208408852</v>
+        <v>1908.16830444419</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
-        <v>0.47267506060278208</v>
+        <v>0</v>
       </c>
       <c r="V14" s="3">
-        <v>130721936.6657657</v>
+        <v>130504106.3683567</v>
       </c>
       <c r="W14" s="3">
-        <v>7530151.3682035357</v>
+        <v>7529815.832129106</v>
       </c>
       <c r="X14" s="4">
         <f>IF(V14=0,0,W14/V14)</f>
-        <v>5.7604343695250498E-2</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="3">
-        <v>6174245.853177595</v>
+        <v>6056561.99351707</v>
       </c>
       <c r="Z14" s="3">
-        <v>117683.8596605249</v>
+        <v>113528.6322764717</v>
       </c>
       <c r="AA14" s="4">
         <f>IF(Y14=0,0,Z14/Y14)</f>
-        <v>1.9060442758358664E-2</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="3">
-        <v>208016.4497539358</v>
+        <v>207427.2646575113</v>
       </c>
       <c r="AC14" s="3">
-        <v>589.18509642445133</v>
+        <v>536.4685351653607</v>
       </c>
       <c r="AD14" s="4">
         <f>IF(AB14=0,0,AC14/AB14)</f>
-        <v>2.8323966547905356E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30">
       <c r="B15" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="3">
         <f>J15+M15+G15+P15</f>
-        <v>465.42086281069476</v>
+        <v>0</v>
       </c>
       <c r="D15" s="3">
         <f>G15</f>
-        <v>147.87505405504081</v>
+        <v>0</v>
       </c>
       <c r="E15" s="3">
         <f>J15+M15+P15</f>
-        <v>317.54580875565398</v>
+        <v>0</v>
       </c>
       <c r="F15" s="3">
-        <v>346.92132413597358</v>
+        <v>320.8109788943828</v>
       </c>
       <c r="G15" s="3">
-        <v>147.87505405504081</v>
+        <v>136.7455314648333</v>
       </c>
       <c r="H15" s="4">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.42624953776863289</v>
+        <v>0</v>
       </c>
       <c r="I15" s="3">
-        <v>3787.0627176324879</v>
+        <v>3777.348955767648</v>
       </c>
       <c r="J15" s="3">
-        <v>275.14154783459333</v>
+        <v>273.8748450018219</v>
       </c>
       <c r="K15" s="4">
         <f>IF(I15=0,0,J15/I15)</f>
-        <v>7.2653021180119307E-2</v>
+        <v>0</v>
       </c>
       <c r="L15" s="3">
-        <v>15402.279753726511</v>
+        <v>15367.67605497631</v>
       </c>
       <c r="M15" s="3">
-        <v>34.603698750201623</v>
+        <v>30.71036729697697</v>
       </c>
       <c r="N15" s="4">
         <f>IF(L15=0,0,M15/L15)</f>
-        <v>2.2466608387520957E-3</v>
+        <v>0</v>
       </c>
       <c r="O15" s="3">
-        <v>477.03495714807917</v>
+        <v>469.2343949772201</v>
       </c>
       <c r="P15" s="3">
-        <v>7.8005621708590773</v>
+        <v>6.561405479874811</v>
       </c>
       <c r="Q15" s="4">
         <f>IF(O15=0,0,P15/O15)</f>
-        <v>1.6352181436543361E-2</v>
+        <v>0</v>
       </c>
       <c r="S15" s="3">
-        <v>3856.4793665810321</v>
+        <v>3566.229097505511</v>
       </c>
       <c r="T15" s="3">
-        <v>1643.8225474194351</v>
+        <v>1520.103504388773</v>
       </c>
       <c r="U15" s="4">
         <f>IF(S15=0,0,T15/S15)</f>
-        <v>0.42624953776863289</v>
+        <v>0</v>
       </c>
       <c r="V15" s="3">
-        <v>121072766.34225529</v>
+        <v>120904784.0220684</v>
       </c>
       <c r="W15" s="3">
-        <v>6967680.9027350992</v>
+        <v>6963839.795960322</v>
       </c>
       <c r="X15" s="4">
         <f>IF(V15=0,0,W15/V15)</f>
-        <v>5.7549530858479497E-2</v>
+        <v>0</v>
       </c>
       <c r="Y15" s="3">
-        <v>5221398.5281040482</v>
+        <v>5132795.053668289</v>
       </c>
       <c r="Z15" s="3">
-        <v>88603.474435759708</v>
+        <v>85655.40422302578</v>
       </c>
       <c r="AA15" s="4">
         <f>IF(Y15=0,0,Z15/Y15)</f>
-        <v>1.6969299309151312E-2</v>
+        <v>0</v>
       </c>
       <c r="AB15" s="3">
-        <v>171868.3936012006</v>
+        <v>171483.8728014289</v>
       </c>
       <c r="AC15" s="3">
-        <v>384.52079977173707</v>
+        <v>341.1071610878571</v>
       </c>
       <c r="AD15" s="4">
         <f>IF(AB15=0,0,AC15/AB15)</f>
-        <v>2.2372979214780476E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30">
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="3">
         <f>J16+M16+G16+P16</f>
-        <v>390.69281904965561</v>
+        <v>0</v>
       </c>
       <c r="D16" s="3">
         <f>G16</f>
-        <v>117.07527770472841</v>
+        <v>0</v>
       </c>
       <c r="E16" s="3">
         <f>J16+M16+P16</f>
-        <v>273.61754134492719</v>
+        <v>0</v>
       </c>
       <c r="F16" s="3">
-        <v>308.40246775221379</v>
+        <v>288.0128603408813</v>
       </c>
       <c r="G16" s="3">
-        <v>117.07527770472841</v>
+        <v>109.3350058211387</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
-        <v>0.37961848540976212</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3">
-        <v>3695.2568384953711</v>
+        <v>3687.87367156503</v>
       </c>
       <c r="J16" s="3">
-        <v>238.32047450176211</v>
+        <v>237.3412499570018</v>
       </c>
       <c r="K16" s="4">
         <f>IF(I16=0,0,J16/I16)</f>
-        <v>6.44936157127311E-2</v>
+        <v>0</v>
       </c>
       <c r="L16" s="3">
-        <v>13777.53512556912</v>
+        <v>13749.34694539489</v>
       </c>
       <c r="M16" s="3">
-        <v>28.188180174233391</v>
+        <v>26.21495619864762</v>
       </c>
       <c r="N16" s="4">
         <f>IF(L16=0,0,M16/L16)</f>
-        <v>2.0459523359820865E-3</v>
+        <v>0</v>
       </c>
       <c r="O16" s="3">
-        <v>419.32297040011582</v>
+        <v>412.2140837311841</v>
       </c>
       <c r="P16" s="3">
-        <v>7.1088866689316932</v>
+        <v>3.678403565003595</v>
       </c>
       <c r="Q16" s="4">
         <f>IF(O16=0,0,P16/O16)</f>
-        <v>1.6953248857672715E-2</v>
+        <v>0</v>
       </c>
       <c r="S16" s="3">
-        <v>3428.292441957034</v>
+        <v>3201.635575388428</v>
       </c>
       <c r="T16" s="3">
-        <v>1301.4431843574639</v>
+        <v>1215.400047962967</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
-        <v>0.37961848540976206</v>
+        <v>0</v>
       </c>
       <c r="V16" s="3">
-        <v>118411700.21523701</v>
+        <v>118273982.4631039</v>
       </c>
       <c r="W16" s="3">
-        <v>6061904.1303865612</v>
+        <v>6057749.0648617</v>
       </c>
       <c r="X16" s="4">
         <f>IF(V16=0,0,W16/V16)</f>
-        <v>5.1193455708919262E-2</v>
+        <v>0</v>
       </c>
       <c r="Y16" s="3">
-        <v>4674292.5547931315</v>
+        <v>4603060.971989882</v>
       </c>
       <c r="Z16" s="3">
-        <v>71231.58280325029</v>
+        <v>67998.01526465267</v>
       </c>
       <c r="AA16" s="4">
         <f>IF(Y16=0,0,Z16/Y16)</f>
-        <v>1.5239008249538792E-2</v>
+        <v>0</v>
       </c>
       <c r="AB16" s="3">
-        <v>153755.60334743661</v>
+        <v>153442.4049540742</v>
       </c>
       <c r="AC16" s="3">
-        <v>313.19839336245792</v>
+        <v>291.4915740205033</v>
       </c>
       <c r="AD16" s="4">
         <f>IF(AB16=0,0,AC16/AB16)</f>
-        <v>2.036988483956149E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30">
       <c r="B17" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="3">
         <f>J17+M17+G17+P17</f>
-        <v>322.62345454430164</v>
+        <v>0</v>
       </c>
       <c r="D17" s="3">
         <f>G17</f>
-        <v>99.072823798268359</v>
+        <v>0</v>
       </c>
       <c r="E17" s="3">
         <f>J17+M17+P17</f>
-        <v>223.55063074603328</v>
+        <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>288.78949981879617</v>
+        <v>271.5819334790612</v>
       </c>
       <c r="G17" s="3">
-        <v>99.072823798268359</v>
+        <v>93.16955449989293</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
-        <v>0.3430624169522527</v>
+        <v>0</v>
       </c>
       <c r="I17" s="3">
-        <v>3381.6786244094469</v>
+        <v>3375.640124395373</v>
       </c>
       <c r="J17" s="3">
-        <v>194.02186738080479</v>
+        <v>193.1881464041606</v>
       </c>
       <c r="K17" s="4">
         <f>IF(I17=0,0,J17/I17)</f>
-        <v>5.7374425227851876E-2</v>
+        <v>0</v>
       </c>
       <c r="L17" s="3">
-        <v>12917.49073548635</v>
+        <v>12894.33743826528</v>
       </c>
       <c r="M17" s="3">
-        <v>23.15329722107202</v>
+        <v>21.20628217103705</v>
       </c>
       <c r="N17" s="4">
         <f>IF(L17=0,0,M17/L17)</f>
-        <v>1.7923989802033551E-3</v>
+        <v>0</v>
       </c>
       <c r="O17" s="3">
-        <v>383.40598517692439</v>
+        <v>377.0305190327679</v>
       </c>
       <c r="P17" s="3">
-        <v>6.3754661441564684</v>
+        <v>7.029277368942742</v>
       </c>
       <c r="Q17" s="4">
         <f>IF(O17=0,0,P17/O17)</f>
-        <v>1.6628499268769841E-2</v>
+        <v>0</v>
       </c>
       <c r="S17" s="3">
-        <v>3210.2689280060872</v>
+        <v>3018.984564891375</v>
       </c>
       <c r="T17" s="3">
-        <v>1101.3226175084851</v>
+        <v>1035.700141573183</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
-        <v>0.34306241695225254</v>
+        <v>0</v>
       </c>
       <c r="V17" s="3">
-        <v>111883027.5327851</v>
+        <v>111762860.6181328</v>
       </c>
       <c r="W17" s="3">
-        <v>5178772.0582784116</v>
+        <v>5173153.551915213</v>
       </c>
       <c r="X17" s="4">
         <f>IF(V17=0,0,W17/V17)</f>
-        <v>4.6287378635341943E-2</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="3">
-        <v>4206781.3739942238</v>
+        <v>4143959.549376771</v>
       </c>
       <c r="Z17" s="3">
-        <v>62821.824617452919</v>
+        <v>58840.37821436115</v>
       </c>
       <c r="AA17" s="4">
         <f>IF(Y17=0,0,Z17/Y17)</f>
-        <v>1.4933465524452799E-2</v>
+        <v>0</v>
       </c>
       <c r="AB17" s="3">
-        <v>144170.4921208685</v>
+        <v>143913.1112629568</v>
       </c>
       <c r="AC17" s="3">
-        <v>257.38085791171761</v>
+        <v>235.6740385697631</v>
       </c>
       <c r="AD17" s="4">
         <f>IF(AB17=0,0,AC17/AB17)</f>
-        <v>1.7852533769249863E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30">
       <c r="B18" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="3">
         <f>J18+M18+G18+P18</f>
-        <v>158.36090004176489</v>
+        <v>0</v>
       </c>
       <c r="D18" s="3">
         <f>G18</f>
-        <v>42.981122887243338</v>
+        <v>0</v>
       </c>
       <c r="E18" s="3">
         <f>J18+M18+P18</f>
-        <v>115.37977715452153</v>
+        <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>239.8280399304447</v>
+        <v>231.2949324342337</v>
       </c>
       <c r="G18" s="3">
-        <v>42.981122887243338</v>
+        <v>41.4518499047723</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
-        <v>0.17921642064751389</v>
+        <v>0</v>
       </c>
       <c r="I18" s="3">
-        <v>2995.3735397304449</v>
+        <v>2992.321625738417</v>
       </c>
       <c r="J18" s="3">
-        <v>98.867443883899128</v>
+        <v>98.31675622033933</v>
       </c>
       <c r="K18" s="4">
         <f>IF(I18=0,0,J18/I18)</f>
-        <v>3.3006716048108065E-2</v>
+        <v>0</v>
       </c>
       <c r="L18" s="3">
-        <v>12350.65552086042</v>
+        <v>12338.37231628596</v>
       </c>
       <c r="M18" s="3">
-        <v>12.283204574460161</v>
+        <v>7.532925860725343</v>
       </c>
       <c r="N18" s="4">
         <f>IF(L18=0,0,M18/L18)</f>
-        <v>9.9453867478642454E-4</v>
+        <v>0</v>
       </c>
       <c r="O18" s="3">
-        <v>351.69146690818718</v>
+        <v>347.4623382120249</v>
       </c>
       <c r="P18" s="3">
-        <v>4.2291286961622534</v>
+        <v>4.333501334440312</v>
       </c>
       <c r="Q18" s="4">
         <f>IF(O18=0,0,P18/O18)</f>
-        <v>1.2025110342715004E-2</v>
+        <v>0</v>
       </c>
       <c r="S18" s="3">
-        <v>2665.998954727921</v>
+        <v>2571.142424723851</v>
       </c>
       <c r="T18" s="3">
-        <v>477.79079011635167</v>
+        <v>460.7909423339825</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
-        <v>0.17921642064751397</v>
+        <v>0</v>
       </c>
       <c r="V18" s="3">
-        <v>104895045.790185</v>
+        <v>104825402.4579278</v>
       </c>
       <c r="W18" s="3">
-        <v>2822333.3781914408</v>
+        <v>2816078.964827821</v>
       </c>
       <c r="X18" s="4">
         <f>IF(V18=0,0,W18/V18)</f>
-        <v>2.6906260032878746E-2</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="3">
-        <v>3782982.3163706479</v>
+        <v>3747214.466610681</v>
       </c>
       <c r="Z18" s="3">
-        <v>35767.849759967074</v>
+        <v>31907.42939718673</v>
       </c>
       <c r="AA18" s="4">
         <f>IF(Y18=0,0,Z18/Y18)</f>
-        <v>9.4549344323349525E-3</v>
+        <v>0</v>
       </c>
       <c r="AB18" s="3">
-        <v>137832.10087301829</v>
+        <v>137695.6580085831</v>
       </c>
       <c r="AC18" s="3">
-        <v>136.44286443514281</v>
+        <v>83.72630317611038</v>
       </c>
       <c r="AD18" s="4">
         <f>IF(AB18=0,0,AC18/AB18)</f>
-        <v>9.8992080633556216E-4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30">
       <c r="A20" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30">
       <c r="B21" t="s">
         <v>28</v>
       </c>
       <c r="C21" s="3">
         <f>C23+C24+C25+C26+C27</f>
-        <v>2011.3640256098345</v>
+        <v>0</v>
       </c>
       <c r="D21" s="3">
         <f>D23+D24+D25+D26+D27</f>
-        <v>1075.1027820881886</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3">
         <f>E23+E24+E25+E26+E27</f>
-        <v>936.26124352164572</v>
+        <v>0</v>
       </c>
       <c r="F21" s="3">
         <f>F23+F24+F25+F26+F27</f>
-        <v>1921.9196808294905</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3">
         <f>G23+G24+G25+G26+G27</f>
-        <v>1075.1027820881886</v>
+        <v>0</v>
       </c>
       <c r="H21" s="4">
         <f>IF(F21=0,0,G21/F21)</f>
-        <v>0.55939006859234608</v>
+        <v>0</v>
       </c>
       <c r="I21" s="3">
         <f>I23+I24+I25+I26+I27</f>
-        <v>3682.4352162782898</v>
+        <v>0</v>
       </c>
       <c r="J21" s="3">
         <f>J23+J24+J25+J26+J27</f>
-        <v>585.89953258422668</v>
+        <v>0</v>
       </c>
       <c r="K21" s="4">
         <f>IF(I21=0,0,J21/I21)</f>
-        <v>0.15910654177818098</v>
+        <v>0</v>
       </c>
       <c r="L21" s="3">
         <f>L23+L24+L25+L26+L27</f>
-        <v>75120.106151105079</v>
+        <v>0</v>
       </c>
       <c r="M21" s="3">
         <f>M23+M24+M25+M26+M27</f>
-        <v>270.09622799380867</v>
+        <v>0</v>
       </c>
       <c r="N21" s="4">
         <f>IF(L21=0,0,M21/L21)</f>
-        <v>3.5955251108206179E-3</v>
+        <v>0</v>
       </c>
       <c r="O21" s="3">
         <f>O23+O24+O25+O26+O27</f>
-        <v>1936.1737568351107</v>
+        <v>0</v>
       </c>
       <c r="P21" s="3">
         <f>P23+P24+P25+P26+P27</f>
-        <v>80.265482943610337</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="4">
         <f>IF(O21=0,0,P21/O21)</f>
-        <v>4.1455723000198653E-2</v>
+        <v>0</v>
       </c>
       <c r="S21" s="3">
         <f>S23+S24+S25+S26+S27</f>
-        <v>21364.623843185575</v>
+        <v>0</v>
       </c>
       <c r="T21" s="3">
         <f>T23+T24+T25+T26+T27</f>
-        <v>11951.158397089252</v>
+        <v>0</v>
       </c>
       <c r="U21" s="4">
         <f>IF(S21=0,0,T21/S21)</f>
-        <v>0.55939006859234608</v>
+        <v>0</v>
       </c>
       <c r="V21" s="3">
         <f>V23+V24+V25+V26+V27</f>
-        <v>106670224.92367341</v>
+        <v>0</v>
       </c>
       <c r="W21" s="3">
         <f>W23+W24+W25+W26+W27</f>
-        <v>13782093.295542261</v>
+        <v>0</v>
       </c>
       <c r="X21" s="4">
         <f>IF(V21=0,0,W21/V21)</f>
-        <v>0.12920281461301755</v>
+        <v>0</v>
       </c>
       <c r="Y21" s="3">
         <f>Y23+Y24+Y25+Y26+Y27</f>
-        <v>8082003.8383214176</v>
+        <v>0</v>
       </c>
       <c r="Z21" s="3">
         <f>Z23+Z24+Z25+Z26+Z27</f>
-        <v>334084.07649866142</v>
+        <v>0</v>
       </c>
       <c r="AA21" s="4">
         <f>IF(Y21=0,0,Z21/Y21)</f>
-        <v>4.1336787655875284E-2</v>
+        <v>0</v>
       </c>
       <c r="AB21" s="3">
         <f>AB23+AB24+AB25+AB26+AB27</f>
-        <v>844449.53447731666</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="3">
         <f>AC23+AC24+AC25+AC26+AC27</f>
-        <v>2999.0317686344206</v>
+        <v>0</v>
       </c>
       <c r="AD21" s="4">
         <f>IF(AB21=0,0,AC21/AB21)</f>
-        <v>3.5514635821200509E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30">
       <c r="A22" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30">
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="3">
         <f>J23+M23+G23+P23</f>
-        <v>525.35232482572508</v>
+        <v>0</v>
       </c>
       <c r="D23" s="3">
         <f>G23</f>
-        <v>277.48144279559921</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3">
         <f>J23+M23+P23</f>
-        <v>247.87088203012584</v>
+        <v>0</v>
       </c>
       <c r="F23" s="3">
-        <v>428.09244082133358</v>
+        <v>413.6052490085787</v>
       </c>
       <c r="G23" s="3">
-        <v>277.48144279559921</v>
+        <v>268.406433964483</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
-        <v>0.64818113177431091</v>
+        <v>0</v>
       </c>
       <c r="I23" s="3">
-        <v>991.82050542122556</v>
+        <v>991.8205054212256</v>
       </c>
       <c r="J23" s="3">
-        <v>137.38025624613479</v>
+        <v>137.3802562461348</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
-        <v>0.13851322441432029</v>
+        <v>0</v>
       </c>
       <c r="L23" s="3">
-        <v>18248.150900694091</v>
+        <v>18248.15090069409</v>
       </c>
       <c r="M23" s="3">
-        <v>92.706822166558354</v>
+        <v>92.70682216655835</v>
       </c>
       <c r="N23" s="4">
         <f>IF(L23=0,0,M23/L23)</f>
-        <v>5.0803406148418103E-3</v>
+        <v>0</v>
       </c>
       <c r="O23" s="3">
-        <v>476.04818802351332</v>
+        <v>476.0481880235133</v>
       </c>
       <c r="P23" s="3">
         <v>17.78380361743271</v>
       </c>
       <c r="Q23" s="4">
         <f>IF(O23=0,0,P23/O23)</f>
-        <v>3.7357150105472768E-2</v>
+        <v>0</v>
       </c>
       <c r="S23" s="3">
-        <v>4758.8013481976486</v>
+        <v>4597.75746758657</v>
       </c>
       <c r="T23" s="3">
-        <v>3084.5652437638678</v>
+        <v>2983.684779307255</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
-        <v>0.6481811317743108</v>
+        <v>0</v>
       </c>
       <c r="V23" s="3">
-        <v>25699987.560610589</v>
+        <v>25699987.56061059</v>
       </c>
       <c r="W23" s="3">
-        <v>2724438.1987594548</v>
+        <v>2724438.198759455</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
-        <v>0.10600931974516203</v>
+        <v>0</v>
       </c>
       <c r="Y23" s="3">
-        <v>1959206.3612258229</v>
+        <v>1959206.361225823</v>
       </c>
       <c r="Z23" s="3">
-        <v>81685.476824872196</v>
+        <v>81685.4768248722</v>
       </c>
       <c r="AA23" s="4">
         <f>IF(Y23=0,0,Z23/Y23)</f>
-        <v>4.1693145980683619E-2</v>
+        <v>0</v>
       </c>
       <c r="AB23" s="3">
-        <v>205054.68928072241</v>
+        <v>205054.6892807224</v>
       </c>
       <c r="AC23" s="3">
-        <v>1029.3601439886841</v>
+        <v>1029.360143988684</v>
       </c>
       <c r="AD23" s="4">
         <f>IF(AB23=0,0,AC23/AB23)</f>
-        <v>5.0199297933610151E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30">
       <c r="B24" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="3">
         <f>J24+M24+G24+P24</f>
-        <v>502.10011734093223</v>
+        <v>0</v>
       </c>
       <c r="D24" s="3">
         <f>G24</f>
-        <v>273.77050166811682</v>
+        <v>0</v>
       </c>
       <c r="E24" s="3">
         <f>J24+M24+P24</f>
-        <v>228.32961567281538</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>437.75116549754102</v>
+        <v>422.9371101765626</v>
       </c>
       <c r="G24" s="3">
-        <v>273.77050166811682</v>
+        <v>264.8490662071024</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
-        <v>0.62540210796915552</v>
+        <v>0</v>
       </c>
       <c r="I24" s="3">
-        <v>847.52939170447485</v>
+        <v>847.5293917044748</v>
       </c>
       <c r="J24" s="3">
-        <v>129.63861091745869</v>
+        <v>129.6386109174587</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
-        <v>0.15296060784009058</v>
+        <v>0</v>
       </c>
       <c r="L24" s="3">
         <v>18442.648959675</v>
       </c>
       <c r="M24" s="3">
-        <v>78.360818720057608</v>
+        <v>78.36081872005761</v>
       </c>
       <c r="N24" s="4">
         <f>IF(L24=0,0,M24/L24)</f>
-        <v>4.2488917341209588E-3</v>
+        <v>0</v>
       </c>
       <c r="O24" s="3">
-        <v>476.56393826290048</v>
+        <v>476.5639382629005</v>
       </c>
       <c r="P24" s="3">
-        <v>20.330186035299089</v>
+        <v>20.33018603529909</v>
       </c>
       <c r="Q24" s="4">
         <f>IF(O24=0,0,P24/O24)</f>
-        <v>4.2659933752863553E-2</v>
+        <v>0</v>
       </c>
       <c r="S24" s="3">
-        <v>4866.1705694873763</v>
+        <v>4701.493178084503</v>
       </c>
       <c r="T24" s="3">
-        <v>3043.3133318948712</v>
+        <v>2944.140034141051</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
-        <v>0.62540210796915552</v>
+        <v>0</v>
       </c>
       <c r="V24" s="3">
-        <v>23322467.600951109</v>
+        <v>23322467.60095111</v>
       </c>
       <c r="W24" s="3">
-        <v>2821008.1417387952</v>
+        <v>2821008.141738795</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
-        <v>0.12095667534012362</v>
+        <v>0</v>
       </c>
       <c r="Y24" s="3">
-        <v>2033978.1299748039</v>
+        <v>2033978.129974804</v>
       </c>
       <c r="Z24" s="3">
-        <v>83922.171154072974</v>
+        <v>83922.17115407297</v>
       </c>
       <c r="AA24" s="4">
         <f>IF(Y24=0,0,Z24/Y24)</f>
-        <v>4.1260114805222889E-2</v>
+        <v>0</v>
       </c>
       <c r="AB24" s="3">
-        <v>207305.28823611679</v>
+        <v>207305.2882361168</v>
       </c>
       <c r="AC24" s="3">
-        <v>870.34467375359964</v>
+        <v>870.3446737535996</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(AB24=0,0,AC24/AB24)</f>
-        <v>4.1983717885782706E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30">
       <c r="B25" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="3">
         <f>J25+M25+G25+P25</f>
-        <v>397.67985371592215</v>
+        <v>0</v>
       </c>
       <c r="D25" s="3">
         <f>G25</f>
-        <v>214.2843575815979</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3">
         <f>J25+M25+P25</f>
-        <v>183.39549613432428</v>
+        <v>0</v>
       </c>
       <c r="F25" s="3">
-        <v>396.28526128416758</v>
+        <v>382.8744648174589</v>
       </c>
       <c r="G25" s="3">
-        <v>214.2843575815979</v>
+        <v>207.4137355149925</v>
       </c>
       <c r="H25" s="4">
         <f>IF(F25=0,0,G25/F25)</f>
-        <v>0.54073259471524793</v>
+        <v>0</v>
       </c>
       <c r="I25" s="3">
-        <v>721.62080381298233</v>
+        <v>721.6208038129823</v>
       </c>
       <c r="J25" s="3">
         <v>117.9993820939182</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
-        <v>0.16351992829255976</v>
+        <v>0</v>
       </c>
       <c r="L25" s="3">
-        <v>15355.961975565249</v>
+        <v>15355.96197556525</v>
       </c>
       <c r="M25" s="3">
-        <v>48.616281052693722</v>
+        <v>48.61628105269372</v>
       </c>
       <c r="N25" s="4">
         <f>IF(L25=0,0,M25/L25)</f>
-        <v>3.1659547692325001E-3</v>
+        <v>0</v>
       </c>
       <c r="O25" s="3">
         <v>391.5266582641886</v>
@@ -2338,221 +2309,221 @@
       </c>
       <c r="Q25" s="4">
         <f>IF(O25=0,0,P25/O25)</f>
-        <v>4.2857446954199227E-2</v>
+        <v>0</v>
       </c>
       <c r="S25" s="3">
-        <v>4405.2233953297473</v>
+        <v>4256.145041636478</v>
       </c>
       <c r="T25" s="3">
-        <v>2382.0478768569678</v>
+        <v>2305.6720233362</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
-        <v>0.54073259471524771</v>
+        <v>0</v>
       </c>
       <c r="V25" s="3">
-        <v>21162807.846375171</v>
+        <v>21162807.84637517</v>
       </c>
       <c r="W25" s="3">
-        <v>2800683.8604466021</v>
+        <v>2800683.860446602</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
-        <v>0.13233989935443805</v>
+        <v>0</v>
       </c>
       <c r="Y25" s="3">
         <v>1664123.912966297</v>
       </c>
       <c r="Z25" s="3">
-        <v>70162.630031719338</v>
+        <v>70162.63003171934</v>
       </c>
       <c r="AA25" s="4">
         <f>IF(Y25=0,0,Z25/Y25)</f>
-        <v>4.2161902419066026E-2</v>
+        <v>0</v>
       </c>
       <c r="AB25" s="3">
         <v>172634.6152091868</v>
       </c>
       <c r="AC25" s="3">
-        <v>539.59249566448852</v>
+        <v>539.5924956644885</v>
       </c>
       <c r="AD25" s="4">
         <f>IF(AB25=0,0,AC25/AB25)</f>
-        <v>3.1256332631242425E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30">
       <c r="B26" t="s">
         <v>33</v>
       </c>
       <c r="C26" s="3">
         <f>J26+M26+G26+P26</f>
-        <v>325.4816190604223</v>
+        <v>0</v>
       </c>
       <c r="D26" s="3">
         <f>G26</f>
-        <v>169.09086715748001</v>
+        <v>0</v>
       </c>
       <c r="E26" s="3">
         <f>J26+M26+P26</f>
-        <v>156.39075190294236</v>
+        <v>0</v>
       </c>
       <c r="F26" s="3">
-        <v>351.26672270713158</v>
+        <v>339.3794107528897</v>
       </c>
       <c r="G26" s="3">
-        <v>169.09086715748001</v>
+        <v>163.7500164709789</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
-        <v>0.48137456874461582</v>
+        <v>0</v>
       </c>
       <c r="I26" s="3">
-        <v>656.23600296293523</v>
+        <v>656.2360029629352</v>
       </c>
       <c r="J26" s="3">
         <v>111.9114792464019</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
-        <v>0.17053541521817839</v>
+        <v>0</v>
       </c>
       <c r="L26" s="3">
-        <v>12320.893910346331</v>
+        <v>12320.89391034633</v>
       </c>
       <c r="M26" s="3">
-        <v>30.922360504940151</v>
+        <v>30.92236050494015</v>
       </c>
       <c r="N26" s="4">
         <f>IF(L26=0,0,M26/L26)</f>
-        <v>2.5097497576026888E-3</v>
+        <v>0</v>
       </c>
       <c r="O26" s="3">
-        <v>305.89771512841492</v>
+        <v>305.8977151284149</v>
       </c>
       <c r="P26" s="3">
         <v>13.55691215160029</v>
       </c>
       <c r="Q26" s="4">
         <f>IF(O26=0,0,P26/O26)</f>
-        <v>4.4318448556927403E-2</v>
+        <v>0</v>
       </c>
       <c r="S26" s="3">
-        <v>3904.7840938011818</v>
+        <v>3772.641241557029</v>
       </c>
       <c r="T26" s="3">
-        <v>1879.66375919438</v>
+        <v>1820.293293790503</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
-        <v>0.48137456874461598</v>
+        <v>0</v>
       </c>
       <c r="V26" s="3">
-        <v>20232379.411657181</v>
+        <v>20232379.41165718</v>
       </c>
       <c r="W26" s="3">
         <v>2815905.181914039</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
-        <v>0.13917815223905963</v>
+        <v>0</v>
       </c>
       <c r="Y26" s="3">
-        <v>1291512.2728871789</v>
+        <v>1291512.272887179</v>
       </c>
       <c r="Z26" s="3">
-        <v>51650.776301899918</v>
+        <v>51650.77630189992</v>
       </c>
       <c r="AA26" s="4">
         <f>IF(Y26=0,0,Z26/Y26)</f>
-        <v>3.9992478109739119E-2</v>
+        <v>0</v>
       </c>
       <c r="AB26" s="3">
-        <v>138538.51808137319</v>
+        <v>138538.5180813732</v>
       </c>
       <c r="AC26" s="3">
         <v>343.4734157078783</v>
       </c>
       <c r="AD26" s="4">
         <f>IF(AB26=0,0,AC26/AB26)</f>
-        <v>2.479262954914335E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30">
       <c r="B27" t="s">
         <v>34</v>
       </c>
       <c r="C27" s="3">
         <f>J27+M27+G27+P27</f>
-        <v>260.75011066683265</v>
+        <v>0</v>
       </c>
       <c r="D27" s="3">
         <f>G27</f>
-        <v>140.47561288539481</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3">
         <f>J27+M27+P27</f>
-        <v>120.27449778143787</v>
+        <v>0</v>
       </c>
       <c r="F27" s="3">
-        <v>308.52409051931693</v>
+        <v>298.0832435152593</v>
       </c>
       <c r="G27" s="3">
-        <v>140.47561288539481</v>
+        <v>136.0735620028871</v>
       </c>
       <c r="H27" s="4">
         <f>IF(F27=0,0,G27/F27)</f>
-        <v>0.4553148917769827</v>
+        <v>0</v>
       </c>
       <c r="I27" s="3">
-        <v>465.22851237667129</v>
+        <v>465.2285123766713</v>
       </c>
       <c r="J27" s="3">
-        <v>88.969804080313125</v>
+        <v>88.96980408031312</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
-        <v>0.19123893251039376</v>
+        <v>0</v>
       </c>
       <c r="L27" s="3">
-        <v>10752.450404824391</v>
+        <v>10752.45040482439</v>
       </c>
       <c r="M27" s="3">
-        <v>19.489945549558851</v>
+        <v>19.48994554955885</v>
       </c>
       <c r="N27" s="4">
         <f>IF(L27=0,0,M27/L27)</f>
-        <v>1.8126050170679359E-3</v>
+        <v>0</v>
       </c>
       <c r="O27" s="3">
-        <v>286.13725715609343</v>
+        <v>286.1372571560934</v>
       </c>
       <c r="P27" s="3">
-        <v>11.814748151565899</v>
+        <v>11.8147481515659</v>
       </c>
       <c r="Q27" s="4">
         <f>IF(O27=0,0,P27/O27)</f>
-        <v>4.12904920840865E-2</v>
+        <v>0</v>
       </c>
       <c r="S27" s="3">
-        <v>3429.6444363696219</v>
+        <v>3313.580913491462</v>
       </c>
       <c r="T27" s="3">
-        <v>1561.568185379165</v>
+        <v>1512.633694421276</v>
       </c>
       <c r="U27" s="4">
         <f>IF(S27=0,0,T27/S27)</f>
-        <v>0.45531489177698264</v>
+        <v>0</v>
       </c>
       <c r="V27" s="3">
-        <v>16252582.504079361</v>
+        <v>16252582.50407936</v>
       </c>
       <c r="W27" s="3">
-        <v>2620057.9126833701</v>
+        <v>2620057.91268337</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
-        <v>0.16120871326299938</v>
+        <v>0</v>
       </c>
       <c r="Y27" s="3">
         <v>1133183.161267315</v>
@@ -2562,274 +2533,274 @@
       </c>
       <c r="AA27" s="4">
         <f>IF(Y27=0,0,Z27/Y27)</f>
-        <v>4.1178711245506497E-2</v>
+        <v>0</v>
       </c>
       <c r="AB27" s="3">
-        <v>120916.42366991749</v>
+        <v>120916.4236699175</v>
       </c>
       <c r="AC27" s="3">
-        <v>216.26103951976981</v>
+        <v>216.2610395197698</v>
       </c>
       <c r="AD27" s="4">
         <f>IF(AB27=0,0,AC27/AB27)</f>
-        <v>1.7885166709042592E-3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30">
       <c r="A29" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30">
       <c r="B30" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="3">
         <f>C32+C33+C34+C35+C36</f>
-        <v>283.3332129957933</v>
+        <v>0</v>
       </c>
       <c r="D30" s="3">
         <f>D32+D33+D34+D35+D36</f>
-        <v>192.3778145952281</v>
+        <v>0</v>
       </c>
       <c r="E30" s="3">
         <f>E32+E33+E34+E35+E36</f>
-        <v>90.955398400565215</v>
+        <v>0</v>
       </c>
       <c r="F30" s="3">
         <f>F32+F33+F34+F35+F36</f>
-        <v>1921.9196808294905</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3">
         <f>G32+G33+G34+G35+G36</f>
-        <v>192.3778145952281</v>
+        <v>0</v>
       </c>
       <c r="H30" s="4">
         <f>IF(F30=0,0,G30/F30)</f>
-        <v>0.10009669837617712</v>
+        <v>0</v>
       </c>
       <c r="I30" s="3">
         <f>I32+I33+I34+I35+I36</f>
-        <v>3682.4352162782898</v>
+        <v>0</v>
       </c>
       <c r="J30" s="3">
         <f>J32+J33+J34+J35+J36</f>
-        <v>73.986991036804866</v>
+        <v>0</v>
       </c>
       <c r="K30" s="4">
         <f>IF(I30=0,0,J30/I30)</f>
-        <v>2.0091864945714095E-2</v>
+        <v>0</v>
       </c>
       <c r="L30" s="3">
         <f>L32+L33+L34+L35+L36</f>
-        <v>75120.106151105079</v>
+        <v>0</v>
       </c>
       <c r="M30" s="3">
         <f>M32+M33+M34+M35+M36</f>
-        <v>7.7175543162524711</v>
+        <v>0</v>
       </c>
       <c r="N30" s="4">
         <f>IF(L30=0,0,M30/L30)</f>
-        <v>1.0273620088779572E-4</v>
+        <v>0</v>
       </c>
       <c r="O30" s="3">
         <f>O32+O33+O34+O35+O36</f>
-        <v>1936.1737568351107</v>
+        <v>0</v>
       </c>
       <c r="P30" s="3">
         <f>P32+P33+P34+P35+P36</f>
-        <v>9.2508530475078743</v>
+        <v>0</v>
       </c>
       <c r="Q30" s="4">
         <f>IF(O30=0,0,P30/O30)</f>
-        <v>4.7779043667183123E-3</v>
+        <v>0</v>
       </c>
       <c r="S30" s="3">
         <f>S32+S33+S34+S35+S36</f>
-        <v>21364.623843185575</v>
+        <v>0</v>
       </c>
       <c r="T30" s="3">
         <f>T32+T33+T34+T35+T36</f>
-        <v>2138.5283087518278</v>
+        <v>0</v>
       </c>
       <c r="U30" s="4">
         <f>IF(S30=0,0,T30/S30)</f>
-        <v>0.10009669837617709</v>
+        <v>0</v>
       </c>
       <c r="V30" s="3">
         <f>V32+V33+V34+V35+V36</f>
-        <v>106670224.92367341</v>
+        <v>0</v>
       </c>
       <c r="W30" s="3">
         <f>W32+W33+W34+W35+W36</f>
-        <v>1767252.4081023186</v>
+        <v>0</v>
       </c>
       <c r="X30" s="4">
         <f>IF(V30=0,0,W30/V30)</f>
-        <v>1.6567438658415267E-2</v>
+        <v>0</v>
       </c>
       <c r="Y30" s="3">
         <f>Y32+Y33+Y34+Y35+Y36</f>
-        <v>8082003.8383214176</v>
+        <v>0</v>
       </c>
       <c r="Z30" s="3">
         <f>Z32+Z33+Z34+Z35+Z36</f>
-        <v>39755.677394214319</v>
+        <v>0</v>
       </c>
       <c r="AA30" s="4">
         <f>IF(Y30=0,0,Z30/Y30)</f>
-        <v>4.9190371830448582E-3</v>
+        <v>0</v>
       </c>
       <c r="AB30" s="3">
         <f>AB32+AB33+AB34+AB35+AB36</f>
-        <v>844449.53447731666</v>
+        <v>0</v>
       </c>
       <c r="AC30" s="3">
         <f>AC32+AC33+AC34+AC35+AC36</f>
-        <v>85.868353927085991</v>
+        <v>0</v>
       </c>
       <c r="AD30" s="4">
         <f>IF(AB30=0,0,AC30/AB30)</f>
-        <v>1.0168559567059903E-4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30">
       <c r="A31" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30">
       <c r="B32" t="s">
         <v>30</v>
       </c>
       <c r="C32" s="3">
         <f>J32+M32+G32+P32</f>
-        <v>31.154475954145141</v>
+        <v>0</v>
       </c>
       <c r="D32" s="3">
         <f>G32</f>
-        <v>17.026035953983609</v>
+        <v>0</v>
       </c>
       <c r="E32" s="3">
         <f>J32+M32+P32</f>
-        <v>14.128440000161532</v>
+        <v>0</v>
       </c>
       <c r="F32" s="3">
-        <v>428.09244082133358</v>
+        <v>413.6052490085787</v>
       </c>
       <c r="G32" s="3">
-        <v>17.026035953983609</v>
+        <v>17.31045199131634</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
-        <v>3.9771867780046849E-2</v>
+        <v>0</v>
       </c>
       <c r="I32" s="3">
-        <v>991.82050542122556</v>
+        <v>991.8205054212256</v>
       </c>
       <c r="J32" s="3">
         <v>11.67126541163598</v>
       </c>
       <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
-        <v>1.1767517759354251E-2</v>
+        <v>0</v>
       </c>
       <c r="L32" s="3">
-        <v>18248.150900694091</v>
+        <v>18248.15090069409</v>
       </c>
       <c r="M32" s="3">
-        <v>1.0535630249716339</v>
+        <v>1.053563024971634</v>
       </c>
       <c r="N32" s="4">
         <f>IF(L32=0,0,M32/L32)</f>
-        <v>5.773533059349922E-5</v>
+        <v>0</v>
       </c>
       <c r="O32" s="3">
-        <v>476.04818802351332</v>
+        <v>476.0481880235133</v>
       </c>
       <c r="P32" s="3">
         <v>1.403611563553917</v>
       </c>
       <c r="Q32" s="4">
         <f>IF(O32=0,0,P32/O32)</f>
-        <v>2.9484653000813204E-3</v>
+        <v>0</v>
       </c>
       <c r="S32" s="3">
-        <v>4758.8013481976486</v>
+        <v>4597.75746758657</v>
       </c>
       <c r="T32" s="3">
-        <v>189.2664180120255</v>
+        <v>192.4280702460892</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
-        <v>3.9771867780046835E-2</v>
+        <v>0</v>
       </c>
       <c r="V32" s="3">
-        <v>25699987.560610589</v>
+        <v>25699987.56061059</v>
       </c>
       <c r="W32" s="3">
-        <v>227272.75268540901</v>
+        <v>227272.752685409</v>
       </c>
       <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
-        <v>8.8433020502212793E-3</v>
+        <v>0</v>
       </c>
       <c r="Y32" s="3">
-        <v>1959206.3612258229</v>
+        <v>1959206.361225823</v>
       </c>
       <c r="Z32" s="3">
-        <v>6013.3033886032636</v>
+        <v>6013.303388603264</v>
       </c>
       <c r="AA32" s="4">
         <f>IF(Y32=0,0,Z32/Y32)</f>
-        <v>3.0692547286549749E-3</v>
+        <v>0</v>
       </c>
       <c r="AB32" s="3">
-        <v>205054.68928072241</v>
+        <v>205054.6892807224</v>
       </c>
       <c r="AC32" s="3">
         <v>11.66113448393298</v>
       </c>
       <c r="AD32" s="4">
         <f>IF(AB32=0,0,AC32/AB32)</f>
-        <v>5.686841166538134E-5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:30">
       <c r="B33" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="3">
         <f>J33+M33+G33+P33</f>
-        <v>51.454722558748443</v>
+        <v>0</v>
       </c>
       <c r="D33" s="3">
         <f>G33</f>
-        <v>33.74848177556315</v>
+        <v>0</v>
       </c>
       <c r="E33" s="3">
         <f>J33+M33+P33</f>
-        <v>17.706240783185294</v>
+        <v>0</v>
       </c>
       <c r="F33" s="3">
-        <v>437.75116549754102</v>
+        <v>422.9371101765626</v>
       </c>
       <c r="G33" s="3">
-        <v>33.74848177556315</v>
+        <v>33.45220057492261</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
-        <v>7.7095127176201025E-2</v>
+        <v>0</v>
       </c>
       <c r="I33" s="3">
-        <v>847.52939170447485</v>
+        <v>847.5293917044748</v>
       </c>
       <c r="J33" s="3">
         <v>14.3231196181163</v>
       </c>
       <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
-        <v>1.6899850032706158E-2</v>
+        <v>0</v>
       </c>
       <c r="L33" s="3">
         <v>18442.648959675</v>
@@ -2839,104 +2810,104 @@
       </c>
       <c r="N33" s="4">
         <f>IF(L33=0,0,M33/L33)</f>
-        <v>9.2629689549605278E-5</v>
+        <v>0</v>
       </c>
       <c r="O33" s="3">
-        <v>476.56393826290048</v>
+        <v>476.5639382629005</v>
       </c>
       <c r="P33" s="3">
-        <v>1.6747843174619479</v>
+        <v>1.674784317461948</v>
       </c>
       <c r="Q33" s="4">
         <f>IF(O33=0,0,P33/O33)</f>
-        <v>3.514290912498795E-3</v>
+        <v>0</v>
       </c>
       <c r="S33" s="3">
-        <v>4866.1705694873763</v>
+        <v>4701.493178084503</v>
       </c>
       <c r="T33" s="3">
-        <v>375.15803891571608</v>
+        <v>371.8644900402705</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
-        <v>7.7095127176201067E-2</v>
+        <v>0</v>
       </c>
       <c r="V33" s="3">
-        <v>23322467.600951109</v>
+        <v>23322467.60095111</v>
       </c>
       <c r="W33" s="3">
         <v>307442.101903148</v>
       </c>
       <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
-        <v>1.3182228705962926E-2</v>
+        <v>0</v>
       </c>
       <c r="Y33" s="3">
-        <v>2033978.1299748039</v>
+        <v>2033978.129974804</v>
       </c>
       <c r="Z33" s="3">
-        <v>8632.8553056851961</v>
+        <v>8632.855305685196</v>
       </c>
       <c r="AA33" s="4">
         <f>IF(Y33=0,0,Z33/Y33)</f>
-        <v>4.244320614102245E-3</v>
+        <v>0</v>
       </c>
       <c r="AB33" s="3">
-        <v>207305.28823611679</v>
+        <v>207305.2882361168</v>
       </c>
       <c r="AC33" s="3">
-        <v>19.081856428296309</v>
+        <v>19.08185642829631</v>
       </c>
       <c r="AD33" s="4">
         <f>IF(AB33=0,0,AC33/AB33)</f>
-        <v>9.2047128129999444E-5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:30">
       <c r="B34" t="s">
         <v>32</v>
       </c>
       <c r="C34" s="3">
         <f>J34+M34+G34+P34</f>
-        <v>62.342351079779156</v>
+        <v>0</v>
       </c>
       <c r="D34" s="3">
         <f>G34</f>
-        <v>42.554425860531921</v>
+        <v>0</v>
       </c>
       <c r="E34" s="3">
         <f>J34+M34+P34</f>
-        <v>19.787925219247239</v>
+        <v>0</v>
       </c>
       <c r="F34" s="3">
-        <v>396.28526128416758</v>
+        <v>382.8744648174589</v>
       </c>
       <c r="G34" s="3">
-        <v>42.554425860531921</v>
+        <v>41.85489240021754</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
-        <v>0.10738331706466636</v>
+        <v>0</v>
       </c>
       <c r="I34" s="3">
-        <v>721.62080381298233</v>
+        <v>721.6208038129823</v>
       </c>
       <c r="J34" s="3">
         <v>15.78004529479356</v>
       </c>
       <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
-        <v>2.1867503280688632E-2</v>
+        <v>0</v>
       </c>
       <c r="L34" s="3">
-        <v>15355.961975565249</v>
+        <v>15355.96197556525</v>
       </c>
       <c r="M34" s="3">
         <v>1.813587757010013</v>
       </c>
       <c r="N34" s="4">
         <f>IF(L34=0,0,M34/L34)</f>
-        <v>1.181031680005352E-4</v>
+        <v>0</v>
       </c>
       <c r="O34" s="3">
         <v>391.5266582641886</v>
@@ -2946,259 +2917,259 @@
       </c>
       <c r="Q34" s="4">
         <f>IF(O34=0,0,P34/O34)</f>
-        <v>5.6044515006256198E-3</v>
+        <v>0</v>
       </c>
       <c r="S34" s="3">
-        <v>4405.2233953297473</v>
+        <v>4256.145041636478</v>
       </c>
       <c r="T34" s="3">
-        <v>473.04750060138031</v>
+        <v>465.271281129561</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
-        <v>0.10738331706466635</v>
+        <v>0</v>
       </c>
       <c r="V34" s="3">
-        <v>21162807.846375171</v>
+        <v>21162807.84637517</v>
       </c>
       <c r="W34" s="3">
-        <v>369371.39764320478</v>
+        <v>369371.3976432048</v>
       </c>
       <c r="X34" s="4">
         <f>IF(V34=0,0,W34/V34)</f>
-        <v>1.7453799152009584E-2</v>
+        <v>0</v>
       </c>
       <c r="Y34" s="3">
         <v>1664123.912966297</v>
       </c>
       <c r="Z34" s="3">
-        <v>9278.7286326091271</v>
+        <v>9278.728632609127</v>
       </c>
       <c r="AA34" s="4">
         <f>IF(Y34=0,0,Z34/Y34)</f>
-        <v>5.5757438255122568E-3</v>
+        <v>0</v>
       </c>
       <c r="AB34" s="3">
         <v>172634.6152091868</v>
       </c>
       <c r="AC34" s="3">
-        <v>20.141959563101409</v>
+        <v>20.14195956310141</v>
       </c>
       <c r="AD34" s="4">
         <f>IF(AB34=0,0,AC34/AB34)</f>
-        <v>1.1667393320102554E-4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:30">
       <c r="B35" t="s">
         <v>33</v>
       </c>
       <c r="C35" s="3">
         <f>J35+M35+G35+P35</f>
-        <v>70.415390099069029</v>
+        <v>0</v>
       </c>
       <c r="D35" s="3">
         <f>G35</f>
-        <v>50.158449486042947</v>
+        <v>0</v>
       </c>
       <c r="E35" s="3">
         <f>J35+M35+P35</f>
-        <v>20.256940613026089</v>
+        <v>0</v>
       </c>
       <c r="F35" s="3">
-        <v>351.26672270713158</v>
+        <v>339.3794107528897</v>
       </c>
       <c r="G35" s="3">
-        <v>50.158449486042947</v>
+        <v>49.09141688271048</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
-        <v>0.14279305793467525</v>
+        <v>0</v>
       </c>
       <c r="I35" s="3">
-        <v>656.23600296293523</v>
+        <v>656.2360029629352</v>
       </c>
       <c r="J35" s="3">
-        <v>17.337373260950319</v>
+        <v>17.33737326095032</v>
       </c>
       <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
-        <v>2.6419417987844761E-2</v>
+        <v>0</v>
       </c>
       <c r="L35" s="3">
-        <v>12320.893910346331</v>
+        <v>12320.89391034633</v>
       </c>
       <c r="M35" s="3">
-        <v>0.76115932066179814</v>
+        <v>0.7611593206617981</v>
       </c>
       <c r="N35" s="4">
         <f>IF(L35=0,0,M35/L35)</f>
-        <v>6.1777929929469097E-5</v>
+        <v>0</v>
       </c>
       <c r="O35" s="3">
-        <v>305.89771512841492</v>
+        <v>305.8977151284149</v>
       </c>
       <c r="P35" s="3">
         <v>2.158408031413972</v>
       </c>
       <c r="Q35" s="4">
         <f>IF(O35=0,0,P35/O35)</f>
-        <v>7.0559795796705412E-3</v>
+        <v>0</v>
       </c>
       <c r="S35" s="3">
-        <v>3904.7840938011818</v>
+        <v>3772.641241557029</v>
       </c>
       <c r="T35" s="3">
-        <v>557.57606132855017</v>
+        <v>545.7146134095751</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
-        <v>0.14279305793467514</v>
+        <v>0</v>
       </c>
       <c r="V35" s="3">
-        <v>20232379.411657181</v>
+        <v>20232379.41165718</v>
       </c>
       <c r="W35" s="3">
-        <v>430534.00670235232</v>
+        <v>430534.0067023523</v>
       </c>
       <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
-        <v>2.1279454973758244E-2</v>
+        <v>0</v>
       </c>
       <c r="Y35" s="3">
-        <v>1291512.2728871789</v>
+        <v>1291512.272887179</v>
       </c>
       <c r="Z35" s="3">
-        <v>8071.8257655487396</v>
+        <v>8071.82576554874</v>
       </c>
       <c r="AA35" s="4">
         <f>IF(Y35=0,0,Z35/Y35)</f>
-        <v>6.2499024864116487E-3</v>
+        <v>0</v>
       </c>
       <c r="AB35" s="3">
-        <v>138538.51808137319</v>
+        <v>138538.5180813732</v>
       </c>
       <c r="AC35" s="3">
-        <v>8.4808250792266335</v>
+        <v>8.480825079226634</v>
       </c>
       <c r="AD35" s="4">
         <f>IF(AB35=0,0,AC35/AB35)</f>
-        <v>6.1216369257286713E-5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30">
       <c r="B36" t="s">
         <v>34</v>
       </c>
       <c r="C36" s="3">
         <f>J36+M36+G36+P36</f>
-        <v>67.966273304051526</v>
+        <v>0</v>
       </c>
       <c r="D36" s="3">
         <f>G36</f>
-        <v>48.890421519106461</v>
+        <v>0</v>
       </c>
       <c r="E36" s="3">
         <f>J36+M36+P36</f>
-        <v>19.075851784945058</v>
+        <v>0</v>
       </c>
       <c r="F36" s="3">
-        <v>308.52409051931693</v>
+        <v>298.0832435152593</v>
       </c>
       <c r="G36" s="3">
-        <v>48.890421519106461</v>
+        <v>47.77947036092321</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
-        <v>0.15846549109605235</v>
+        <v>0</v>
       </c>
       <c r="I36" s="3">
-        <v>465.22851237667129</v>
+        <v>465.2285123766713</v>
       </c>
       <c r="J36" s="3">
         <v>14.87518745130871</v>
       </c>
       <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
-        <v>3.1973937657683901E-2</v>
+        <v>0</v>
       </c>
       <c r="L36" s="3">
-        <v>10752.450404824391</v>
+        <v>10752.45040482439</v>
       </c>
       <c r="M36" s="3">
-        <v>2.3809073660019791</v>
+        <v>2.380907366001979</v>
       </c>
       <c r="N36" s="4">
         <f>IF(L36=0,0,M36/L36)</f>
-        <v>2.2142928136024861E-4</v>
+        <v>0</v>
       </c>
       <c r="O36" s="3">
-        <v>286.13725715609343</v>
+        <v>286.1372571560934</v>
       </c>
       <c r="P36" s="3">
-        <v>1.8197569676343699</v>
+        <v>1.81975696763437</v>
       </c>
       <c r="Q36" s="4">
         <f>IF(O36=0,0,P36/O36)</f>
-        <v>6.3597344355672538E-3</v>
+        <v>0</v>
       </c>
       <c r="S36" s="3">
-        <v>3429.6444363696219</v>
+        <v>3313.580913491462</v>
       </c>
       <c r="T36" s="3">
-        <v>543.4802898941557</v>
+        <v>531.1306304159348</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
-        <v>0.15846549109605232</v>
+        <v>0</v>
       </c>
       <c r="V36" s="3">
-        <v>16252582.504079361</v>
+        <v>16252582.50407936</v>
       </c>
       <c r="W36" s="3">
-        <v>432632.14916820452</v>
+        <v>432632.1491682045</v>
       </c>
       <c r="X36" s="4">
         <f>IF(V36=0,0,W36/V36)</f>
-        <v>2.6619286446299524E-2</v>
+        <v>0</v>
       </c>
       <c r="Y36" s="3">
         <v>1133183.161267315</v>
       </c>
       <c r="Z36" s="3">
-        <v>7758.9643017679919</v>
+        <v>7758.964301767992</v>
       </c>
       <c r="AA36" s="4">
         <f>IF(Y36=0,0,Z36/Y36)</f>
-        <v>6.8470522391901939E-3</v>
+        <v>0</v>
       </c>
       <c r="AB36" s="3">
-        <v>120916.42366991749</v>
+        <v>120916.4236699175</v>
       </c>
       <c r="AC36" s="3">
         <v>26.50257837252866</v>
       </c>
       <c r="AD36" s="4">
         <f>IF(AB36=0,0,AC36/AB36)</f>
-        <v>2.1918096457166532E-4</v>
-      </c>
-    </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:30">
       <c r="A38" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30">
       <c r="B39" t="s">
         <v>28</v>
       </c>
       <c r="C39" s="3">
         <f>C41+C42+C43+C44+C45</f>
-        <v>280.76919049490539</v>
+        <v>0</v>
       </c>
       <c r="D39" s="3">
         <f>D41+D42+D43+D44+D45</f>
-        <v>280.76919049490539</v>
+        <v>0</v>
       </c>
       <c r="E39" s="3">
         <f>E41+E42+E43+E44+E45</f>
@@ -3206,27 +3177,27 @@
       </c>
       <c r="F39" s="3">
         <f>F41+F42+F43+F44+F45</f>
-        <v>660.80113298361266</v>
+        <v>0</v>
       </c>
       <c r="G39" s="3">
         <f>G41+G42+G43+G44+G45</f>
-        <v>273.59501122623988</v>
+        <v>0</v>
       </c>
       <c r="H39" s="4">
         <f>IF(F39=0,0,G39/F39)</f>
-        <v>0.41403532404812754</v>
+        <v>0</v>
       </c>
       <c r="I39" s="3">
         <f>I41+I42+I43+I44+I45</f>
-        <v>814.53034621778045</v>
+        <v>0</v>
       </c>
       <c r="J39" s="6">
         <f>J41+J42+J43+J44+J45</f>
-        <v>7.1741792686655108</v>
+        <v>0</v>
       </c>
       <c r="K39" s="7">
         <f>IF(I39=0,0,J39/I39)</f>
-        <v>8.8077495233644196E-3</v>
+        <v>0</v>
       </c>
       <c r="L39" s="3">
         <f>L41+L42+L43+L44+L45</f>
@@ -3254,27 +3225,27 @@
       </c>
       <c r="S39" s="3">
         <f>S41+S42+S43+S44+S45</f>
-        <v>7345.6595414292105</v>
+        <v>0</v>
       </c>
       <c r="T39" s="3">
         <f>T41+T42+T43+T44+T45</f>
-        <v>3041.3625285828634</v>
+        <v>0</v>
       </c>
       <c r="U39" s="4">
         <f>IF(S39=0,0,T39/S39)</f>
-        <v>0.4140353240481276</v>
+        <v>0</v>
       </c>
       <c r="V39" s="3">
         <f>V41+V42+V43+V44+V45</f>
-        <v>26890169.836246081</v>
+        <v>0</v>
       </c>
       <c r="W39" s="6">
         <f>W41+W42+W43+W44+W45</f>
-        <v>267021.30009852862</v>
+        <v>0</v>
       </c>
       <c r="X39" s="7">
         <f>IF(V39=0,0,W39/V39)</f>
-        <v>9.9300711644670411E-3</v>
+        <v>0</v>
       </c>
       <c r="Y39" s="3">
         <f>Y41+Y42+Y43+Y44+Y45</f>
@@ -3301,46 +3272,46 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30">
       <c r="A40" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30">
       <c r="B41" t="s">
         <v>30</v>
       </c>
       <c r="C41" s="3">
         <f>J41+M41+G41+P41</f>
-        <v>75.545013639823878</v>
+        <v>0</v>
       </c>
       <c r="D41" s="3">
         <f>G41+J41</f>
-        <v>75.545013639823878</v>
+        <v>0</v>
       </c>
       <c r="E41" s="3">
-        <f>M41+P41</f>
+        <f>P41+M41</f>
         <v>0</v>
       </c>
       <c r="F41" s="3">
-        <v>158.01636350616181</v>
+        <v>155.6388197021622</v>
       </c>
       <c r="G41" s="3">
-        <v>73.076706089663659</v>
+        <v>72.14250991153671</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
-        <v>0.46246290237412058</v>
+        <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>289.90090139463632</v>
+        <v>289.9009013946363</v>
       </c>
       <c r="J41" s="6">
-        <v>2.468307550160215</v>
+        <v>2.57749961572641</v>
       </c>
       <c r="K41" s="7">
         <f>IF(I41=0,0,J41/I41)</f>
-        <v>8.5143148513365848E-3</v>
+        <v>0</v>
       </c>
       <c r="L41" s="3">
         <v>0</v>
@@ -3363,24 +3334,24 @@
         <v>0</v>
       </c>
       <c r="S41" s="3">
-        <v>1756.5563228532919</v>
+        <v>1730.126847391954</v>
       </c>
       <c r="T41" s="3">
-        <v>812.34213525034636</v>
+        <v>801.9573360620632</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
-        <v>0.46246290237412069</v>
+        <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>7917202.4300766056</v>
+        <v>7917202.430076606</v>
       </c>
       <c r="W41" s="6">
-        <v>72642.66277817823</v>
+        <v>75888.02632279508</v>
       </c>
       <c r="X41" s="7">
         <f>IF(V41=0,0,W41/V41)</f>
-        <v>9.1752943567814452E-3</v>
+        <v>0</v>
       </c>
       <c r="Y41" s="3">
         <v>0</v>
@@ -3403,41 +3374,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30">
       <c r="B42" t="s">
         <v>31</v>
       </c>
       <c r="C42" s="3">
         <f>J42+M42+G42+P42</f>
-        <v>75.523020712148451</v>
+        <v>0</v>
       </c>
       <c r="D42" s="3">
         <f>G42+J42</f>
-        <v>75.523020712148451</v>
+        <v>0</v>
       </c>
       <c r="E42" s="3">
-        <f>M42+P42</f>
+        <f>P42+M42</f>
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>150.30970532381971</v>
+        <v>148.048117342397</v>
       </c>
       <c r="G42" s="3">
-        <v>73.847323583703343</v>
+        <v>72.88503207356277</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
-        <v>0.49130110011599293</v>
+        <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>172.51020331953049</v>
+        <v>172.5102033195305</v>
       </c>
       <c r="J42" s="6">
-        <v>1.6756971284451141</v>
+        <v>2.092952702855459</v>
       </c>
       <c r="K42" s="7">
         <f>IF(I42=0,0,J42/I42)</f>
-        <v>9.7136116948475151E-3</v>
+        <v>0</v>
       </c>
       <c r="L42" s="3">
         <v>0</v>
@@ -3460,24 +3431,24 @@
         <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>1670.8868462377629</v>
+        <v>1645.746369768679</v>
       </c>
       <c r="T42" s="3">
-        <v>820.90854572595504</v>
+        <v>810.2114305724377</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
-        <v>0.49130110011599304</v>
+        <v>0</v>
       </c>
       <c r="V42" s="3">
         <v>5775458.9344058</v>
       </c>
       <c r="W42" s="6">
-        <v>65017.803183237091</v>
+        <v>81365.06762592774</v>
       </c>
       <c r="X42" s="7">
         <f>IF(V42=0,0,W42/V42)</f>
-        <v>1.1257599425720159E-2</v>
+        <v>0</v>
       </c>
       <c r="Y42" s="3">
         <v>0</v>
@@ -3500,41 +3471,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30">
       <c r="B43" t="s">
         <v>32</v>
       </c>
       <c r="C43" s="3">
         <f>J43+M43+G43+P43</f>
-        <v>75.681017568814596</v>
+        <v>0</v>
       </c>
       <c r="D43" s="3">
         <f>G43+J43</f>
-        <v>75.681017568814596</v>
+        <v>0</v>
       </c>
       <c r="E43" s="3">
-        <f>M43+P43</f>
+        <f>P43+M43</f>
         <v>0</v>
       </c>
       <c r="F43" s="3">
-        <v>136.8081181206467</v>
+        <v>134.74967754932</v>
       </c>
       <c r="G43" s="3">
-        <v>73.912686379217163</v>
+        <v>72.9230042046555</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
-        <v>0.54026535409277343</v>
+        <v>0</v>
       </c>
       <c r="I43" s="3">
-        <v>135.45605543604131</v>
+        <v>135.4560554360413</v>
       </c>
       <c r="J43" s="6">
-        <v>1.768331189597433</v>
+        <v>2.287314210165379</v>
       </c>
       <c r="K43" s="7">
         <f>IF(I43=0,0,J43/I43)</f>
-        <v>1.3054648490280239E-2</v>
+        <v>0</v>
       </c>
       <c r="L43" s="3">
         <v>0</v>
@@ -3557,24 +3528,24 @@
         <v>0</v>
       </c>
       <c r="S43" s="3">
-        <v>1520.7992360431149</v>
+        <v>1497.917005870538</v>
       </c>
       <c r="T43" s="3">
-        <v>821.63513776485274</v>
+        <v>810.6335399380957</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
-        <v>0.54026535409277343</v>
+        <v>0</v>
       </c>
       <c r="V43" s="3">
-        <v>4941006.3189266957</v>
+        <v>4941006.318926696</v>
       </c>
       <c r="W43" s="6">
-        <v>72259.685244018212</v>
+        <v>93694.98213961534</v>
       </c>
       <c r="X43" s="7">
         <f>IF(V43=0,0,W43/V43)</f>
-        <v>1.4624487519318684E-2</v>
+        <v>0</v>
       </c>
       <c r="Y43" s="3">
         <v>0</v>
@@ -3597,41 +3568,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30">
       <c r="B44" t="s">
         <v>33</v>
       </c>
       <c r="C44" s="3">
         <f>J44+M44+G44+P44</f>
-        <v>34.237463857077486</v>
+        <v>0</v>
       </c>
       <c r="D44" s="3">
         <f>G44+J44</f>
-        <v>34.237463857077486</v>
+        <v>0</v>
       </c>
       <c r="E44" s="3">
-        <f>M44+P44</f>
+        <f>P44+M44</f>
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>120.55842024780129</v>
+        <v>118.7444756744663</v>
       </c>
       <c r="G44" s="3">
-        <v>33.537270644134047</v>
+        <v>33.20204370990226</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
-        <v>0.27818273145251909</v>
+        <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>131.31388542968341</v>
+        <v>131.3138854296834</v>
       </c>
       <c r="J44" s="6">
-        <v>0.70019321294344261</v>
+        <v>0.8526697489883809</v>
       </c>
       <c r="K44" s="7">
         <f>IF(I44=0,0,J44/I44)</f>
-        <v>5.3322099993635894E-3</v>
+        <v>0</v>
       </c>
       <c r="L44" s="3">
         <v>0</v>
@@ -3654,24 +3625,24 @@
         <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>1340.1628202336269</v>
+        <v>1319.998479409059</v>
       </c>
       <c r="T44" s="3">
-        <v>372.81015392370171</v>
+        <v>369.0836728311747</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
-        <v>0.27818273145251915</v>
+        <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>4714339.9302510964</v>
+        <v>4714339.930251096</v>
       </c>
       <c r="W44" s="6">
-        <v>30505.503986442462</v>
+        <v>37175.27322141826</v>
       </c>
       <c r="X44" s="7">
         <f>IF(V44=0,0,W44/V44)</f>
-        <v>6.4707900655813907E-3</v>
+        <v>0</v>
       </c>
       <c r="Y44" s="3">
         <v>0</v>
@@ -3694,41 +3665,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30">
       <c r="B45" t="s">
         <v>34</v>
       </c>
       <c r="C45" s="3">
         <f>J45+M45+G45+P45</f>
-        <v>19.782674717040955</v>
+        <v>0</v>
       </c>
       <c r="D45" s="3">
         <f>G45+J45</f>
-        <v>19.782674717040955</v>
+        <v>0</v>
       </c>
       <c r="E45" s="3">
-        <f>M45+P45</f>
+        <f>P45+M45</f>
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>95.10852578518319</v>
+        <v>93.67750509105568</v>
       </c>
       <c r="G45" s="3">
-        <v>19.22102452952165</v>
+        <v>19.07953157899767</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
-        <v>0.20209570457369094</v>
+        <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>85.349300637888987</v>
+        <v>85.34930063788899</v>
       </c>
       <c r="J45" s="6">
-        <v>0.56165018751930618</v>
+        <v>0.6193965967932891</v>
       </c>
       <c r="K45" s="7">
         <f>IF(I45=0,0,J45/I45)</f>
-        <v>6.5806067925760327E-3</v>
+        <v>0</v>
       </c>
       <c r="L45" s="3">
         <v>0</v>
@@ -3751,24 +3722,24 @@
         <v>0</v>
       </c>
       <c r="S45" s="3">
-        <v>1057.2543160614141</v>
+        <v>1041.346669583361</v>
       </c>
       <c r="T45" s="3">
-        <v>213.66655591800719</v>
+        <v>212.0936787085381</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
-        <v>0.20209570457369092</v>
+        <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>3542162.2225858839</v>
+        <v>3542162.222585884</v>
       </c>
       <c r="W45" s="6">
-        <v>26595.644906652629</v>
+        <v>29337.3724585874</v>
       </c>
       <c r="X45" s="7">
         <f>IF(V45=0,0,W45/V45)</f>
-        <v>7.5083079868761672E-3</v>
+        <v>0</v>
       </c>
       <c r="Y45" s="3">
         <v>0</v>
@@ -3791,22 +3762,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30">
       <c r="A47" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30">
       <c r="B48" t="s">
         <v>28</v>
       </c>
       <c r="C48" s="3">
         <f>C50+C51+C52+C53+C54</f>
-        <v>531.36419183716009</v>
+        <v>0</v>
       </c>
       <c r="D48" s="3">
         <f>D50+D51+D52+D53+D54</f>
-        <v>531.36419183716009</v>
+        <v>0</v>
       </c>
       <c r="E48" s="3">
         <f>E50+E51+E52+E53+E54</f>
@@ -3814,27 +3785,27 @@
       </c>
       <c r="F48" s="3">
         <f>F50+F51+F52+F53+F54</f>
-        <v>660.80113298361266</v>
+        <v>0</v>
       </c>
       <c r="G48" s="3">
         <f>G50+G51+G52+G53+G54</f>
-        <v>504.69626905365925</v>
+        <v>0</v>
       </c>
       <c r="H48" s="4">
         <f>IF(F48=0,0,G48/F48)</f>
-        <v>0.76376423081310807</v>
+        <v>0</v>
       </c>
       <c r="I48" s="3">
         <f>I50+I51+I52+I53+I54</f>
-        <v>814.53034621778045</v>
+        <v>0</v>
       </c>
       <c r="J48" s="6">
         <f>J50+J51+J52+J53+J54</f>
-        <v>26.667922783500853</v>
+        <v>0</v>
       </c>
       <c r="K48" s="7">
         <f>IF(I48=0,0,J48/I48)</f>
-        <v>3.2740244617443223E-2</v>
+        <v>0</v>
       </c>
       <c r="L48" s="3">
         <f>L50+L51+L52+L53+L54</f>
@@ -3862,27 +3833,27 @@
       </c>
       <c r="S48" s="3">
         <f>S50+S51+S52+S53+S54</f>
-        <v>7345.6595414292105</v>
+        <v>0</v>
       </c>
       <c r="T48" s="3">
         <f>T50+T51+T52+T53+T54</f>
-        <v>5610.3520094746491</v>
+        <v>0</v>
       </c>
       <c r="U48" s="4">
         <f>IF(S48=0,0,T48/S48)</f>
-        <v>0.76376423081310807</v>
+        <v>0</v>
       </c>
       <c r="V48" s="3">
         <f>V50+V51+V52+V53+V54</f>
-        <v>26890169.836246081</v>
+        <v>0</v>
       </c>
       <c r="W48" s="6">
         <f>W50+W51+W52+W53+W54</f>
-        <v>1013392.394379443</v>
+        <v>0</v>
       </c>
       <c r="X48" s="7">
         <f>IF(V48=0,0,W48/V48)</f>
-        <v>3.7686351575714504E-2</v>
+        <v>0</v>
       </c>
       <c r="Y48" s="3">
         <f>Y50+Y51+Y52+Y53+Y54</f>
@@ -3909,46 +3880,46 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30">
       <c r="A49" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30">
       <c r="B50" t="s">
         <v>30</v>
       </c>
       <c r="C50" s="3">
         <f>J50+M50+G50+P50</f>
-        <v>139.20125997283833</v>
+        <v>0</v>
       </c>
       <c r="D50" s="3">
         <f>G50+J50</f>
-        <v>139.20125997283833</v>
+        <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>M50+P50</f>
+        <f>P50+M50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
-        <v>158.01636350616181</v>
+        <v>155.6388197021622</v>
       </c>
       <c r="G50" s="3">
-        <v>129.99805657434101</v>
+        <v>128.0966173135081</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
-        <v>0.82268730712355476</v>
+        <v>0</v>
       </c>
       <c r="I50" s="3">
-        <v>289.90090139463632</v>
+        <v>289.9009013946363</v>
       </c>
       <c r="J50" s="6">
-        <v>9.2032033984973101</v>
+        <v>9.579560738421627</v>
       </c>
       <c r="K50" s="7">
         <f>IF(I50=0,0,J50/I50)</f>
-        <v>3.1746032365622665E-2</v>
+        <v>0</v>
       </c>
       <c r="L50" s="3">
         <v>0</v>
@@ -3971,24 +3942,24 @@
         <v>0</v>
       </c>
       <c r="S50" s="3">
-        <v>1756.5563228532919</v>
+        <v>1730.126847391954</v>
       </c>
       <c r="T50" s="3">
-        <v>1445.096591059028</v>
+        <v>1423.95963358179</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
-        <v>0.82268730712355465</v>
+        <v>0</v>
       </c>
       <c r="V50" s="3">
-        <v>7917202.4300766056</v>
+        <v>7917202.430076606</v>
       </c>
       <c r="W50" s="6">
-        <v>278133.08442789782</v>
+        <v>289948.8097963436</v>
       </c>
       <c r="X50" s="7">
         <f>IF(V50=0,0,W50/V50)</f>
-        <v>3.5130222687157771E-2</v>
+        <v>0</v>
       </c>
       <c r="Y50" s="3">
         <v>0</v>
@@ -4011,41 +3982,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:30">
       <c r="B51" t="s">
         <v>31</v>
       </c>
       <c r="C51" s="3">
         <f>J51+M51+G51+P51</f>
-        <v>132.6820338646759</v>
+        <v>0</v>
       </c>
       <c r="D51" s="3">
         <f>G51+J51</f>
-        <v>132.6820338646759</v>
+        <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>M51+P51</f>
+        <f>P51+M51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <v>150.30970532381971</v>
+        <v>148.048117342397</v>
       </c>
       <c r="G51" s="3">
-        <v>126.503663964271</v>
+        <v>124.6466030827076</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
-        <v>0.84162006499672015</v>
+        <v>0</v>
       </c>
       <c r="I51" s="3">
-        <v>172.51020331953049</v>
+        <v>172.5102033195305</v>
       </c>
       <c r="J51" s="6">
-        <v>6.1783699004049124</v>
+        <v>7.55612644698788</v>
       </c>
       <c r="K51" s="7">
         <f>IF(I51=0,0,J51/I51)</f>
-        <v>3.581451868653289E-2</v>
+        <v>0</v>
       </c>
       <c r="L51" s="3">
         <v>0</v>
@@ -4068,24 +4039,24 @@
         <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>1670.8868462377629</v>
+        <v>1645.746369768679</v>
       </c>
       <c r="T51" s="3">
-        <v>1406.251896132791</v>
+        <v>1385.608261758136</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
-        <v>0.84162006499672026</v>
+        <v>0</v>
       </c>
       <c r="V51" s="3">
         <v>5775458.9344058</v>
       </c>
       <c r="W51" s="6">
-        <v>244923.17248689849</v>
+        <v>301589.2033798397</v>
       </c>
       <c r="X51" s="7">
         <f>IF(V51=0,0,W51/V51)</f>
-        <v>4.2407568864845036E-2</v>
+        <v>0</v>
       </c>
       <c r="Y51" s="3">
         <v>0</v>
@@ -4108,41 +4079,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30">
       <c r="B52" t="s">
         <v>32</v>
       </c>
       <c r="C52" s="3">
         <f>J52+M52+G52+P52</f>
-        <v>125.46678963002367</v>
+        <v>0</v>
       </c>
       <c r="D52" s="3">
         <f>G52+J52</f>
-        <v>125.46678963002367</v>
+        <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>M52+P52</f>
+        <f>P52+M52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
-        <v>136.8081181206467</v>
+        <v>134.74967754932</v>
       </c>
       <c r="G52" s="3">
-        <v>119.03235492283009</v>
+        <v>117.2759712044506</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
-        <v>0.87006792109996922</v>
+        <v>0</v>
       </c>
       <c r="I52" s="3">
-        <v>135.45605543604131</v>
+        <v>135.4560554360413</v>
       </c>
       <c r="J52" s="6">
-        <v>6.434434707193577</v>
+        <v>8.085542072412819</v>
       </c>
       <c r="K52" s="7">
         <f>IF(I52=0,0,J52/I52)</f>
-        <v>4.7502008577473623E-2</v>
+        <v>0</v>
       </c>
       <c r="L52" s="3">
         <v>0</v>
@@ -4165,24 +4136,24 @@
         <v>0</v>
       </c>
       <c r="S52" s="3">
-        <v>1520.7992360431149</v>
+        <v>1497.917005870538</v>
       </c>
       <c r="T52" s="3">
-        <v>1323.198629714454</v>
+        <v>1303.674152265284</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
-        <v>0.870067921099969</v>
+        <v>0</v>
       </c>
       <c r="V52" s="3">
-        <v>4941006.3189266957</v>
+        <v>4941006.318926696</v>
       </c>
       <c r="W52" s="6">
-        <v>268918.30092897639</v>
+        <v>340742.8114436772</v>
       </c>
       <c r="X52" s="7">
         <f>IF(V52=0,0,W52/V52)</f>
-        <v>5.4425816032429575E-2</v>
+        <v>0</v>
       </c>
       <c r="Y52" s="3">
         <v>0</v>
@@ -4205,41 +4176,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:30">
       <c r="B53" t="s">
         <v>33</v>
       </c>
       <c r="C53" s="3">
         <f>J53+M53+G53+P53</f>
-        <v>80.839654447488186</v>
+        <v>0</v>
       </c>
       <c r="D53" s="3">
         <f>G53+J53</f>
-        <v>80.839654447488186</v>
+        <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>M53+P53</f>
+        <f>P53+M53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
-        <v>120.55842024780129</v>
+        <v>118.7444756744663</v>
       </c>
       <c r="G53" s="3">
-        <v>78.153950601004468</v>
+        <v>77.06056921867676</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
-        <v>0.64826621351178337</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
-        <v>131.31388542968341</v>
+        <v>131.3138854296834</v>
       </c>
       <c r="J53" s="6">
-        <v>2.6857038464837242</v>
+        <v>3.240305918559723</v>
       </c>
       <c r="K53" s="7">
         <f>IF(I53=0,0,J53/I53)</f>
-        <v>2.0452550297294172E-2</v>
+        <v>0</v>
       </c>
       <c r="L53" s="3">
         <v>0</v>
@@ -4262,24 +4233,24 @@
         <v>0</v>
       </c>
       <c r="S53" s="3">
-        <v>1340.1628202336269</v>
+        <v>1319.998479409059</v>
       </c>
       <c r="T53" s="3">
-        <v>868.78227696212616</v>
+        <v>856.6279282744163</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
-        <v>0.64826621351178337</v>
+        <v>0</v>
       </c>
       <c r="V53" s="3">
-        <v>4714339.9302510964</v>
+        <v>4714339.930251096</v>
       </c>
       <c r="W53" s="6">
-        <v>118125.7799676377</v>
+        <v>142904.1636235043</v>
       </c>
       <c r="X53" s="7">
         <f>IF(V53=0,0,W53/V53)</f>
-        <v>2.5056695468573489E-2</v>
+        <v>0</v>
       </c>
       <c r="Y53" s="3">
         <v>0</v>
@@ -4302,41 +4273,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:30">
       <c r="B54" t="s">
         <v>34</v>
       </c>
       <c r="C54" s="3">
         <f>J54+M54+G54+P54</f>
-        <v>53.17445392213402</v>
+        <v>0</v>
       </c>
       <c r="D54" s="3">
         <f>G54+J54</f>
-        <v>53.17445392213402</v>
+        <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>M54+P54</f>
+        <f>P54+M54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <v>95.10852578518319</v>
+        <v>93.67750509105568</v>
       </c>
       <c r="G54" s="3">
-        <v>51.008242991212697</v>
+        <v>50.32660180257193</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
-        <v>0.53631619847018164</v>
+        <v>0</v>
       </c>
       <c r="I54" s="3">
-        <v>85.349300637888987</v>
+        <v>85.34930063788899</v>
       </c>
       <c r="J54" s="6">
-        <v>2.1662109309213271</v>
+        <v>2.379898399251702</v>
       </c>
       <c r="K54" s="7">
         <f>IF(I54=0,0,J54/I54)</f>
-        <v>2.5380535220925808E-2</v>
+        <v>0</v>
       </c>
       <c r="L54" s="3">
         <v>0</v>
@@ -4359,24 +4330,24 @@
         <v>0</v>
       </c>
       <c r="S54" s="3">
-        <v>1057.2543160614141</v>
+        <v>1041.346669583361</v>
       </c>
       <c r="T54" s="3">
-        <v>567.0226156062497</v>
+        <v>559.4452918832071</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
-        <v>0.53631619847018186</v>
+        <v>0</v>
       </c>
       <c r="V54" s="3">
-        <v>3542162.2225858839</v>
+        <v>3542162.222585884</v>
       </c>
       <c r="W54" s="6">
-        <v>103292.0565680326</v>
+        <v>113587.6470628493</v>
       </c>
       <c r="X54" s="7">
         <f>IF(V54=0,0,W54/V54)</f>
-        <v>2.9160735753267199E-2</v>
+        <v>0</v>
       </c>
       <c r="Y54" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
Write down some additional notes on running, include death to case conversion for NTDs
</commit_message>
<xml_diff>
--- a/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
+++ b/legacy/vivarium_gates_lsff_by_wealth_quintile/5000_analyze_results/results_spreadsheet.xlsx
@@ -175,13 +175,13 @@
     <t>Maternal Disorders DALYs Averted by Iron Fortification (%)</t>
   </si>
   <si>
-    <t>Baseline Annual NTD Deaths and Stillbirths</t>
+    <t>Baseline Annual NTD Cases</t>
   </si>
   <si>
-    <t>Annual NTD Deaths and Stillbirths Averted</t>
+    <t>Annual NTD Cases Averted</t>
   </si>
   <si>
-    <t>Annual NTD Deaths and Stillbirths Averted (%)</t>
+    <t>Annual NTD Cases Averted (%)</t>
   </si>
   <si>
     <t>Baseline Prevalent Anemia Cases</t>
@@ -862,10 +862,10 @@
         <v>0</v>
       </c>
       <c r="F5" s="3">
-        <v>363.1566259346982</v>
+        <v>363.2412074975357</v>
       </c>
       <c r="G5" s="3">
-        <v>25.60632743086544</v>
+        <v>25.61229131266783</v>
       </c>
       <c r="H5" s="4">
         <f>IF(F5=0,0,G5/F5)</f>
@@ -902,10 +902,10 @@
         <v>0</v>
       </c>
       <c r="S5" s="3">
-        <v>4036.955751400944</v>
+        <v>5246.786650973078</v>
       </c>
       <c r="T5" s="3">
-        <v>284.647459008158</v>
+        <v>369.9531478984281</v>
       </c>
       <c r="U5" s="4">
         <f>IF(S5=0,0,T5/S5)</f>
@@ -959,10 +959,10 @@
         <v>0</v>
       </c>
       <c r="F6" s="3">
-        <v>320.8109788943828</v>
+        <v>320.8856978779631</v>
       </c>
       <c r="G6" s="3">
-        <v>19.29712236727314</v>
+        <v>19.30161679378641</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
@@ -999,10 +999,10 @@
         <v>0</v>
       </c>
       <c r="S6" s="3">
-        <v>3566.229097505511</v>
+        <v>4634.988435682091</v>
       </c>
       <c r="T6" s="3">
-        <v>214.5124818404361</v>
+        <v>278.7994953367825</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
@@ -1056,10 +1056,10 @@
         <v>0</v>
       </c>
       <c r="F7" s="3">
-        <v>288.0128603408813</v>
+        <v>288.0799404272827</v>
       </c>
       <c r="G7" s="3">
-        <v>14.64607722620195</v>
+        <v>14.64948839376098</v>
       </c>
       <c r="H7" s="4">
         <f>IF(F7=0,0,G7/F7)</f>
@@ -1096,10 +1096,10 @@
         <v>0</v>
       </c>
       <c r="S7" s="3">
-        <v>3201.635575388428</v>
+        <v>4161.130275554546</v>
       </c>
       <c r="T7" s="3">
-        <v>162.8100975484062</v>
+        <v>211.6024794584778</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
@@ -1153,10 +1153,10 @@
         <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>271.5819334790612</v>
+        <v>271.6451866947031</v>
       </c>
       <c r="G8" s="3">
-        <v>12.00853732205968</v>
+        <v>12.01133418925607</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
@@ -1193,10 +1193,10 @@
         <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3018.984564891375</v>
+        <v>3923.740781421468</v>
       </c>
       <c r="T8" s="3">
-        <v>133.4904290495269</v>
+        <v>173.4960312425264</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
@@ -1250,10 +1250,10 @@
         <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>231.2949324342337</v>
+        <v>231.3488025427889</v>
       </c>
       <c r="G9" s="3">
-        <v>4.584187797725841</v>
+        <v>4.58525548516633</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
@@ -1290,10 +1290,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>2571.142424723851</v>
+        <v>3341.685315007511</v>
       </c>
       <c r="T9" s="3">
-        <v>50.95917842033032</v>
+        <v>66.23107944336061</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
@@ -1470,10 +1470,10 @@
         <v>0</v>
       </c>
       <c r="F14" s="3">
-        <v>363.1566259346982</v>
+        <v>363.2412074975357</v>
       </c>
       <c r="G14" s="3">
-        <v>171.6550801719853</v>
+        <v>171.6950597673253</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
@@ -1510,10 +1510,10 @@
         <v>0</v>
       </c>
       <c r="S14" s="3">
-        <v>4036.955751400944</v>
+        <v>5246.786650973078</v>
       </c>
       <c r="T14" s="3">
-        <v>1908.16830444419</v>
+        <v>2480.025198218567</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
@@ -1567,10 +1567,10 @@
         <v>0</v>
       </c>
       <c r="F15" s="3">
-        <v>320.8109788943828</v>
+        <v>320.8856978779631</v>
       </c>
       <c r="G15" s="3">
-        <v>136.7455314648333</v>
+        <v>136.7773803970469</v>
       </c>
       <c r="H15" s="4">
         <f>IF(F15=0,0,G15/F15)</f>
@@ -1607,10 +1607,10 @@
         <v>0</v>
       </c>
       <c r="S15" s="3">
-        <v>3566.229097505511</v>
+        <v>4634.988435682091</v>
       </c>
       <c r="T15" s="3">
-        <v>1520.103504388773</v>
+        <v>1975.66167827245</v>
       </c>
       <c r="U15" s="4">
         <f>IF(S15=0,0,T15/S15)</f>
@@ -1664,10 +1664,10 @@
         <v>0</v>
       </c>
       <c r="F16" s="3">
-        <v>288.0128603408813</v>
+        <v>288.0799404272827</v>
       </c>
       <c r="G16" s="3">
-        <v>109.3350058211387</v>
+        <v>109.3604706619396</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
@@ -1704,10 +1704,10 @@
         <v>0</v>
       </c>
       <c r="S16" s="3">
-        <v>3201.635575388428</v>
+        <v>4161.130275554546</v>
       </c>
       <c r="T16" s="3">
-        <v>1215.400047962967</v>
+        <v>1579.641972798723</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
@@ -1761,10 +1761,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>271.5819334790612</v>
+        <v>271.6451866947031</v>
       </c>
       <c r="G17" s="3">
-        <v>93.16955449989293</v>
+        <v>93.19125430093101</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
@@ -1801,10 +1801,10 @@
         <v>0</v>
       </c>
       <c r="S17" s="3">
-        <v>3018.984564891375</v>
+        <v>3923.740781421468</v>
       </c>
       <c r="T17" s="3">
-        <v>1035.700141573183</v>
+        <v>1346.087995968573</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
@@ -1858,10 +1858,10 @@
         <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>231.2949324342337</v>
+        <v>231.3488025427889</v>
       </c>
       <c r="G18" s="3">
-        <v>41.4518499047723</v>
+        <v>41.46150431280741</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
@@ -1898,10 +1898,10 @@
         <v>0</v>
       </c>
       <c r="S18" s="3">
-        <v>2571.142424723851</v>
+        <v>3341.685315007511</v>
       </c>
       <c r="T18" s="3">
-        <v>460.7909423339825</v>
+        <v>598.8848810860113</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
@@ -2078,10 +2078,10 @@
         <v>0</v>
       </c>
       <c r="F23" s="3">
-        <v>413.6052490085787</v>
+        <v>414.1174655591563</v>
       </c>
       <c r="G23" s="3">
-        <v>268.406433964483</v>
+        <v>268.7388335606863</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
@@ -2118,10 +2118,10 @@
         <v>0</v>
       </c>
       <c r="S23" s="3">
-        <v>4597.75746758657</v>
+        <v>7595.550633139525</v>
       </c>
       <c r="T23" s="3">
-        <v>2983.684779307255</v>
+        <v>4929.083139840336</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
@@ -2175,10 +2175,10 @@
         <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>422.9371101765626</v>
+        <v>423.4608834802265</v>
       </c>
       <c r="G24" s="3">
-        <v>264.8490662071024</v>
+        <v>265.1770602919006</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
@@ -2215,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="S24" s="3">
-        <v>4701.493178084503</v>
+        <v>7766.92327449926</v>
       </c>
       <c r="T24" s="3">
-        <v>2944.140034141051</v>
+        <v>4863.754745225788</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="F25" s="3">
-        <v>382.8744648174589</v>
+        <v>383.3486237845976</v>
       </c>
       <c r="G25" s="3">
-        <v>207.4137355149925</v>
+        <v>207.6706006016967</v>
       </c>
       <c r="H25" s="4">
         <f>IF(F25=0,0,G25/F25)</f>
@@ -2312,10 +2312,10 @@
         <v>0</v>
       </c>
       <c r="S25" s="3">
-        <v>4256.145041636478</v>
+        <v>7031.20279693764</v>
       </c>
       <c r="T25" s="3">
-        <v>2305.6720233362</v>
+        <v>3808.997912596752</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
@@ -2369,10 +2369,10 @@
         <v>0</v>
       </c>
       <c r="F26" s="3">
-        <v>339.3794107528897</v>
+        <v>339.7997046237476</v>
       </c>
       <c r="G26" s="3">
-        <v>163.7500164709789</v>
+        <v>163.9528075835068</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
@@ -2409,10 +2409,10 @@
         <v>0</v>
       </c>
       <c r="S26" s="3">
-        <v>3772.641241557029</v>
+        <v>6232.448704163242</v>
       </c>
       <c r="T26" s="3">
-        <v>1820.293293790503</v>
+        <v>3007.146413794556</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
@@ -2466,10 +2466,10 @@
         <v>0</v>
       </c>
       <c r="F27" s="3">
-        <v>298.0832435152593</v>
+        <v>298.4523954328049</v>
       </c>
       <c r="G27" s="3">
-        <v>136.0735620028871</v>
+        <v>136.242078071581</v>
       </c>
       <c r="H27" s="4">
         <f>IF(F27=0,0,G27/F27)</f>
@@ -2506,10 +2506,10 @@
         <v>0</v>
       </c>
       <c r="S27" s="3">
-        <v>3313.580913491462</v>
+        <v>5474.075521134529</v>
       </c>
       <c r="T27" s="3">
-        <v>1512.633694421276</v>
+        <v>2498.889055450901</v>
       </c>
       <c r="U27" s="4">
         <f>IF(S27=0,0,T27/S27)</f>
@@ -2686,10 +2686,10 @@
         <v>0</v>
       </c>
       <c r="F32" s="3">
-        <v>413.6052490085787</v>
+        <v>414.1174655591563</v>
       </c>
       <c r="G32" s="3">
-        <v>17.31045199131634</v>
+        <v>17.33188958193897</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
@@ -2726,10 +2726,10 @@
         <v>0</v>
       </c>
       <c r="S32" s="3">
-        <v>4597.75746758657</v>
+        <v>7595.550633139525</v>
       </c>
       <c r="T32" s="3">
-        <v>192.4280702460892</v>
+        <v>317.8934863562181</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
@@ -2783,10 +2783,10 @@
         <v>0</v>
       </c>
       <c r="F33" s="3">
-        <v>422.9371101765626</v>
+        <v>423.4608834802265</v>
       </c>
       <c r="G33" s="3">
-        <v>33.45220057492261</v>
+        <v>33.49362841180107</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
@@ -2823,10 +2823,10 @@
         <v>0</v>
       </c>
       <c r="S33" s="3">
-        <v>4701.493178084503</v>
+        <v>7766.92327449926</v>
       </c>
       <c r="T33" s="3">
-        <v>371.8644900402705</v>
+        <v>614.3246099168791</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
@@ -2880,10 +2880,10 @@
         <v>0</v>
       </c>
       <c r="F34" s="3">
-        <v>382.8744648174589</v>
+        <v>383.3486237845976</v>
       </c>
       <c r="G34" s="3">
-        <v>41.85489240021754</v>
+        <v>41.90672628932121</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
@@ -2920,10 +2920,10 @@
         <v>0</v>
       </c>
       <c r="S34" s="3">
-        <v>4256.145041636478</v>
+        <v>7031.20279693764</v>
       </c>
       <c r="T34" s="3">
-        <v>465.271281129561</v>
+        <v>768.6337521888199</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
@@ -2977,10 +2977,10 @@
         <v>0</v>
       </c>
       <c r="F35" s="3">
-        <v>339.3794107528897</v>
+        <v>339.7997046237476</v>
       </c>
       <c r="G35" s="3">
-        <v>49.09141688271048</v>
+        <v>49.15221262038295</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
@@ -3017,10 +3017,10 @@
         <v>0</v>
       </c>
       <c r="S35" s="3">
-        <v>3772.641241557029</v>
+        <v>6232.448704163242</v>
       </c>
       <c r="T35" s="3">
-        <v>545.7146134095751</v>
+        <v>901.527104597878</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
@@ -3074,10 +3074,10 @@
         <v>0</v>
       </c>
       <c r="F36" s="3">
-        <v>298.0832435152593</v>
+        <v>298.4523954328049</v>
       </c>
       <c r="G36" s="3">
-        <v>47.77947036092321</v>
+        <v>47.83864135924927</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
@@ -3114,10 +3114,10 @@
         <v>0</v>
       </c>
       <c r="S36" s="3">
-        <v>3313.580913491462</v>
+        <v>5474.075521134529</v>
       </c>
       <c r="T36" s="3">
-        <v>531.1306304159348</v>
+        <v>877.4341892925413</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
@@ -3286,18 +3286,18 @@
         <v>0</v>
       </c>
       <c r="D41" s="3">
-        <f>G41+J41</f>
+        <f>J41+G41</f>
         <v>0</v>
       </c>
       <c r="E41" s="3">
-        <f>P41+M41</f>
+        <f>M41+P41</f>
         <v>0</v>
       </c>
       <c r="F41" s="3">
-        <v>155.6388197021622</v>
+        <v>155.693183623828</v>
       </c>
       <c r="G41" s="3">
-        <v>72.14250991153671</v>
+        <v>72.16770895741165</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
@@ -3334,10 +3334,10 @@
         <v>0</v>
       </c>
       <c r="S41" s="3">
-        <v>1730.126847391954</v>
+        <v>2076.424364219953</v>
       </c>
       <c r="T41" s="3">
-        <v>801.9573360620632</v>
+        <v>962.4749504201816</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
@@ -3383,18 +3383,18 @@
         <v>0</v>
       </c>
       <c r="D42" s="3">
-        <f>G42+J42</f>
+        <f>J42+G42</f>
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <f>P42+M42</f>
+        <f>M42+P42</f>
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>148.048117342397</v>
+        <v>148.099829866749</v>
       </c>
       <c r="G42" s="3">
-        <v>72.88503207356277</v>
+        <v>72.91049047900319</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
@@ -3431,10 +3431,10 @@
         <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>1645.746369768679</v>
+        <v>1975.154518101098</v>
       </c>
       <c r="T42" s="3">
-        <v>810.2114305724377</v>
+        <v>972.3811621940484</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
@@ -3480,18 +3480,18 @@
         <v>0</v>
       </c>
       <c r="D43" s="3">
-        <f>G43+J43</f>
+        <f>J43+G43</f>
         <v>0</v>
       </c>
       <c r="E43" s="3">
-        <f>P43+M43</f>
+        <f>M43+P43</f>
         <v>0</v>
       </c>
       <c r="F43" s="3">
-        <v>134.74967754932</v>
+        <v>134.796744990006</v>
       </c>
       <c r="G43" s="3">
-        <v>72.9230042046555</v>
+        <v>72.9484758735861</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
@@ -3528,10 +3528,10 @@
         <v>0</v>
       </c>
       <c r="S43" s="3">
-        <v>1497.917005870538</v>
+        <v>1797.736028001397</v>
       </c>
       <c r="T43" s="3">
-        <v>810.6335399380957</v>
+        <v>972.8877598302499</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
@@ -3577,18 +3577,18 @@
         <v>0</v>
       </c>
       <c r="D44" s="3">
-        <f>G44+J44</f>
+        <f>J44+G44</f>
         <v>0</v>
       </c>
       <c r="E44" s="3">
-        <f>P44+M44</f>
+        <f>M44+P44</f>
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>118.7444756744663</v>
+        <v>118.7859525719791</v>
       </c>
       <c r="G44" s="3">
-        <v>33.20204370990226</v>
+        <v>33.21364103058893</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
@@ -3625,10 +3625,10 @@
         <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>1319.998479409059</v>
+        <v>1584.205809828305</v>
       </c>
       <c r="T44" s="3">
-        <v>369.0836728311747</v>
+        <v>442.958463917078</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
@@ -3674,18 +3674,18 @@
         <v>0</v>
       </c>
       <c r="D45" s="3">
-        <f>G45+J45</f>
+        <f>J45+G45</f>
         <v>0</v>
       </c>
       <c r="E45" s="3">
-        <f>P45+M45</f>
+        <f>M45+P45</f>
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>93.67750509105568</v>
+        <v>93.71022621139285</v>
       </c>
       <c r="G45" s="3">
-        <v>19.07953157899767</v>
+        <v>19.08619597135289</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
@@ -3722,10 +3722,10 @@
         <v>0</v>
       </c>
       <c r="S45" s="3">
-        <v>1041.346669583361</v>
+        <v>1249.779806366036</v>
       </c>
       <c r="T45" s="3">
-        <v>212.0936787085381</v>
+        <v>254.545776589339</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
@@ -3894,18 +3894,18 @@
         <v>0</v>
       </c>
       <c r="D50" s="3">
-        <f>G50+J50</f>
+        <f>J50+G50</f>
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>P50+M50</f>
+        <f>M50+P50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
-        <v>155.6388197021622</v>
+        <v>155.693183623828</v>
       </c>
       <c r="G50" s="3">
-        <v>128.0966173135081</v>
+        <v>128.1413608709483</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
@@ -3942,10 +3942,10 @@
         <v>0</v>
       </c>
       <c r="S50" s="3">
-        <v>1730.126847391954</v>
+        <v>2076.424364219953</v>
       </c>
       <c r="T50" s="3">
-        <v>1423.95963358179</v>
+        <v>1708.975547828781</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -3991,18 +3991,18 @@
         <v>0</v>
       </c>
       <c r="D51" s="3">
-        <f>G51+J51</f>
+        <f>J51+G51</f>
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>P51+M51</f>
+        <f>M51+P51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <v>148.048117342397</v>
+        <v>148.099829866749</v>
       </c>
       <c r="G51" s="3">
-        <v>124.6466030827076</v>
+        <v>124.690141566094</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4039,10 +4039,10 @@
         <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>1645.746369768679</v>
+        <v>1975.154518101098</v>
       </c>
       <c r="T51" s="3">
-        <v>1385.608261758136</v>
+        <v>1662.947869005153</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
@@ -4088,18 +4088,18 @@
         <v>0</v>
       </c>
       <c r="D52" s="3">
-        <f>G52+J52</f>
+        <f>J52+G52</f>
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>P52+M52</f>
+        <f>M52+P52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
-        <v>134.74967754932</v>
+        <v>134.796744990006</v>
       </c>
       <c r="G52" s="3">
-        <v>117.2759712044506</v>
+        <v>117.3169351601271</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4136,10 +4136,10 @@
         <v>0</v>
       </c>
       <c r="S52" s="3">
-        <v>1497.917005870538</v>
+        <v>1797.736028001397</v>
       </c>
       <c r="T52" s="3">
-        <v>1303.674152265284</v>
+        <v>1564.614049454244</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
@@ -4185,18 +4185,18 @@
         <v>0</v>
       </c>
       <c r="D53" s="3">
-        <f>G53+J53</f>
+        <f>J53+G53</f>
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>P53+M53</f>
+        <f>M53+P53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
-        <v>118.7444756744663</v>
+        <v>118.7859525719791</v>
       </c>
       <c r="G53" s="3">
-        <v>77.06056921867676</v>
+        <v>77.0874861199776</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4233,10 +4233,10 @@
         <v>0</v>
       </c>
       <c r="S53" s="3">
-        <v>1319.998479409059</v>
+        <v>1584.205809828305</v>
       </c>
       <c r="T53" s="3">
-        <v>856.6279282744163</v>
+        <v>1028.088260708491</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4282,18 +4282,18 @@
         <v>0</v>
       </c>
       <c r="D54" s="3">
-        <f>G54+J54</f>
+        <f>J54+G54</f>
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>P54+M54</f>
+        <f>M54+P54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <v>93.67750509105568</v>
+        <v>93.71022621139285</v>
       </c>
       <c r="G54" s="3">
-        <v>50.32660180257193</v>
+        <v>50.34418065239444</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4330,10 +4330,10 @@
         <v>0</v>
       </c>
       <c r="S54" s="3">
-        <v>1041.346669583361</v>
+        <v>1249.779806366036</v>
       </c>
       <c r="T54" s="3">
-        <v>559.4452918832071</v>
+        <v>671.4223504857664</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>

</xml_diff>